<commit_message>
ref: refactor Export PR as PDF
</commit_message>
<xml_diff>
--- a/procurement_documents/PR Template.xlsx
+++ b/procurement_documents/PR Template.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr defaultThemeVersion="124226"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emman\itrac\procurement_documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{948BF3B4-E106-44B8-96FC-3118DECA9B30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76FDDAE1-7AA0-4405-B9AA-108DE8B8A00F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="739" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="39">
   <si>
     <t>Department:</t>
   </si>
@@ -134,9 +134,6 @@
     <t>pr_approved_by</t>
   </si>
   <si>
-    <t>pr_approved_by_designation</t>
-  </si>
-  <si>
     <t>saved_by_user_id_fk</t>
   </si>
   <si>
@@ -144,6 +141,21 @@
   </si>
   <si>
     <t>?? role : department</t>
+  </si>
+  <si>
+    <t>pr_items_quantity</t>
+  </si>
+  <si>
+    <t>pr_items_unit</t>
+  </si>
+  <si>
+    <t>pr_items_descrip, + pr_spec_spec</t>
+  </si>
+  <si>
+    <t>pr_items_cost</t>
+  </si>
+  <si>
+    <t>pr_unique_code</t>
   </si>
 </sst>
 </file>
@@ -836,7 +848,7 @@
     </xf>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="95">
+  <cellXfs count="99">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -935,75 +947,132 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="36" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="22" fontId="21" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="22" fontId="21" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="36" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="22" fontId="21" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="22" fontId="21" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -1019,35 +1088,17 @@
     <xf numFmtId="39" fontId="25" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -1057,44 +1108,17 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="10">
@@ -1425,78 +1449,6 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>155161</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>36313</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>111539</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>54309</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C396833A-A7B5-49A0-9231-7B29761AB3FD}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="155161" y="36313"/>
-          <a:ext cx="642178" cy="741896"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-          <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:miter lim="800000"/>
-              <a:headEnd/>
-              <a:tailEnd/>
-            </a14:hiddenLine>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1787,19 +1739,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C126E29C-91B2-4103-86A7-16F40F6D1729}">
-  <sheetPr>
+  <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N53"/>
+  <dimension ref="A1:N54"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.28515625" style="3" customWidth="1"/>
-    <col min="2" max="2" width="9.85546875" style="3" customWidth="1"/>
-    <col min="3" max="3" width="29.28515625" style="3" customWidth="1"/>
-    <col min="4" max="4" width="29.140625" style="3" customWidth="1"/>
-    <col min="5" max="5" width="15" style="3" customWidth="1"/>
-    <col min="6" max="6" width="1.7109375" style="3" customWidth="1"/>
-    <col min="7" max="7" width="19.85546875" style="3" customWidth="1"/>
+    <col min="1" max="1" width="11.85546875" style="3" customWidth="1"/>
+    <col min="2" max="2" width="11.28515625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="33.85546875" style="3" customWidth="1"/>
+    <col min="4" max="4" width="33.7109375" style="3" customWidth="1"/>
+    <col min="5" max="5" width="17.28515625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="1.85546875" style="3" customWidth="1"/>
+    <col min="7" max="7" width="22.85546875" style="3" customWidth="1"/>
     <col min="8" max="8" width="8.140625" style="3" customWidth="1"/>
     <col min="9" max="16384" width="8.85546875" style="3"/>
   </cols>
@@ -1817,51 +1769,51 @@
     </row>
     <row r="2" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="14"/>
-      <c r="B2" s="85" t="s">
+      <c r="B2" s="38" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="85"/>
-      <c r="D2" s="86"/>
-      <c r="E2" s="89" t="s">
+      <c r="C2" s="38"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="40" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="85"/>
-      <c r="G2" s="86"/>
+      <c r="F2" s="38"/>
+      <c r="G2" s="39"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="15"/>
-      <c r="B3" s="87" t="s">
+      <c r="B3" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="87"/>
-      <c r="D3" s="88"/>
-      <c r="E3" s="93" t="s">
+      <c r="C3" s="41"/>
+      <c r="D3" s="42"/>
+      <c r="E3" s="95" t="s">
         <v>28</v>
       </c>
-      <c r="F3" s="92"/>
-      <c r="G3" s="94"/>
+      <c r="F3" s="96"/>
+      <c r="G3" s="97"/>
     </row>
     <row r="4" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="14"/>
-      <c r="B4" s="85"/>
-      <c r="C4" s="85"/>
-      <c r="D4" s="86"/>
+      <c r="B4" s="38"/>
+      <c r="C4" s="38"/>
+      <c r="D4" s="39"/>
       <c r="E4" s="34"/>
       <c r="F4" s="34"/>
       <c r="G4" s="35"/>
     </row>
     <row r="5" spans="1:14" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="30"/>
-      <c r="B5" s="40" t="s">
+      <c r="B5" s="43" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="40"/>
-      <c r="D5" s="41"/>
-      <c r="E5" s="42" t="s">
+      <c r="C5" s="43"/>
+      <c r="D5" s="44"/>
+      <c r="E5" s="45" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="42"/>
-      <c r="G5" s="43"/>
+      <c r="F5" s="45"/>
+      <c r="G5" s="46"/>
     </row>
     <row r="6" spans="1:14" ht="4.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="16"/>
@@ -1885,37 +1837,37 @@
       <c r="A8" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B8" s="46"/>
-      <c r="C8" s="47"/>
-      <c r="D8" s="48"/>
+      <c r="B8" s="47"/>
+      <c r="C8" s="48"/>
+      <c r="D8" s="49"/>
       <c r="E8" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="F8" s="49"/>
-      <c r="G8" s="50"/>
+      <c r="F8" s="50"/>
+      <c r="G8" s="51"/>
       <c r="H8" s="4"/>
     </row>
     <row r="9" spans="1:14" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="51"/>
-      <c r="C9" s="52"/>
-      <c r="D9" s="53"/>
+      <c r="B9" s="52"/>
+      <c r="C9" s="53"/>
+      <c r="D9" s="54"/>
       <c r="E9" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="54"/>
-      <c r="G9" s="55"/>
+      <c r="F9" s="55"/>
+      <c r="G9" s="56"/>
     </row>
     <row r="10" spans="1:14" ht="5.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="56"/>
-      <c r="B10" s="56"/>
-      <c r="C10" s="56"/>
-      <c r="D10" s="56"/>
-      <c r="E10" s="56"/>
-      <c r="F10" s="56"/>
-      <c r="G10" s="56"/>
+      <c r="A10" s="57"/>
+      <c r="B10" s="57"/>
+      <c r="C10" s="57"/>
+      <c r="D10" s="57"/>
+      <c r="E10" s="57"/>
+      <c r="F10" s="57"/>
+      <c r="G10" s="57"/>
     </row>
     <row r="11" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
@@ -1924,14 +1876,14 @@
       <c r="B11" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="57" t="s">
+      <c r="C11" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="D11" s="58"/>
-      <c r="E11" s="57" t="s">
+      <c r="D11" s="37"/>
+      <c r="E11" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="F11" s="58"/>
+      <c r="F11" s="37"/>
       <c r="G11" s="22" t="s">
         <v>4</v>
       </c>
@@ -1939,10 +1891,10 @@
     <row r="12" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="12"/>
       <c r="B12" s="1"/>
-      <c r="C12" s="44"/>
-      <c r="D12" s="45"/>
-      <c r="E12" s="38"/>
-      <c r="F12" s="39"/>
+      <c r="C12" s="58"/>
+      <c r="D12" s="59"/>
+      <c r="E12" s="60"/>
+      <c r="F12" s="61"/>
       <c r="G12" s="23"/>
       <c r="H12" s="11"/>
       <c r="I12" s="5"/>
@@ -1955,10 +1907,10 @@
     <row r="13" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="12"/>
       <c r="B13" s="1"/>
-      <c r="C13" s="44"/>
-      <c r="D13" s="45"/>
-      <c r="E13" s="38"/>
-      <c r="F13" s="39"/>
+      <c r="C13" s="58"/>
+      <c r="D13" s="59"/>
+      <c r="E13" s="60"/>
+      <c r="F13" s="61"/>
       <c r="G13" s="23"/>
       <c r="H13" s="11"/>
       <c r="I13" s="8"/>
@@ -1969,403 +1921,406 @@
     <row r="14" spans="1:14" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="13"/>
       <c r="B14" s="1"/>
-      <c r="C14" s="44"/>
-      <c r="D14" s="45"/>
-      <c r="E14" s="38"/>
-      <c r="F14" s="39"/>
+      <c r="C14" s="58"/>
+      <c r="D14" s="59"/>
+      <c r="E14" s="60"/>
+      <c r="F14" s="61"/>
       <c r="G14" s="23"/>
       <c r="H14" s="11"/>
     </row>
     <row r="15" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="13"/>
       <c r="B15" s="1"/>
-      <c r="C15" s="44"/>
-      <c r="D15" s="45"/>
-      <c r="E15" s="38"/>
-      <c r="F15" s="39"/>
+      <c r="C15" s="58"/>
+      <c r="D15" s="59"/>
+      <c r="E15" s="60"/>
+      <c r="F15" s="61"/>
       <c r="G15" s="23"/>
       <c r="H15" s="11"/>
     </row>
     <row r="16" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="13"/>
       <c r="B16" s="2"/>
-      <c r="C16" s="44"/>
-      <c r="D16" s="45"/>
-      <c r="E16" s="38"/>
-      <c r="F16" s="39"/>
+      <c r="C16" s="58"/>
+      <c r="D16" s="59"/>
+      <c r="E16" s="60"/>
+      <c r="F16" s="61"/>
       <c r="G16" s="23"/>
       <c r="H16" s="11"/>
     </row>
     <row r="17" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="13"/>
       <c r="B17" s="2"/>
-      <c r="C17" s="44"/>
-      <c r="D17" s="45"/>
-      <c r="E17" s="38"/>
-      <c r="F17" s="39"/>
+      <c r="C17" s="58"/>
+      <c r="D17" s="59"/>
+      <c r="E17" s="60"/>
+      <c r="F17" s="61"/>
       <c r="G17" s="23"/>
       <c r="H17" s="11"/>
     </row>
     <row r="18" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="13"/>
       <c r="B18" s="2"/>
-      <c r="C18" s="36"/>
-      <c r="D18" s="37"/>
-      <c r="E18" s="38"/>
-      <c r="F18" s="39"/>
+      <c r="C18" s="62"/>
+      <c r="D18" s="63"/>
+      <c r="E18" s="60"/>
+      <c r="F18" s="61"/>
       <c r="G18" s="23"/>
       <c r="H18" s="11"/>
     </row>
     <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="13"/>
       <c r="B19" s="2"/>
-      <c r="C19" s="36"/>
-      <c r="D19" s="37"/>
-      <c r="E19" s="38"/>
-      <c r="F19" s="39"/>
+      <c r="C19" s="62"/>
+      <c r="D19" s="63"/>
+      <c r="E19" s="60"/>
+      <c r="F19" s="61"/>
       <c r="G19" s="23"/>
       <c r="H19" s="10"/>
     </row>
     <row r="20" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="13"/>
       <c r="B20" s="2"/>
-      <c r="C20" s="36"/>
-      <c r="D20" s="37"/>
-      <c r="E20" s="38"/>
-      <c r="F20" s="39"/>
+      <c r="C20" s="62"/>
+      <c r="D20" s="63"/>
+      <c r="E20" s="60"/>
+      <c r="F20" s="61"/>
       <c r="G20" s="23"/>
       <c r="H20" s="10"/>
     </row>
     <row r="21" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="13"/>
       <c r="B21" s="2"/>
-      <c r="C21" s="36"/>
-      <c r="D21" s="37"/>
-      <c r="E21" s="38"/>
-      <c r="F21" s="39"/>
+      <c r="C21" s="62"/>
+      <c r="D21" s="63"/>
+      <c r="E21" s="60"/>
+      <c r="F21" s="61"/>
       <c r="G21" s="23"/>
       <c r="H21" s="10"/>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="13"/>
       <c r="B22" s="2"/>
-      <c r="C22" s="36"/>
-      <c r="D22" s="37"/>
-      <c r="E22" s="38"/>
-      <c r="F22" s="39"/>
+      <c r="C22" s="62"/>
+      <c r="D22" s="63"/>
+      <c r="E22" s="60"/>
+      <c r="F22" s="61"/>
       <c r="G22" s="23"/>
       <c r="H22" s="10"/>
     </row>
     <row r="23" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="13"/>
       <c r="B23" s="2"/>
-      <c r="C23" s="36"/>
-      <c r="D23" s="37"/>
-      <c r="E23" s="38"/>
-      <c r="F23" s="39"/>
+      <c r="C23" s="62"/>
+      <c r="D23" s="63"/>
+      <c r="E23" s="60"/>
+      <c r="F23" s="61"/>
       <c r="G23" s="23"/>
       <c r="H23" s="10"/>
     </row>
     <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="13"/>
       <c r="B24" s="2"/>
-      <c r="C24" s="36"/>
-      <c r="D24" s="37"/>
-      <c r="E24" s="38"/>
-      <c r="F24" s="39"/>
+      <c r="C24" s="62"/>
+      <c r="D24" s="63"/>
+      <c r="E24" s="60"/>
+      <c r="F24" s="61"/>
       <c r="G24" s="23"/>
       <c r="H24" s="10"/>
     </row>
     <row r="25" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="13"/>
       <c r="B25" s="2"/>
-      <c r="C25" s="36"/>
-      <c r="D25" s="37"/>
-      <c r="E25" s="38"/>
-      <c r="F25" s="39"/>
+      <c r="C25" s="62"/>
+      <c r="D25" s="63"/>
+      <c r="E25" s="60"/>
+      <c r="F25" s="61"/>
       <c r="G25" s="23"/>
       <c r="H25" s="10"/>
     </row>
     <row r="26" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="13"/>
       <c r="B26" s="2"/>
-      <c r="C26" s="36"/>
-      <c r="D26" s="37"/>
-      <c r="E26" s="38"/>
-      <c r="F26" s="39"/>
+      <c r="C26" s="62"/>
+      <c r="D26" s="63"/>
+      <c r="E26" s="60"/>
+      <c r="F26" s="61"/>
       <c r="G26" s="23"/>
       <c r="H26" s="10"/>
     </row>
     <row r="27" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="13"/>
       <c r="B27" s="2"/>
-      <c r="C27" s="36"/>
-      <c r="D27" s="37"/>
-      <c r="E27" s="38"/>
-      <c r="F27" s="39"/>
+      <c r="C27" s="62"/>
+      <c r="D27" s="63"/>
+      <c r="E27" s="60"/>
+      <c r="F27" s="61"/>
       <c r="G27" s="23"/>
       <c r="H27" s="10"/>
     </row>
     <row r="28" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="13"/>
       <c r="B28" s="2"/>
-      <c r="C28" s="59"/>
-      <c r="D28" s="60"/>
-      <c r="E28" s="38"/>
-      <c r="F28" s="39"/>
+      <c r="C28" s="64"/>
+      <c r="D28" s="65"/>
+      <c r="E28" s="60"/>
+      <c r="F28" s="61"/>
       <c r="G28" s="23"/>
       <c r="H28" s="10"/>
     </row>
     <row r="29" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="13"/>
       <c r="B29" s="2"/>
-      <c r="C29" s="59"/>
-      <c r="D29" s="60"/>
-      <c r="E29" s="38"/>
-      <c r="F29" s="39"/>
+      <c r="C29" s="64"/>
+      <c r="D29" s="65"/>
+      <c r="E29" s="60"/>
+      <c r="F29" s="61"/>
       <c r="G29" s="23"/>
       <c r="H29" s="10"/>
     </row>
     <row r="30" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="13"/>
       <c r="B30" s="2"/>
-      <c r="C30" s="59"/>
-      <c r="D30" s="60"/>
-      <c r="E30" s="38"/>
-      <c r="F30" s="39"/>
+      <c r="C30" s="64"/>
+      <c r="D30" s="65"/>
+      <c r="E30" s="60"/>
+      <c r="F30" s="61"/>
       <c r="G30" s="23"/>
       <c r="H30" s="10"/>
     </row>
     <row r="31" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="13"/>
       <c r="B31" s="2"/>
-      <c r="C31" s="36"/>
-      <c r="D31" s="37"/>
-      <c r="E31" s="38"/>
-      <c r="F31" s="39"/>
+      <c r="C31" s="62"/>
+      <c r="D31" s="63"/>
+      <c r="E31" s="60"/>
+      <c r="F31" s="61"/>
       <c r="G31" s="23"/>
       <c r="H31" s="10"/>
     </row>
     <row r="32" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="13"/>
       <c r="B32" s="2"/>
-      <c r="C32" s="36"/>
-      <c r="D32" s="37"/>
-      <c r="E32" s="38"/>
-      <c r="F32" s="39"/>
+      <c r="C32" s="62"/>
+      <c r="D32" s="63"/>
+      <c r="E32" s="60"/>
+      <c r="F32" s="61"/>
       <c r="G32" s="23"/>
       <c r="H32" s="10"/>
     </row>
     <row r="33" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="13"/>
       <c r="B33" s="2"/>
-      <c r="C33" s="36"/>
-      <c r="D33" s="37"/>
-      <c r="E33" s="38"/>
-      <c r="F33" s="39"/>
+      <c r="C33" s="62"/>
+      <c r="D33" s="63"/>
+      <c r="E33" s="60"/>
+      <c r="F33" s="61"/>
       <c r="G33" s="23"/>
       <c r="H33" s="10"/>
     </row>
     <row r="34" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="13"/>
       <c r="B34" s="2"/>
-      <c r="C34" s="36"/>
-      <c r="D34" s="37"/>
-      <c r="E34" s="38"/>
-      <c r="F34" s="39"/>
+      <c r="C34" s="62"/>
+      <c r="D34" s="63"/>
+      <c r="E34" s="60"/>
+      <c r="F34" s="61"/>
       <c r="G34" s="23"/>
       <c r="H34" s="10"/>
     </row>
     <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="13"/>
       <c r="B35" s="2"/>
-      <c r="C35" s="36"/>
-      <c r="D35" s="37"/>
-      <c r="E35" s="38"/>
-      <c r="F35" s="39"/>
+      <c r="C35" s="62"/>
+      <c r="D35" s="63"/>
+      <c r="E35" s="60"/>
+      <c r="F35" s="61"/>
       <c r="G35" s="23"/>
       <c r="H35" s="10"/>
     </row>
     <row r="36" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="13"/>
       <c r="B36" s="2"/>
-      <c r="C36" s="36"/>
-      <c r="D36" s="37"/>
-      <c r="E36" s="38"/>
-      <c r="F36" s="39"/>
+      <c r="C36" s="62"/>
+      <c r="D36" s="63"/>
+      <c r="E36" s="60"/>
+      <c r="F36" s="61"/>
       <c r="G36" s="23"/>
       <c r="H36" s="10"/>
     </row>
     <row r="37" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="13"/>
       <c r="B37" s="2"/>
-      <c r="C37" s="36"/>
-      <c r="D37" s="37"/>
-      <c r="E37" s="38"/>
-      <c r="F37" s="39"/>
+      <c r="C37" s="62"/>
+      <c r="D37" s="63"/>
+      <c r="E37" s="60"/>
+      <c r="F37" s="61"/>
       <c r="G37" s="23"/>
       <c r="H37" s="10"/>
     </row>
     <row r="38" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="13"/>
       <c r="B38" s="2"/>
-      <c r="C38" s="36"/>
-      <c r="D38" s="37"/>
-      <c r="E38" s="38"/>
-      <c r="F38" s="39"/>
+      <c r="C38" s="62"/>
+      <c r="D38" s="63"/>
+      <c r="E38" s="60"/>
+      <c r="F38" s="61"/>
       <c r="G38" s="23"/>
       <c r="H38" s="10"/>
     </row>
     <row r="39" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="13"/>
       <c r="B39" s="2"/>
-      <c r="C39" s="90"/>
-      <c r="D39" s="91"/>
-      <c r="E39" s="38"/>
-      <c r="F39" s="39"/>
+      <c r="C39" s="66"/>
+      <c r="D39" s="67"/>
+      <c r="E39" s="60"/>
+      <c r="F39" s="61"/>
       <c r="G39" s="23"/>
       <c r="H39" s="10"/>
     </row>
     <row r="40" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="13"/>
       <c r="B40" s="2"/>
-      <c r="C40" s="36"/>
-      <c r="D40" s="37"/>
-      <c r="E40" s="38"/>
-      <c r="F40" s="39"/>
+      <c r="C40" s="62"/>
+      <c r="D40" s="63"/>
+      <c r="E40" s="60"/>
+      <c r="F40" s="61"/>
       <c r="G40" s="23"/>
       <c r="H40" s="10"/>
     </row>
     <row r="41" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="13"/>
       <c r="B41" s="2"/>
-      <c r="C41" s="36"/>
-      <c r="D41" s="37"/>
-      <c r="E41" s="38"/>
-      <c r="F41" s="39"/>
+      <c r="C41" s="62"/>
+      <c r="D41" s="63"/>
+      <c r="E41" s="60"/>
+      <c r="F41" s="61"/>
       <c r="G41" s="23"/>
       <c r="H41" s="10"/>
     </row>
     <row r="42" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="13"/>
       <c r="B42" s="2"/>
-      <c r="C42" s="36"/>
-      <c r="D42" s="37"/>
-      <c r="E42" s="38"/>
-      <c r="F42" s="39"/>
+      <c r="C42" s="62"/>
+      <c r="D42" s="63"/>
+      <c r="E42" s="60"/>
+      <c r="F42" s="61"/>
       <c r="G42" s="23"/>
       <c r="H42" s="10"/>
     </row>
     <row r="43" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="13"/>
       <c r="B43" s="2"/>
-      <c r="C43" s="36"/>
-      <c r="D43" s="37"/>
-      <c r="E43" s="38"/>
-      <c r="F43" s="39"/>
+      <c r="C43" s="62"/>
+      <c r="D43" s="63"/>
+      <c r="E43" s="60"/>
+      <c r="F43" s="61"/>
       <c r="G43" s="23"/>
       <c r="H43" s="10"/>
     </row>
     <row r="44" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="13"/>
       <c r="B44" s="2"/>
-      <c r="C44" s="36"/>
-      <c r="D44" s="37"/>
-      <c r="E44" s="38"/>
-      <c r="F44" s="39"/>
+      <c r="C44" s="62"/>
+      <c r="D44" s="63"/>
+      <c r="E44" s="60"/>
+      <c r="F44" s="61"/>
       <c r="G44" s="23"/>
       <c r="H44" s="10"/>
     </row>
     <row r="45" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="13"/>
       <c r="B45" s="2"/>
-      <c r="C45" s="36"/>
-      <c r="D45" s="37"/>
-      <c r="E45" s="38"/>
-      <c r="F45" s="39"/>
+      <c r="C45" s="62"/>
+      <c r="D45" s="63"/>
+      <c r="E45" s="60"/>
+      <c r="F45" s="61"/>
       <c r="G45" s="23"/>
       <c r="H45" s="10"/>
     </row>
     <row r="46" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="13"/>
       <c r="B46" s="2"/>
-      <c r="C46" s="36"/>
-      <c r="D46" s="37"/>
-      <c r="E46" s="38"/>
-      <c r="F46" s="39"/>
+      <c r="C46" s="62"/>
+      <c r="D46" s="63"/>
+      <c r="E46" s="60"/>
+      <c r="F46" s="61"/>
       <c r="G46" s="23"/>
       <c r="H46" s="10"/>
     </row>
     <row r="47" spans="1:8" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A47" s="13"/>
       <c r="B47" s="2"/>
-      <c r="C47" s="36"/>
-      <c r="D47" s="37"/>
-      <c r="E47" s="38"/>
-      <c r="F47" s="39"/>
+      <c r="C47" s="62"/>
+      <c r="D47" s="63"/>
+      <c r="E47" s="60"/>
+      <c r="F47" s="61"/>
       <c r="G47" s="23"/>
     </row>
     <row r="48" spans="1:8" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="61" t="s">
+      <c r="A48" s="80" t="s">
         <v>14</v>
       </c>
-      <c r="B48" s="62"/>
-      <c r="C48" s="62"/>
-      <c r="D48" s="62"/>
-      <c r="E48" s="63"/>
-      <c r="F48" s="64"/>
-      <c r="G48" s="65"/>
+      <c r="B48" s="81"/>
+      <c r="C48" s="81"/>
+      <c r="D48" s="81"/>
+      <c r="E48" s="82"/>
+      <c r="F48" s="83"/>
+      <c r="G48" s="84"/>
     </row>
     <row r="49" spans="1:7" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="50" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="71" t="s">
+      <c r="A50" s="85" t="s">
         <v>20</v>
       </c>
-      <c r="B50" s="72"/>
-      <c r="C50" s="68"/>
-      <c r="D50" s="69"/>
-      <c r="E50" s="69"/>
-      <c r="F50" s="69"/>
-      <c r="G50" s="70"/>
+      <c r="B50" s="86"/>
+      <c r="C50" s="87"/>
+      <c r="D50" s="88"/>
+      <c r="E50" s="88"/>
+      <c r="F50" s="88"/>
+      <c r="G50" s="89"/>
     </row>
     <row r="51" spans="1:7" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="77" t="s">
+      <c r="A51" s="75" t="s">
         <v>15</v>
       </c>
-      <c r="B51" s="78"/>
-      <c r="C51" s="66"/>
-      <c r="D51" s="67"/>
-      <c r="E51" s="79" t="s">
+      <c r="B51" s="76"/>
+      <c r="C51" s="90"/>
+      <c r="D51" s="91"/>
+      <c r="E51" s="92" t="s">
         <v>5</v>
       </c>
-      <c r="F51" s="80"/>
-      <c r="G51" s="81"/>
+      <c r="F51" s="93"/>
+      <c r="G51" s="94"/>
     </row>
     <row r="52" spans="1:7" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A52" s="77" t="s">
+      <c r="A52" s="75" t="s">
         <v>27</v>
       </c>
-      <c r="B52" s="78"/>
+      <c r="B52" s="76"/>
       <c r="C52" s="32"/>
       <c r="D52" s="31"/>
-      <c r="E52" s="82" t="s">
+      <c r="E52" s="68" t="s">
         <v>18</v>
       </c>
-      <c r="F52" s="83"/>
-      <c r="G52" s="84"/>
+      <c r="F52" s="69"/>
+      <c r="G52" s="70"/>
     </row>
     <row r="53" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="73" t="s">
+      <c r="A53" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="B53" s="74"/>
+      <c r="B53" s="72"/>
       <c r="C53" s="33"/>
       <c r="D53" s="25"/>
-      <c r="E53" s="75" t="s">
+      <c r="E53" s="73" t="s">
         <v>6</v>
       </c>
-      <c r="F53" s="75"/>
-      <c r="G53" s="76"/>
+      <c r="F53" s="73"/>
+      <c r="G53" s="74"/>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G54" s="98"/>
     </row>
   </sheetData>
   <mergeCells count="97">
@@ -2374,6 +2329,10 @@
     <mergeCell ref="B3:D3"/>
     <mergeCell ref="E2:G2"/>
     <mergeCell ref="B2:D2"/>
+    <mergeCell ref="E36:F36"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="C34:D34"/>
     <mergeCell ref="C42:D42"/>
     <mergeCell ref="E42:F42"/>
     <mergeCell ref="C39:D39"/>
@@ -2382,12 +2341,12 @@
     <mergeCell ref="E40:F40"/>
     <mergeCell ref="C41:D41"/>
     <mergeCell ref="E41:F41"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="E31:F31"/>
     <mergeCell ref="C37:D37"/>
     <mergeCell ref="E37:F37"/>
     <mergeCell ref="C47:D47"/>
     <mergeCell ref="E47:F47"/>
+    <mergeCell ref="C38:D38"/>
+    <mergeCell ref="E38:F38"/>
     <mergeCell ref="A53:B53"/>
     <mergeCell ref="E53:G53"/>
     <mergeCell ref="A51:B51"/>
@@ -2399,16 +2358,6 @@
     <mergeCell ref="C51:D51"/>
     <mergeCell ref="C50:G50"/>
     <mergeCell ref="A50:B50"/>
-    <mergeCell ref="C38:D38"/>
-    <mergeCell ref="E38:F38"/>
-    <mergeCell ref="E32:F32"/>
-    <mergeCell ref="E33:F33"/>
-    <mergeCell ref="E34:F34"/>
-    <mergeCell ref="E35:F35"/>
-    <mergeCell ref="E36:F36"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="C34:D34"/>
     <mergeCell ref="C35:D35"/>
     <mergeCell ref="C36:D36"/>
     <mergeCell ref="C27:D27"/>
@@ -2419,6 +2368,12 @@
     <mergeCell ref="E30:F30"/>
     <mergeCell ref="E29:F29"/>
     <mergeCell ref="C29:D29"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="E32:F32"/>
+    <mergeCell ref="E33:F33"/>
+    <mergeCell ref="E34:F34"/>
+    <mergeCell ref="E35:F35"/>
     <mergeCell ref="C25:D25"/>
     <mergeCell ref="E25:F25"/>
     <mergeCell ref="C26:D26"/>
@@ -2475,10 +2430,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9B4EF7B-1FC4-4773-AAD0-7037BE84CF61}">
-  <sheetPr>
+  <sheetPr codeName="Sheet2">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N53"/>
+  <dimension ref="A1:N54"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.28515625" style="3" customWidth="1"/>
@@ -2505,51 +2460,51 @@
     </row>
     <row r="2" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="14"/>
-      <c r="B2" s="85" t="s">
+      <c r="B2" s="38" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="85"/>
-      <c r="D2" s="86"/>
-      <c r="E2" s="89" t="s">
+      <c r="C2" s="38"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="40" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="85"/>
-      <c r="G2" s="86"/>
+      <c r="F2" s="38"/>
+      <c r="G2" s="39"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="15"/>
-      <c r="B3" s="87" t="s">
+      <c r="B3" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="87"/>
-      <c r="D3" s="88"/>
-      <c r="E3" s="93" t="s">
+      <c r="C3" s="41"/>
+      <c r="D3" s="42"/>
+      <c r="E3" s="77" t="s">
         <v>28</v>
       </c>
-      <c r="F3" s="92"/>
-      <c r="G3" s="94"/>
+      <c r="F3" s="78"/>
+      <c r="G3" s="79"/>
     </row>
     <row r="4" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="14"/>
-      <c r="B4" s="85"/>
-      <c r="C4" s="85"/>
-      <c r="D4" s="86"/>
+      <c r="B4" s="38"/>
+      <c r="C4" s="38"/>
+      <c r="D4" s="39"/>
       <c r="E4" s="34"/>
       <c r="F4" s="34"/>
       <c r="G4" s="35"/>
     </row>
     <row r="5" spans="1:14" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="30"/>
-      <c r="B5" s="40" t="s">
+      <c r="B5" s="43" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="40"/>
-      <c r="D5" s="41"/>
-      <c r="E5" s="42" t="s">
+      <c r="C5" s="43"/>
+      <c r="D5" s="44"/>
+      <c r="E5" s="45" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="42"/>
-      <c r="G5" s="43"/>
+      <c r="F5" s="45"/>
+      <c r="G5" s="46"/>
     </row>
     <row r="6" spans="1:14" ht="4.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="16"/>
@@ -2573,45 +2528,45 @@
       <c r="A8" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B8" s="46" t="s">
+      <c r="B8" s="47" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="47"/>
-      <c r="D8" s="48"/>
+      <c r="C8" s="48"/>
+      <c r="D8" s="49"/>
       <c r="E8" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="F8" s="49" t="s">
+      <c r="F8" s="50" t="s">
         <v>24</v>
       </c>
-      <c r="G8" s="50"/>
+      <c r="G8" s="51"/>
       <c r="H8" s="4"/>
     </row>
     <row r="9" spans="1:14" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="51" t="s">
+      <c r="B9" s="52" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="52"/>
-      <c r="D9" s="53"/>
+      <c r="C9" s="53"/>
+      <c r="D9" s="54"/>
       <c r="E9" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="54" t="s">
+      <c r="F9" s="55" t="s">
         <v>25</v>
       </c>
-      <c r="G9" s="55"/>
+      <c r="G9" s="56"/>
     </row>
     <row r="10" spans="1:14" ht="5.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="56"/>
-      <c r="B10" s="56"/>
-      <c r="C10" s="56"/>
-      <c r="D10" s="56"/>
-      <c r="E10" s="56"/>
-      <c r="F10" s="56"/>
-      <c r="G10" s="56"/>
+      <c r="A10" s="57"/>
+      <c r="B10" s="57"/>
+      <c r="C10" s="57"/>
+      <c r="D10" s="57"/>
+      <c r="E10" s="57"/>
+      <c r="F10" s="57"/>
+      <c r="G10" s="57"/>
     </row>
     <row r="11" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
@@ -2620,25 +2575,33 @@
       <c r="B11" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="57" t="s">
+      <c r="C11" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="D11" s="58"/>
-      <c r="E11" s="57" t="s">
+      <c r="D11" s="37"/>
+      <c r="E11" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="F11" s="58"/>
+      <c r="F11" s="37"/>
       <c r="G11" s="22" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="12"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="44"/>
-      <c r="D12" s="45"/>
-      <c r="E12" s="38"/>
-      <c r="F12" s="39"/>
+      <c r="A12" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" s="58" t="s">
+        <v>36</v>
+      </c>
+      <c r="D12" s="59"/>
+      <c r="E12" s="60" t="s">
+        <v>37</v>
+      </c>
+      <c r="F12" s="61"/>
       <c r="G12" s="23"/>
       <c r="H12" s="11"/>
       <c r="I12" s="5"/>
@@ -2651,10 +2614,10 @@
     <row r="13" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="12"/>
       <c r="B13" s="1"/>
-      <c r="C13" s="44"/>
-      <c r="D13" s="45"/>
-      <c r="E13" s="38"/>
-      <c r="F13" s="39"/>
+      <c r="C13" s="58"/>
+      <c r="D13" s="59"/>
+      <c r="E13" s="60"/>
+      <c r="F13" s="61"/>
       <c r="G13" s="23"/>
       <c r="H13" s="11"/>
       <c r="I13" s="8"/>
@@ -2665,413 +2628,418 @@
     <row r="14" spans="1:14" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="13"/>
       <c r="B14" s="1"/>
-      <c r="C14" s="44"/>
-      <c r="D14" s="45"/>
-      <c r="E14" s="38"/>
-      <c r="F14" s="39"/>
+      <c r="C14" s="58"/>
+      <c r="D14" s="59"/>
+      <c r="E14" s="60"/>
+      <c r="F14" s="61"/>
       <c r="G14" s="23"/>
       <c r="H14" s="11"/>
     </row>
     <row r="15" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="13"/>
       <c r="B15" s="1"/>
-      <c r="C15" s="44"/>
-      <c r="D15" s="45"/>
-      <c r="E15" s="38"/>
-      <c r="F15" s="39"/>
+      <c r="C15" s="58"/>
+      <c r="D15" s="59"/>
+      <c r="E15" s="60"/>
+      <c r="F15" s="61"/>
       <c r="G15" s="23"/>
       <c r="H15" s="11"/>
     </row>
     <row r="16" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="13"/>
       <c r="B16" s="2"/>
-      <c r="C16" s="44"/>
-      <c r="D16" s="45"/>
-      <c r="E16" s="38"/>
-      <c r="F16" s="39"/>
+      <c r="C16" s="58"/>
+      <c r="D16" s="59"/>
+      <c r="E16" s="60"/>
+      <c r="F16" s="61"/>
       <c r="G16" s="23"/>
       <c r="H16" s="11"/>
     </row>
     <row r="17" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="13"/>
       <c r="B17" s="2"/>
-      <c r="C17" s="44"/>
-      <c r="D17" s="45"/>
-      <c r="E17" s="38"/>
-      <c r="F17" s="39"/>
+      <c r="C17" s="58"/>
+      <c r="D17" s="59"/>
+      <c r="E17" s="60"/>
+      <c r="F17" s="61"/>
       <c r="G17" s="23"/>
       <c r="H17" s="11"/>
     </row>
     <row r="18" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="13"/>
       <c r="B18" s="2"/>
-      <c r="C18" s="36"/>
-      <c r="D18" s="37"/>
-      <c r="E18" s="38"/>
-      <c r="F18" s="39"/>
+      <c r="C18" s="62"/>
+      <c r="D18" s="63"/>
+      <c r="E18" s="60"/>
+      <c r="F18" s="61"/>
       <c r="G18" s="23"/>
       <c r="H18" s="11"/>
     </row>
     <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="13"/>
       <c r="B19" s="2"/>
-      <c r="C19" s="36"/>
-      <c r="D19" s="37"/>
-      <c r="E19" s="38"/>
-      <c r="F19" s="39"/>
+      <c r="C19" s="62"/>
+      <c r="D19" s="63"/>
+      <c r="E19" s="60"/>
+      <c r="F19" s="61"/>
       <c r="G19" s="23"/>
       <c r="H19" s="10"/>
     </row>
     <row r="20" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="13"/>
       <c r="B20" s="2"/>
-      <c r="C20" s="36"/>
-      <c r="D20" s="37"/>
-      <c r="E20" s="38"/>
-      <c r="F20" s="39"/>
+      <c r="C20" s="62"/>
+      <c r="D20" s="63"/>
+      <c r="E20" s="60"/>
+      <c r="F20" s="61"/>
       <c r="G20" s="23"/>
       <c r="H20" s="10"/>
     </row>
     <row r="21" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="13"/>
       <c r="B21" s="2"/>
-      <c r="C21" s="36"/>
-      <c r="D21" s="37"/>
-      <c r="E21" s="38"/>
-      <c r="F21" s="39"/>
+      <c r="C21" s="62"/>
+      <c r="D21" s="63"/>
+      <c r="E21" s="60"/>
+      <c r="F21" s="61"/>
       <c r="G21" s="23"/>
       <c r="H21" s="10"/>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="13"/>
       <c r="B22" s="2"/>
-      <c r="C22" s="36"/>
-      <c r="D22" s="37"/>
-      <c r="E22" s="38"/>
-      <c r="F22" s="39"/>
+      <c r="C22" s="62"/>
+      <c r="D22" s="63"/>
+      <c r="E22" s="60"/>
+      <c r="F22" s="61"/>
       <c r="G22" s="23"/>
       <c r="H22" s="10"/>
     </row>
     <row r="23" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="13"/>
       <c r="B23" s="2"/>
-      <c r="C23" s="36"/>
-      <c r="D23" s="37"/>
-      <c r="E23" s="38"/>
-      <c r="F23" s="39"/>
+      <c r="C23" s="62"/>
+      <c r="D23" s="63"/>
+      <c r="E23" s="60"/>
+      <c r="F23" s="61"/>
       <c r="G23" s="23"/>
       <c r="H23" s="10"/>
     </row>
     <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="13"/>
       <c r="B24" s="2"/>
-      <c r="C24" s="36"/>
-      <c r="D24" s="37"/>
-      <c r="E24" s="38"/>
-      <c r="F24" s="39"/>
+      <c r="C24" s="62"/>
+      <c r="D24" s="63"/>
+      <c r="E24" s="60"/>
+      <c r="F24" s="61"/>
       <c r="G24" s="23"/>
       <c r="H24" s="10"/>
     </row>
     <row r="25" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="13"/>
       <c r="B25" s="2"/>
-      <c r="C25" s="36"/>
-      <c r="D25" s="37"/>
-      <c r="E25" s="38"/>
-      <c r="F25" s="39"/>
+      <c r="C25" s="62"/>
+      <c r="D25" s="63"/>
+      <c r="E25" s="60"/>
+      <c r="F25" s="61"/>
       <c r="G25" s="23"/>
       <c r="H25" s="10"/>
     </row>
     <row r="26" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="13"/>
       <c r="B26" s="2"/>
-      <c r="C26" s="36"/>
-      <c r="D26" s="37"/>
-      <c r="E26" s="38"/>
-      <c r="F26" s="39"/>
+      <c r="C26" s="62"/>
+      <c r="D26" s="63"/>
+      <c r="E26" s="60"/>
+      <c r="F26" s="61"/>
       <c r="G26" s="23"/>
       <c r="H26" s="10"/>
     </row>
     <row r="27" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="13"/>
       <c r="B27" s="2"/>
-      <c r="C27" s="36"/>
-      <c r="D27" s="37"/>
-      <c r="E27" s="38"/>
-      <c r="F27" s="39"/>
+      <c r="C27" s="62"/>
+      <c r="D27" s="63"/>
+      <c r="E27" s="60"/>
+      <c r="F27" s="61"/>
       <c r="G27" s="23"/>
       <c r="H27" s="10"/>
     </row>
     <row r="28" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="13"/>
       <c r="B28" s="2"/>
-      <c r="C28" s="59"/>
-      <c r="D28" s="60"/>
-      <c r="E28" s="38"/>
-      <c r="F28" s="39"/>
+      <c r="C28" s="64"/>
+      <c r="D28" s="65"/>
+      <c r="E28" s="60"/>
+      <c r="F28" s="61"/>
       <c r="G28" s="23"/>
       <c r="H28" s="10"/>
     </row>
     <row r="29" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="13"/>
       <c r="B29" s="2"/>
-      <c r="C29" s="59"/>
-      <c r="D29" s="60"/>
-      <c r="E29" s="38"/>
-      <c r="F29" s="39"/>
+      <c r="C29" s="64"/>
+      <c r="D29" s="65"/>
+      <c r="E29" s="60"/>
+      <c r="F29" s="61"/>
       <c r="G29" s="23"/>
       <c r="H29" s="10"/>
     </row>
     <row r="30" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="13"/>
       <c r="B30" s="2"/>
-      <c r="C30" s="59"/>
-      <c r="D30" s="60"/>
-      <c r="E30" s="38"/>
-      <c r="F30" s="39"/>
+      <c r="C30" s="64"/>
+      <c r="D30" s="65"/>
+      <c r="E30" s="60"/>
+      <c r="F30" s="61"/>
       <c r="G30" s="23"/>
       <c r="H30" s="10"/>
     </row>
     <row r="31" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="13"/>
       <c r="B31" s="2"/>
-      <c r="C31" s="36"/>
-      <c r="D31" s="37"/>
-      <c r="E31" s="38"/>
-      <c r="F31" s="39"/>
+      <c r="C31" s="62"/>
+      <c r="D31" s="63"/>
+      <c r="E31" s="60"/>
+      <c r="F31" s="61"/>
       <c r="G31" s="23"/>
       <c r="H31" s="10"/>
     </row>
     <row r="32" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="13"/>
       <c r="B32" s="2"/>
-      <c r="C32" s="36"/>
-      <c r="D32" s="37"/>
-      <c r="E32" s="38"/>
-      <c r="F32" s="39"/>
+      <c r="C32" s="62"/>
+      <c r="D32" s="63"/>
+      <c r="E32" s="60"/>
+      <c r="F32" s="61"/>
       <c r="G32" s="23"/>
       <c r="H32" s="10"/>
     </row>
     <row r="33" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="13"/>
       <c r="B33" s="2"/>
-      <c r="C33" s="36"/>
-      <c r="D33" s="37"/>
-      <c r="E33" s="38"/>
-      <c r="F33" s="39"/>
+      <c r="C33" s="62"/>
+      <c r="D33" s="63"/>
+      <c r="E33" s="60"/>
+      <c r="F33" s="61"/>
       <c r="G33" s="23"/>
       <c r="H33" s="10"/>
     </row>
     <row r="34" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="13"/>
       <c r="B34" s="2"/>
-      <c r="C34" s="36"/>
-      <c r="D34" s="37"/>
-      <c r="E34" s="38"/>
-      <c r="F34" s="39"/>
+      <c r="C34" s="62"/>
+      <c r="D34" s="63"/>
+      <c r="E34" s="60"/>
+      <c r="F34" s="61"/>
       <c r="G34" s="23"/>
       <c r="H34" s="10"/>
     </row>
     <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="13"/>
       <c r="B35" s="2"/>
-      <c r="C35" s="36"/>
-      <c r="D35" s="37"/>
-      <c r="E35" s="38"/>
-      <c r="F35" s="39"/>
+      <c r="C35" s="62"/>
+      <c r="D35" s="63"/>
+      <c r="E35" s="60"/>
+      <c r="F35" s="61"/>
       <c r="G35" s="23"/>
       <c r="H35" s="10"/>
     </row>
     <row r="36" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="13"/>
       <c r="B36" s="2"/>
-      <c r="C36" s="36"/>
-      <c r="D36" s="37"/>
-      <c r="E36" s="38"/>
-      <c r="F36" s="39"/>
+      <c r="C36" s="62"/>
+      <c r="D36" s="63"/>
+      <c r="E36" s="60"/>
+      <c r="F36" s="61"/>
       <c r="G36" s="23"/>
       <c r="H36" s="10"/>
     </row>
     <row r="37" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="13"/>
       <c r="B37" s="2"/>
-      <c r="C37" s="36"/>
-      <c r="D37" s="37"/>
-      <c r="E37" s="38"/>
-      <c r="F37" s="39"/>
+      <c r="C37" s="62"/>
+      <c r="D37" s="63"/>
+      <c r="E37" s="60"/>
+      <c r="F37" s="61"/>
       <c r="G37" s="23"/>
       <c r="H37" s="10"/>
     </row>
     <row r="38" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="13"/>
       <c r="B38" s="2"/>
-      <c r="C38" s="36"/>
-      <c r="D38" s="37"/>
-      <c r="E38" s="38"/>
-      <c r="F38" s="39"/>
+      <c r="C38" s="62"/>
+      <c r="D38" s="63"/>
+      <c r="E38" s="60"/>
+      <c r="F38" s="61"/>
       <c r="G38" s="23"/>
       <c r="H38" s="10"/>
     </row>
     <row r="39" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="13"/>
       <c r="B39" s="2"/>
-      <c r="C39" s="90"/>
-      <c r="D39" s="91"/>
-      <c r="E39" s="38"/>
-      <c r="F39" s="39"/>
+      <c r="C39" s="66"/>
+      <c r="D39" s="67"/>
+      <c r="E39" s="60"/>
+      <c r="F39" s="61"/>
       <c r="G39" s="23"/>
       <c r="H39" s="10"/>
     </row>
     <row r="40" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="13"/>
       <c r="B40" s="2"/>
-      <c r="C40" s="36"/>
-      <c r="D40" s="37"/>
-      <c r="E40" s="38"/>
-      <c r="F40" s="39"/>
+      <c r="C40" s="62"/>
+      <c r="D40" s="63"/>
+      <c r="E40" s="60"/>
+      <c r="F40" s="61"/>
       <c r="G40" s="23"/>
       <c r="H40" s="10"/>
     </row>
     <row r="41" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="13"/>
       <c r="B41" s="2"/>
-      <c r="C41" s="36"/>
-      <c r="D41" s="37"/>
-      <c r="E41" s="38"/>
-      <c r="F41" s="39"/>
+      <c r="C41" s="62"/>
+      <c r="D41" s="63"/>
+      <c r="E41" s="60"/>
+      <c r="F41" s="61"/>
       <c r="G41" s="23"/>
       <c r="H41" s="10"/>
     </row>
     <row r="42" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="13"/>
       <c r="B42" s="2"/>
-      <c r="C42" s="36"/>
-      <c r="D42" s="37"/>
-      <c r="E42" s="38"/>
-      <c r="F42" s="39"/>
+      <c r="C42" s="62"/>
+      <c r="D42" s="63"/>
+      <c r="E42" s="60"/>
+      <c r="F42" s="61"/>
       <c r="G42" s="23"/>
       <c r="H42" s="10"/>
     </row>
     <row r="43" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="13"/>
       <c r="B43" s="2"/>
-      <c r="C43" s="36"/>
-      <c r="D43" s="37"/>
-      <c r="E43" s="38"/>
-      <c r="F43" s="39"/>
+      <c r="C43" s="62"/>
+      <c r="D43" s="63"/>
+      <c r="E43" s="60"/>
+      <c r="F43" s="61"/>
       <c r="G43" s="23"/>
       <c r="H43" s="10"/>
     </row>
     <row r="44" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="13"/>
       <c r="B44" s="2"/>
-      <c r="C44" s="36"/>
-      <c r="D44" s="37"/>
-      <c r="E44" s="38"/>
-      <c r="F44" s="39"/>
+      <c r="C44" s="62"/>
+      <c r="D44" s="63"/>
+      <c r="E44" s="60"/>
+      <c r="F44" s="61"/>
       <c r="G44" s="23"/>
       <c r="H44" s="10"/>
     </row>
     <row r="45" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="13"/>
       <c r="B45" s="2"/>
-      <c r="C45" s="36"/>
-      <c r="D45" s="37"/>
-      <c r="E45" s="38"/>
-      <c r="F45" s="39"/>
+      <c r="C45" s="62"/>
+      <c r="D45" s="63"/>
+      <c r="E45" s="60"/>
+      <c r="F45" s="61"/>
       <c r="G45" s="23"/>
       <c r="H45" s="10"/>
     </row>
     <row r="46" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="13"/>
       <c r="B46" s="2"/>
-      <c r="C46" s="36"/>
-      <c r="D46" s="37"/>
-      <c r="E46" s="38"/>
-      <c r="F46" s="39"/>
+      <c r="C46" s="62"/>
+      <c r="D46" s="63"/>
+      <c r="E46" s="60"/>
+      <c r="F46" s="61"/>
       <c r="G46" s="23"/>
       <c r="H46" s="10"/>
     </row>
     <row r="47" spans="1:8" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A47" s="13"/>
       <c r="B47" s="2"/>
-      <c r="C47" s="36"/>
-      <c r="D47" s="37"/>
-      <c r="E47" s="38"/>
-      <c r="F47" s="39"/>
+      <c r="C47" s="62"/>
+      <c r="D47" s="63"/>
+      <c r="E47" s="60"/>
+      <c r="F47" s="61"/>
       <c r="G47" s="23"/>
     </row>
     <row r="48" spans="1:8" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="61" t="s">
+      <c r="A48" s="80" t="s">
         <v>14</v>
       </c>
-      <c r="B48" s="62"/>
-      <c r="C48" s="62"/>
-      <c r="D48" s="62"/>
-      <c r="E48" s="63"/>
-      <c r="F48" s="64"/>
-      <c r="G48" s="65"/>
+      <c r="B48" s="81"/>
+      <c r="C48" s="81"/>
+      <c r="D48" s="81"/>
+      <c r="E48" s="82"/>
+      <c r="F48" s="83"/>
+      <c r="G48" s="84"/>
     </row>
     <row r="49" spans="1:7" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="50" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="71" t="s">
+      <c r="A50" s="85" t="s">
         <v>20</v>
       </c>
-      <c r="B50" s="72"/>
-      <c r="C50" s="68" t="s">
+      <c r="B50" s="86"/>
+      <c r="C50" s="87" t="s">
         <v>26</v>
       </c>
-      <c r="D50" s="69"/>
-      <c r="E50" s="69"/>
-      <c r="F50" s="69"/>
-      <c r="G50" s="70"/>
+      <c r="D50" s="88"/>
+      <c r="E50" s="88"/>
+      <c r="F50" s="88"/>
+      <c r="G50" s="89"/>
     </row>
     <row r="51" spans="1:7" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="77" t="s">
+      <c r="A51" s="75" t="s">
         <v>15</v>
       </c>
-      <c r="B51" s="78"/>
-      <c r="C51" s="66"/>
-      <c r="D51" s="67"/>
-      <c r="E51" s="79" t="s">
+      <c r="B51" s="76"/>
+      <c r="C51" s="90"/>
+      <c r="D51" s="91"/>
+      <c r="E51" s="92" t="s">
         <v>5</v>
       </c>
-      <c r="F51" s="80"/>
-      <c r="G51" s="81"/>
+      <c r="F51" s="93"/>
+      <c r="G51" s="94"/>
     </row>
     <row r="52" spans="1:7" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A52" s="77" t="s">
+      <c r="A52" s="75" t="s">
         <v>27</v>
       </c>
-      <c r="B52" s="78"/>
+      <c r="B52" s="76"/>
       <c r="C52" s="32" t="s">
+        <v>29</v>
+      </c>
+      <c r="D52" s="31" t="s">
+        <v>31</v>
+      </c>
+      <c r="E52" s="68" t="s">
+        <v>30</v>
+      </c>
+      <c r="F52" s="69"/>
+      <c r="G52" s="70"/>
+    </row>
+    <row r="53" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="71" t="s">
+        <v>16</v>
+      </c>
+      <c r="B53" s="72"/>
+      <c r="C53" s="33" t="s">
+        <v>33</v>
+      </c>
+      <c r="D53" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="D52" s="31" t="s">
-        <v>29</v>
-      </c>
-      <c r="E52" s="82" t="s">
-        <v>30</v>
-      </c>
-      <c r="F52" s="83"/>
-      <c r="G52" s="84"/>
-    </row>
-    <row r="53" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="73" t="s">
-        <v>16</v>
-      </c>
-      <c r="B53" s="74"/>
-      <c r="C53" s="33" t="s">
-        <v>34</v>
-      </c>
-      <c r="D53" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="E53" s="75" t="s">
-        <v>31</v>
-      </c>
-      <c r="F53" s="75"/>
-      <c r="G53" s="76"/>
+      <c r="E53" s="73" t="s">
+        <v>32</v>
+      </c>
+      <c r="F53" s="73"/>
+      <c r="G53" s="74"/>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G54" s="3" t="s">
+        <v>38</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="97">
@@ -3159,11 +3127,6 @@
     <mergeCell ref="E13:F13"/>
     <mergeCell ref="C14:D14"/>
     <mergeCell ref="E14:F14"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="A10:G10"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="E11:F11"/>
     <mergeCell ref="B2:D2"/>
@@ -3172,6 +3135,11 @@
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="E5:G5"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="A10:G10"/>
   </mergeCells>
   <pageMargins left="0.51181102362204722" right="0.19685039370078741" top="0.31496062992125984" bottom="0" header="0.51181102362204722" footer="0.51181102362204722"/>
   <pageSetup paperSize="9" scale="83" fitToHeight="0" orientation="portrait" copies="3" r:id="rId1"/>

</xml_diff>

<commit_message>
chore: remove action button in Procure PR tab. ref: revise pr_unique_code pattern
</commit_message>
<xml_diff>
--- a/procurement_documents/PR Template.xlsx
+++ b/procurement_documents/PR Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emman\itrac\procurement_documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76FDDAE1-7AA0-4405-B9AA-108DE8B8A00F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C47CE686-06A3-44B9-BE8E-5A3106F2F0D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="739" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -848,7 +848,7 @@
     </xf>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="99">
+  <cellXfs count="105">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -947,11 +947,17 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -959,64 +965,15 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="36" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="22" fontId="21" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="22" fontId="21" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="164" fontId="5" fillId="2" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1029,14 +986,39 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1046,33 +1028,6 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -1088,37 +1043,100 @@
     <xf numFmtId="39" fontId="25" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="36" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="22" fontId="21" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="22" fontId="21" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="22" fontId="21" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="22" fontId="21" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="10">
@@ -1769,51 +1787,51 @@
     </row>
     <row r="2" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="14"/>
-      <c r="B2" s="38" t="s">
+      <c r="B2" s="40" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="38"/>
-      <c r="D2" s="39"/>
-      <c r="E2" s="40" t="s">
+      <c r="C2" s="40"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="38"/>
-      <c r="G2" s="39"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="41"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="15"/>
-      <c r="B3" s="41" t="s">
+      <c r="B3" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="41"/>
-      <c r="D3" s="42"/>
-      <c r="E3" s="95" t="s">
+      <c r="C3" s="42"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="37" t="s">
         <v>28</v>
       </c>
-      <c r="F3" s="96"/>
-      <c r="G3" s="97"/>
+      <c r="F3" s="38"/>
+      <c r="G3" s="39"/>
     </row>
     <row r="4" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="14"/>
-      <c r="B4" s="38"/>
-      <c r="C4" s="38"/>
-      <c r="D4" s="39"/>
+      <c r="B4" s="40"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="41"/>
       <c r="E4" s="34"/>
       <c r="F4" s="34"/>
       <c r="G4" s="35"/>
     </row>
     <row r="5" spans="1:14" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="30"/>
-      <c r="B5" s="43" t="s">
+      <c r="B5" s="79" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="43"/>
-      <c r="D5" s="44"/>
-      <c r="E5" s="45" t="s">
+      <c r="C5" s="79"/>
+      <c r="D5" s="80"/>
+      <c r="E5" s="81" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="45"/>
-      <c r="G5" s="46"/>
+      <c r="F5" s="81"/>
+      <c r="G5" s="82"/>
     </row>
     <row r="6" spans="1:14" ht="4.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="16"/>
@@ -1837,37 +1855,37 @@
       <c r="A8" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B8" s="47"/>
-      <c r="C8" s="48"/>
-      <c r="D8" s="49"/>
+      <c r="B8" s="83"/>
+      <c r="C8" s="84"/>
+      <c r="D8" s="85"/>
       <c r="E8" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="F8" s="50"/>
-      <c r="G8" s="51"/>
+      <c r="F8" s="86"/>
+      <c r="G8" s="87"/>
       <c r="H8" s="4"/>
     </row>
     <row r="9" spans="1:14" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="52"/>
-      <c r="C9" s="53"/>
-      <c r="D9" s="54"/>
+      <c r="B9" s="88"/>
+      <c r="C9" s="89"/>
+      <c r="D9" s="90"/>
       <c r="E9" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="55"/>
-      <c r="G9" s="56"/>
+      <c r="F9" s="100"/>
+      <c r="G9" s="101"/>
     </row>
     <row r="10" spans="1:14" ht="5.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="57"/>
-      <c r="B10" s="57"/>
-      <c r="C10" s="57"/>
-      <c r="D10" s="57"/>
-      <c r="E10" s="57"/>
-      <c r="F10" s="57"/>
-      <c r="G10" s="57"/>
+      <c r="A10" s="93"/>
+      <c r="B10" s="93"/>
+      <c r="C10" s="93"/>
+      <c r="D10" s="93"/>
+      <c r="E10" s="93"/>
+      <c r="F10" s="93"/>
+      <c r="G10" s="93"/>
     </row>
     <row r="11" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
@@ -1876,14 +1894,14 @@
       <c r="B11" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="36" t="s">
+      <c r="C11" s="94" t="s">
         <v>7</v>
       </c>
-      <c r="D11" s="37"/>
-      <c r="E11" s="36" t="s">
+      <c r="D11" s="95"/>
+      <c r="E11" s="94" t="s">
         <v>3</v>
       </c>
-      <c r="F11" s="37"/>
+      <c r="F11" s="95"/>
       <c r="G11" s="22" t="s">
         <v>4</v>
       </c>
@@ -1891,10 +1909,10 @@
     <row r="12" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="12"/>
       <c r="B12" s="1"/>
-      <c r="C12" s="58"/>
-      <c r="D12" s="59"/>
-      <c r="E12" s="60"/>
-      <c r="F12" s="61"/>
+      <c r="C12" s="77"/>
+      <c r="D12" s="78"/>
+      <c r="E12" s="45"/>
+      <c r="F12" s="46"/>
       <c r="G12" s="23"/>
       <c r="H12" s="11"/>
       <c r="I12" s="5"/>
@@ -1907,10 +1925,10 @@
     <row r="13" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="12"/>
       <c r="B13" s="1"/>
-      <c r="C13" s="58"/>
-      <c r="D13" s="59"/>
-      <c r="E13" s="60"/>
-      <c r="F13" s="61"/>
+      <c r="C13" s="77"/>
+      <c r="D13" s="78"/>
+      <c r="E13" s="45"/>
+      <c r="F13" s="46"/>
       <c r="G13" s="23"/>
       <c r="H13" s="11"/>
       <c r="I13" s="8"/>
@@ -1921,428 +1939,469 @@
     <row r="14" spans="1:14" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="13"/>
       <c r="B14" s="1"/>
-      <c r="C14" s="58"/>
-      <c r="D14" s="59"/>
-      <c r="E14" s="60"/>
-      <c r="F14" s="61"/>
+      <c r="C14" s="77"/>
+      <c r="D14" s="78"/>
+      <c r="E14" s="45"/>
+      <c r="F14" s="46"/>
       <c r="G14" s="23"/>
       <c r="H14" s="11"/>
     </row>
     <row r="15" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="13"/>
       <c r="B15" s="1"/>
-      <c r="C15" s="58"/>
-      <c r="D15" s="59"/>
-      <c r="E15" s="60"/>
-      <c r="F15" s="61"/>
+      <c r="C15" s="77"/>
+      <c r="D15" s="78"/>
+      <c r="E15" s="45"/>
+      <c r="F15" s="46"/>
       <c r="G15" s="23"/>
       <c r="H15" s="11"/>
     </row>
     <row r="16" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="13"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="58"/>
-      <c r="D16" s="59"/>
-      <c r="E16" s="60"/>
-      <c r="F16" s="61"/>
+      <c r="B16" s="99"/>
+      <c r="C16" s="77"/>
+      <c r="D16" s="78"/>
+      <c r="E16" s="45"/>
+      <c r="F16" s="46"/>
       <c r="G16" s="23"/>
       <c r="H16" s="11"/>
     </row>
     <row r="17" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="13"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="58"/>
-      <c r="D17" s="59"/>
-      <c r="E17" s="60"/>
-      <c r="F17" s="61"/>
+      <c r="B17" s="99"/>
+      <c r="C17" s="77"/>
+      <c r="D17" s="78"/>
+      <c r="E17" s="45"/>
+      <c r="F17" s="46"/>
       <c r="G17" s="23"/>
       <c r="H17" s="11"/>
     </row>
     <row r="18" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="13"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="62"/>
-      <c r="D18" s="63"/>
-      <c r="E18" s="60"/>
-      <c r="F18" s="61"/>
+      <c r="B18" s="99"/>
+      <c r="C18" s="47"/>
+      <c r="D18" s="48"/>
+      <c r="E18" s="45"/>
+      <c r="F18" s="46"/>
       <c r="G18" s="23"/>
       <c r="H18" s="11"/>
     </row>
     <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="13"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="62"/>
-      <c r="D19" s="63"/>
-      <c r="E19" s="60"/>
-      <c r="F19" s="61"/>
+      <c r="B19" s="99"/>
+      <c r="C19" s="47"/>
+      <c r="D19" s="48"/>
+      <c r="E19" s="45"/>
+      <c r="F19" s="46"/>
       <c r="G19" s="23"/>
       <c r="H19" s="10"/>
     </row>
     <row r="20" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="13"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="62"/>
-      <c r="D20" s="63"/>
-      <c r="E20" s="60"/>
-      <c r="F20" s="61"/>
+      <c r="B20" s="99"/>
+      <c r="C20" s="47"/>
+      <c r="D20" s="48"/>
+      <c r="E20" s="45"/>
+      <c r="F20" s="46"/>
       <c r="G20" s="23"/>
       <c r="H20" s="10"/>
     </row>
     <row r="21" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="13"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="62"/>
-      <c r="D21" s="63"/>
-      <c r="E21" s="60"/>
-      <c r="F21" s="61"/>
+      <c r="B21" s="99"/>
+      <c r="C21" s="47"/>
+      <c r="D21" s="48"/>
+      <c r="E21" s="45"/>
+      <c r="F21" s="46"/>
       <c r="G21" s="23"/>
       <c r="H21" s="10"/>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="13"/>
-      <c r="B22" s="2"/>
-      <c r="C22" s="62"/>
-      <c r="D22" s="63"/>
-      <c r="E22" s="60"/>
-      <c r="F22" s="61"/>
+      <c r="B22" s="99"/>
+      <c r="C22" s="47"/>
+      <c r="D22" s="48"/>
+      <c r="E22" s="45"/>
+      <c r="F22" s="46"/>
       <c r="G22" s="23"/>
       <c r="H22" s="10"/>
     </row>
     <row r="23" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="13"/>
-      <c r="B23" s="2"/>
-      <c r="C23" s="62"/>
-      <c r="D23" s="63"/>
-      <c r="E23" s="60"/>
-      <c r="F23" s="61"/>
+      <c r="B23" s="99"/>
+      <c r="C23" s="47"/>
+      <c r="D23" s="48"/>
+      <c r="E23" s="45"/>
+      <c r="F23" s="46"/>
       <c r="G23" s="23"/>
       <c r="H23" s="10"/>
     </row>
     <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="13"/>
-      <c r="B24" s="2"/>
-      <c r="C24" s="62"/>
-      <c r="D24" s="63"/>
-      <c r="E24" s="60"/>
-      <c r="F24" s="61"/>
+      <c r="B24" s="99"/>
+      <c r="C24" s="47"/>
+      <c r="D24" s="48"/>
+      <c r="E24" s="45"/>
+      <c r="F24" s="46"/>
       <c r="G24" s="23"/>
       <c r="H24" s="10"/>
     </row>
     <row r="25" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="13"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="62"/>
-      <c r="D25" s="63"/>
-      <c r="E25" s="60"/>
-      <c r="F25" s="61"/>
+      <c r="B25" s="99"/>
+      <c r="C25" s="47"/>
+      <c r="D25" s="48"/>
+      <c r="E25" s="45"/>
+      <c r="F25" s="46"/>
       <c r="G25" s="23"/>
       <c r="H25" s="10"/>
     </row>
     <row r="26" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="13"/>
-      <c r="B26" s="2"/>
-      <c r="C26" s="62"/>
-      <c r="D26" s="63"/>
-      <c r="E26" s="60"/>
-      <c r="F26" s="61"/>
+      <c r="B26" s="99"/>
+      <c r="C26" s="47"/>
+      <c r="D26" s="48"/>
+      <c r="E26" s="45"/>
+      <c r="F26" s="46"/>
       <c r="G26" s="23"/>
       <c r="H26" s="10"/>
     </row>
     <row r="27" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="13"/>
-      <c r="B27" s="2"/>
-      <c r="C27" s="62"/>
-      <c r="D27" s="63"/>
-      <c r="E27" s="60"/>
-      <c r="F27" s="61"/>
+      <c r="B27" s="99"/>
+      <c r="C27" s="47"/>
+      <c r="D27" s="48"/>
+      <c r="E27" s="45"/>
+      <c r="F27" s="46"/>
       <c r="G27" s="23"/>
       <c r="H27" s="10"/>
     </row>
     <row r="28" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="13"/>
-      <c r="B28" s="2"/>
-      <c r="C28" s="64"/>
-      <c r="D28" s="65"/>
-      <c r="E28" s="60"/>
-      <c r="F28" s="61"/>
+      <c r="B28" s="99"/>
+      <c r="C28" s="75"/>
+      <c r="D28" s="76"/>
+      <c r="E28" s="45"/>
+      <c r="F28" s="46"/>
       <c r="G28" s="23"/>
       <c r="H28" s="10"/>
     </row>
     <row r="29" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="13"/>
-      <c r="B29" s="2"/>
-      <c r="C29" s="64"/>
-      <c r="D29" s="65"/>
-      <c r="E29" s="60"/>
-      <c r="F29" s="61"/>
+      <c r="B29" s="99"/>
+      <c r="C29" s="75"/>
+      <c r="D29" s="76"/>
+      <c r="E29" s="45"/>
+      <c r="F29" s="46"/>
       <c r="G29" s="23"/>
       <c r="H29" s="10"/>
     </row>
     <row r="30" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="13"/>
-      <c r="B30" s="2"/>
-      <c r="C30" s="64"/>
-      <c r="D30" s="65"/>
-      <c r="E30" s="60"/>
-      <c r="F30" s="61"/>
+      <c r="B30" s="99"/>
+      <c r="C30" s="75"/>
+      <c r="D30" s="76"/>
+      <c r="E30" s="45"/>
+      <c r="F30" s="46"/>
       <c r="G30" s="23"/>
       <c r="H30" s="10"/>
     </row>
     <row r="31" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="13"/>
-      <c r="B31" s="2"/>
-      <c r="C31" s="62"/>
-      <c r="D31" s="63"/>
-      <c r="E31" s="60"/>
-      <c r="F31" s="61"/>
+      <c r="B31" s="99"/>
+      <c r="C31" s="47"/>
+      <c r="D31" s="48"/>
+      <c r="E31" s="45"/>
+      <c r="F31" s="46"/>
       <c r="G31" s="23"/>
       <c r="H31" s="10"/>
     </row>
     <row r="32" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="13"/>
-      <c r="B32" s="2"/>
-      <c r="C32" s="62"/>
-      <c r="D32" s="63"/>
-      <c r="E32" s="60"/>
-      <c r="F32" s="61"/>
+      <c r="B32" s="99"/>
+      <c r="C32" s="47"/>
+      <c r="D32" s="48"/>
+      <c r="E32" s="45"/>
+      <c r="F32" s="46"/>
       <c r="G32" s="23"/>
       <c r="H32" s="10"/>
     </row>
     <row r="33" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="13"/>
-      <c r="B33" s="2"/>
-      <c r="C33" s="62"/>
-      <c r="D33" s="63"/>
-      <c r="E33" s="60"/>
-      <c r="F33" s="61"/>
+      <c r="B33" s="99"/>
+      <c r="C33" s="47"/>
+      <c r="D33" s="48"/>
+      <c r="E33" s="45"/>
+      <c r="F33" s="46"/>
       <c r="G33" s="23"/>
       <c r="H33" s="10"/>
     </row>
     <row r="34" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="13"/>
-      <c r="B34" s="2"/>
-      <c r="C34" s="62"/>
-      <c r="D34" s="63"/>
-      <c r="E34" s="60"/>
-      <c r="F34" s="61"/>
+      <c r="B34" s="99"/>
+      <c r="C34" s="47"/>
+      <c r="D34" s="48"/>
+      <c r="E34" s="45"/>
+      <c r="F34" s="46"/>
       <c r="G34" s="23"/>
       <c r="H34" s="10"/>
     </row>
     <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="13"/>
-      <c r="B35" s="2"/>
-      <c r="C35" s="62"/>
-      <c r="D35" s="63"/>
-      <c r="E35" s="60"/>
-      <c r="F35" s="61"/>
+      <c r="B35" s="99"/>
+      <c r="C35" s="47"/>
+      <c r="D35" s="48"/>
+      <c r="E35" s="45"/>
+      <c r="F35" s="46"/>
       <c r="G35" s="23"/>
       <c r="H35" s="10"/>
     </row>
     <row r="36" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="13"/>
-      <c r="B36" s="2"/>
-      <c r="C36" s="62"/>
-      <c r="D36" s="63"/>
-      <c r="E36" s="60"/>
-      <c r="F36" s="61"/>
+      <c r="B36" s="99"/>
+      <c r="C36" s="47"/>
+      <c r="D36" s="48"/>
+      <c r="E36" s="45"/>
+      <c r="F36" s="46"/>
       <c r="G36" s="23"/>
       <c r="H36" s="10"/>
     </row>
     <row r="37" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="13"/>
-      <c r="B37" s="2"/>
-      <c r="C37" s="62"/>
-      <c r="D37" s="63"/>
-      <c r="E37" s="60"/>
-      <c r="F37" s="61"/>
+      <c r="B37" s="99"/>
+      <c r="C37" s="47"/>
+      <c r="D37" s="48"/>
+      <c r="E37" s="45"/>
+      <c r="F37" s="46"/>
       <c r="G37" s="23"/>
       <c r="H37" s="10"/>
     </row>
     <row r="38" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="13"/>
-      <c r="B38" s="2"/>
-      <c r="C38" s="62"/>
-      <c r="D38" s="63"/>
-      <c r="E38" s="60"/>
-      <c r="F38" s="61"/>
+      <c r="B38" s="99"/>
+      <c r="C38" s="47"/>
+      <c r="D38" s="48"/>
+      <c r="E38" s="45"/>
+      <c r="F38" s="46"/>
       <c r="G38" s="23"/>
       <c r="H38" s="10"/>
     </row>
     <row r="39" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="13"/>
-      <c r="B39" s="2"/>
-      <c r="C39" s="66"/>
-      <c r="D39" s="67"/>
-      <c r="E39" s="60"/>
-      <c r="F39" s="61"/>
+      <c r="B39" s="99"/>
+      <c r="C39" s="49"/>
+      <c r="D39" s="50"/>
+      <c r="E39" s="45"/>
+      <c r="F39" s="46"/>
       <c r="G39" s="23"/>
       <c r="H39" s="10"/>
     </row>
     <row r="40" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="13"/>
-      <c r="B40" s="2"/>
-      <c r="C40" s="62"/>
-      <c r="D40" s="63"/>
-      <c r="E40" s="60"/>
-      <c r="F40" s="61"/>
+      <c r="B40" s="99"/>
+      <c r="C40" s="47"/>
+      <c r="D40" s="48"/>
+      <c r="E40" s="45"/>
+      <c r="F40" s="46"/>
       <c r="G40" s="23"/>
       <c r="H40" s="10"/>
     </row>
     <row r="41" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="13"/>
-      <c r="B41" s="2"/>
-      <c r="C41" s="62"/>
-      <c r="D41" s="63"/>
-      <c r="E41" s="60"/>
-      <c r="F41" s="61"/>
+      <c r="B41" s="99"/>
+      <c r="C41" s="47"/>
+      <c r="D41" s="48"/>
+      <c r="E41" s="45"/>
+      <c r="F41" s="46"/>
       <c r="G41" s="23"/>
       <c r="H41" s="10"/>
     </row>
     <row r="42" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="13"/>
-      <c r="B42" s="2"/>
-      <c r="C42" s="62"/>
-      <c r="D42" s="63"/>
-      <c r="E42" s="60"/>
-      <c r="F42" s="61"/>
+      <c r="B42" s="99"/>
+      <c r="C42" s="47"/>
+      <c r="D42" s="48"/>
+      <c r="E42" s="45"/>
+      <c r="F42" s="46"/>
       <c r="G42" s="23"/>
       <c r="H42" s="10"/>
     </row>
     <row r="43" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="13"/>
-      <c r="B43" s="2"/>
-      <c r="C43" s="62"/>
-      <c r="D43" s="63"/>
-      <c r="E43" s="60"/>
-      <c r="F43" s="61"/>
+      <c r="B43" s="99"/>
+      <c r="C43" s="47"/>
+      <c r="D43" s="48"/>
+      <c r="E43" s="45"/>
+      <c r="F43" s="46"/>
       <c r="G43" s="23"/>
       <c r="H43" s="10"/>
     </row>
     <row r="44" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="13"/>
-      <c r="B44" s="2"/>
-      <c r="C44" s="62"/>
-      <c r="D44" s="63"/>
-      <c r="E44" s="60"/>
-      <c r="F44" s="61"/>
+      <c r="B44" s="99"/>
+      <c r="C44" s="47"/>
+      <c r="D44" s="48"/>
+      <c r="E44" s="45"/>
+      <c r="F44" s="46"/>
       <c r="G44" s="23"/>
       <c r="H44" s="10"/>
     </row>
     <row r="45" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="13"/>
-      <c r="B45" s="2"/>
-      <c r="C45" s="62"/>
-      <c r="D45" s="63"/>
-      <c r="E45" s="60"/>
-      <c r="F45" s="61"/>
+      <c r="B45" s="99"/>
+      <c r="C45" s="47"/>
+      <c r="D45" s="48"/>
+      <c r="E45" s="45"/>
+      <c r="F45" s="46"/>
       <c r="G45" s="23"/>
       <c r="H45" s="10"/>
     </row>
     <row r="46" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="13"/>
-      <c r="B46" s="2"/>
-      <c r="C46" s="62"/>
-      <c r="D46" s="63"/>
-      <c r="E46" s="60"/>
-      <c r="F46" s="61"/>
+      <c r="B46" s="99"/>
+      <c r="C46" s="47"/>
+      <c r="D46" s="48"/>
+      <c r="E46" s="45"/>
+      <c r="F46" s="46"/>
       <c r="G46" s="23"/>
       <c r="H46" s="10"/>
     </row>
     <row r="47" spans="1:8" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A47" s="13"/>
-      <c r="B47" s="2"/>
-      <c r="C47" s="62"/>
-      <c r="D47" s="63"/>
-      <c r="E47" s="60"/>
-      <c r="F47" s="61"/>
+      <c r="B47" s="99"/>
+      <c r="C47" s="47"/>
+      <c r="D47" s="48"/>
+      <c r="E47" s="45"/>
+      <c r="F47" s="46"/>
       <c r="G47" s="23"/>
     </row>
     <row r="48" spans="1:8" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="80" t="s">
+      <c r="A48" s="63" t="s">
         <v>14</v>
       </c>
-      <c r="B48" s="81"/>
-      <c r="C48" s="81"/>
-      <c r="D48" s="81"/>
-      <c r="E48" s="82"/>
-      <c r="F48" s="83"/>
-      <c r="G48" s="84"/>
+      <c r="B48" s="64"/>
+      <c r="C48" s="64"/>
+      <c r="D48" s="64"/>
+      <c r="E48" s="65"/>
+      <c r="F48" s="66"/>
+      <c r="G48" s="67"/>
     </row>
     <row r="49" spans="1:7" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="50" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="85" t="s">
+      <c r="A50" s="73" t="s">
         <v>20</v>
       </c>
-      <c r="B50" s="86"/>
-      <c r="C50" s="87"/>
-      <c r="D50" s="88"/>
-      <c r="E50" s="88"/>
-      <c r="F50" s="88"/>
-      <c r="G50" s="89"/>
+      <c r="B50" s="74"/>
+      <c r="C50" s="102"/>
+      <c r="D50" s="103"/>
+      <c r="E50" s="103"/>
+      <c r="F50" s="103"/>
+      <c r="G50" s="104"/>
     </row>
     <row r="51" spans="1:7" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="75" t="s">
+      <c r="A51" s="55" t="s">
         <v>15</v>
       </c>
-      <c r="B51" s="76"/>
-      <c r="C51" s="90"/>
-      <c r="D51" s="91"/>
-      <c r="E51" s="92" t="s">
+      <c r="B51" s="56"/>
+      <c r="C51" s="68"/>
+      <c r="D51" s="69"/>
+      <c r="E51" s="57" t="s">
         <v>5</v>
       </c>
-      <c r="F51" s="93"/>
-      <c r="G51" s="94"/>
+      <c r="F51" s="58"/>
+      <c r="G51" s="59"/>
     </row>
     <row r="52" spans="1:7" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A52" s="75" t="s">
+      <c r="A52" s="55" t="s">
         <v>27</v>
       </c>
-      <c r="B52" s="76"/>
+      <c r="B52" s="56"/>
       <c r="C52" s="32"/>
       <c r="D52" s="31"/>
-      <c r="E52" s="68" t="s">
+      <c r="E52" s="60" t="s">
         <v>18</v>
       </c>
-      <c r="F52" s="69"/>
-      <c r="G52" s="70"/>
+      <c r="F52" s="61"/>
+      <c r="G52" s="62"/>
     </row>
     <row r="53" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="71" t="s">
+      <c r="A53" s="51" t="s">
         <v>16</v>
       </c>
-      <c r="B53" s="72"/>
+      <c r="B53" s="52"/>
       <c r="C53" s="33"/>
       <c r="D53" s="25"/>
-      <c r="E53" s="73" t="s">
+      <c r="E53" s="53" t="s">
         <v>6</v>
       </c>
-      <c r="F53" s="73"/>
-      <c r="G53" s="74"/>
+      <c r="F53" s="53"/>
+      <c r="G53" s="54"/>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="G54" s="98"/>
+      <c r="G54" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="97">
-    <mergeCell ref="E3:G3"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="E36:F36"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="C34:D34"/>
-    <mergeCell ref="C42:D42"/>
-    <mergeCell ref="E42:F42"/>
-    <mergeCell ref="C39:D39"/>
-    <mergeCell ref="E39:F39"/>
-    <mergeCell ref="C40:D40"/>
-    <mergeCell ref="E40:F40"/>
-    <mergeCell ref="C41:D41"/>
-    <mergeCell ref="E41:F41"/>
-    <mergeCell ref="C37:D37"/>
-    <mergeCell ref="E37:F37"/>
+    <mergeCell ref="E43:F43"/>
+    <mergeCell ref="C45:D45"/>
+    <mergeCell ref="E45:F45"/>
+    <mergeCell ref="C46:D46"/>
+    <mergeCell ref="E46:F46"/>
+    <mergeCell ref="C44:D44"/>
+    <mergeCell ref="E44:F44"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="A10:G10"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="E35:F35"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="E32:F32"/>
+    <mergeCell ref="E33:F33"/>
+    <mergeCell ref="E34:F34"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="E28:F28"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="E30:F30"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="C29:D29"/>
     <mergeCell ref="C47:D47"/>
     <mergeCell ref="E47:F47"/>
     <mergeCell ref="C38:D38"/>
@@ -2358,69 +2417,28 @@
     <mergeCell ref="C51:D51"/>
     <mergeCell ref="C50:G50"/>
     <mergeCell ref="A50:B50"/>
+    <mergeCell ref="C43:D43"/>
+    <mergeCell ref="E36:F36"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="C42:D42"/>
+    <mergeCell ref="E42:F42"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="E39:F39"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="E40:F40"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="E41:F41"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="E37:F37"/>
     <mergeCell ref="C35:D35"/>
     <mergeCell ref="C36:D36"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="E27:F27"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="E28:F28"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="E30:F30"/>
-    <mergeCell ref="E29:F29"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="E31:F31"/>
-    <mergeCell ref="E32:F32"/>
-    <mergeCell ref="E33:F33"/>
-    <mergeCell ref="E34:F34"/>
-    <mergeCell ref="E35:F35"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="E25:F25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="E26:F26"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="E21:F21"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="E17:F17"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="E12:F12"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="A10:G10"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="C43:D43"/>
-    <mergeCell ref="E43:F43"/>
-    <mergeCell ref="C45:D45"/>
-    <mergeCell ref="E45:F45"/>
-    <mergeCell ref="C46:D46"/>
-    <mergeCell ref="E46:F46"/>
-    <mergeCell ref="C44:D44"/>
-    <mergeCell ref="E44:F44"/>
+    <mergeCell ref="E3:G3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="B2:D2"/>
   </mergeCells>
   <pageMargins left="0.51181102362204722" right="0.19685039370078741" top="0.31496062992125984" bottom="0" header="0.51181102362204722" footer="0.51181102362204722"/>
   <pageSetup paperSize="9" scale="83" fitToHeight="0" orientation="portrait" copies="3" r:id="rId1"/>
@@ -2460,51 +2478,51 @@
     </row>
     <row r="2" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="14"/>
-      <c r="B2" s="38" t="s">
+      <c r="B2" s="40" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="38"/>
-      <c r="D2" s="39"/>
-      <c r="E2" s="40" t="s">
+      <c r="C2" s="40"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="38"/>
-      <c r="G2" s="39"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="41"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="15"/>
-      <c r="B3" s="41" t="s">
+      <c r="B3" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="41"/>
-      <c r="D3" s="42"/>
-      <c r="E3" s="77" t="s">
+      <c r="C3" s="42"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="96" t="s">
         <v>28</v>
       </c>
-      <c r="F3" s="78"/>
-      <c r="G3" s="79"/>
+      <c r="F3" s="97"/>
+      <c r="G3" s="98"/>
     </row>
     <row r="4" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="14"/>
-      <c r="B4" s="38"/>
-      <c r="C4" s="38"/>
-      <c r="D4" s="39"/>
+      <c r="B4" s="40"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="41"/>
       <c r="E4" s="34"/>
       <c r="F4" s="34"/>
       <c r="G4" s="35"/>
     </row>
     <row r="5" spans="1:14" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="30"/>
-      <c r="B5" s="43" t="s">
+      <c r="B5" s="79" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="43"/>
-      <c r="D5" s="44"/>
-      <c r="E5" s="45" t="s">
+      <c r="C5" s="79"/>
+      <c r="D5" s="80"/>
+      <c r="E5" s="81" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="45"/>
-      <c r="G5" s="46"/>
+      <c r="F5" s="81"/>
+      <c r="G5" s="82"/>
     </row>
     <row r="6" spans="1:14" ht="4.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="16"/>
@@ -2528,45 +2546,45 @@
       <c r="A8" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B8" s="47" t="s">
+      <c r="B8" s="83" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="48"/>
-      <c r="D8" s="49"/>
+      <c r="C8" s="84"/>
+      <c r="D8" s="85"/>
       <c r="E8" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="F8" s="50" t="s">
+      <c r="F8" s="86" t="s">
         <v>24</v>
       </c>
-      <c r="G8" s="51"/>
+      <c r="G8" s="87"/>
       <c r="H8" s="4"/>
     </row>
     <row r="9" spans="1:14" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="52" t="s">
+      <c r="B9" s="88" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="53"/>
-      <c r="D9" s="54"/>
+      <c r="C9" s="89"/>
+      <c r="D9" s="90"/>
       <c r="E9" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="55" t="s">
+      <c r="F9" s="91" t="s">
         <v>25</v>
       </c>
-      <c r="G9" s="56"/>
+      <c r="G9" s="92"/>
     </row>
     <row r="10" spans="1:14" ht="5.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="57"/>
-      <c r="B10" s="57"/>
-      <c r="C10" s="57"/>
-      <c r="D10" s="57"/>
-      <c r="E10" s="57"/>
-      <c r="F10" s="57"/>
-      <c r="G10" s="57"/>
+      <c r="A10" s="93"/>
+      <c r="B10" s="93"/>
+      <c r="C10" s="93"/>
+      <c r="D10" s="93"/>
+      <c r="E10" s="93"/>
+      <c r="F10" s="93"/>
+      <c r="G10" s="93"/>
     </row>
     <row r="11" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
@@ -2575,14 +2593,14 @@
       <c r="B11" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="36" t="s">
+      <c r="C11" s="94" t="s">
         <v>7</v>
       </c>
-      <c r="D11" s="37"/>
-      <c r="E11" s="36" t="s">
+      <c r="D11" s="95"/>
+      <c r="E11" s="94" t="s">
         <v>3</v>
       </c>
-      <c r="F11" s="37"/>
+      <c r="F11" s="95"/>
       <c r="G11" s="22" t="s">
         <v>4</v>
       </c>
@@ -2594,14 +2612,14 @@
       <c r="B12" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C12" s="58" t="s">
+      <c r="C12" s="77" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="59"/>
-      <c r="E12" s="60" t="s">
+      <c r="D12" s="78"/>
+      <c r="E12" s="45" t="s">
         <v>37</v>
       </c>
-      <c r="F12" s="61"/>
+      <c r="F12" s="46"/>
       <c r="G12" s="23"/>
       <c r="H12" s="11"/>
       <c r="I12" s="5"/>
@@ -2614,10 +2632,10 @@
     <row r="13" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="12"/>
       <c r="B13" s="1"/>
-      <c r="C13" s="58"/>
-      <c r="D13" s="59"/>
-      <c r="E13" s="60"/>
-      <c r="F13" s="61"/>
+      <c r="C13" s="77"/>
+      <c r="D13" s="78"/>
+      <c r="E13" s="45"/>
+      <c r="F13" s="46"/>
       <c r="G13" s="23"/>
       <c r="H13" s="11"/>
       <c r="I13" s="8"/>
@@ -2628,413 +2646,413 @@
     <row r="14" spans="1:14" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="13"/>
       <c r="B14" s="1"/>
-      <c r="C14" s="58"/>
-      <c r="D14" s="59"/>
-      <c r="E14" s="60"/>
-      <c r="F14" s="61"/>
+      <c r="C14" s="77"/>
+      <c r="D14" s="78"/>
+      <c r="E14" s="45"/>
+      <c r="F14" s="46"/>
       <c r="G14" s="23"/>
       <c r="H14" s="11"/>
     </row>
     <row r="15" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="13"/>
       <c r="B15" s="1"/>
-      <c r="C15" s="58"/>
-      <c r="D15" s="59"/>
-      <c r="E15" s="60"/>
-      <c r="F15" s="61"/>
+      <c r="C15" s="77"/>
+      <c r="D15" s="78"/>
+      <c r="E15" s="45"/>
+      <c r="F15" s="46"/>
       <c r="G15" s="23"/>
       <c r="H15" s="11"/>
     </row>
     <row r="16" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="13"/>
       <c r="B16" s="2"/>
-      <c r="C16" s="58"/>
-      <c r="D16" s="59"/>
-      <c r="E16" s="60"/>
-      <c r="F16" s="61"/>
+      <c r="C16" s="77"/>
+      <c r="D16" s="78"/>
+      <c r="E16" s="45"/>
+      <c r="F16" s="46"/>
       <c r="G16" s="23"/>
       <c r="H16" s="11"/>
     </row>
     <row r="17" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="13"/>
       <c r="B17" s="2"/>
-      <c r="C17" s="58"/>
-      <c r="D17" s="59"/>
-      <c r="E17" s="60"/>
-      <c r="F17" s="61"/>
+      <c r="C17" s="77"/>
+      <c r="D17" s="78"/>
+      <c r="E17" s="45"/>
+      <c r="F17" s="46"/>
       <c r="G17" s="23"/>
       <c r="H17" s="11"/>
     </row>
     <row r="18" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="13"/>
       <c r="B18" s="2"/>
-      <c r="C18" s="62"/>
-      <c r="D18" s="63"/>
-      <c r="E18" s="60"/>
-      <c r="F18" s="61"/>
+      <c r="C18" s="47"/>
+      <c r="D18" s="48"/>
+      <c r="E18" s="45"/>
+      <c r="F18" s="46"/>
       <c r="G18" s="23"/>
       <c r="H18" s="11"/>
     </row>
     <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="13"/>
       <c r="B19" s="2"/>
-      <c r="C19" s="62"/>
-      <c r="D19" s="63"/>
-      <c r="E19" s="60"/>
-      <c r="F19" s="61"/>
+      <c r="C19" s="47"/>
+      <c r="D19" s="48"/>
+      <c r="E19" s="45"/>
+      <c r="F19" s="46"/>
       <c r="G19" s="23"/>
       <c r="H19" s="10"/>
     </row>
     <row r="20" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="13"/>
       <c r="B20" s="2"/>
-      <c r="C20" s="62"/>
-      <c r="D20" s="63"/>
-      <c r="E20" s="60"/>
-      <c r="F20" s="61"/>
+      <c r="C20" s="47"/>
+      <c r="D20" s="48"/>
+      <c r="E20" s="45"/>
+      <c r="F20" s="46"/>
       <c r="G20" s="23"/>
       <c r="H20" s="10"/>
     </row>
     <row r="21" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="13"/>
       <c r="B21" s="2"/>
-      <c r="C21" s="62"/>
-      <c r="D21" s="63"/>
-      <c r="E21" s="60"/>
-      <c r="F21" s="61"/>
+      <c r="C21" s="47"/>
+      <c r="D21" s="48"/>
+      <c r="E21" s="45"/>
+      <c r="F21" s="46"/>
       <c r="G21" s="23"/>
       <c r="H21" s="10"/>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="13"/>
       <c r="B22" s="2"/>
-      <c r="C22" s="62"/>
-      <c r="D22" s="63"/>
-      <c r="E22" s="60"/>
-      <c r="F22" s="61"/>
+      <c r="C22" s="47"/>
+      <c r="D22" s="48"/>
+      <c r="E22" s="45"/>
+      <c r="F22" s="46"/>
       <c r="G22" s="23"/>
       <c r="H22" s="10"/>
     </row>
     <row r="23" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="13"/>
       <c r="B23" s="2"/>
-      <c r="C23" s="62"/>
-      <c r="D23" s="63"/>
-      <c r="E23" s="60"/>
-      <c r="F23" s="61"/>
+      <c r="C23" s="47"/>
+      <c r="D23" s="48"/>
+      <c r="E23" s="45"/>
+      <c r="F23" s="46"/>
       <c r="G23" s="23"/>
       <c r="H23" s="10"/>
     </row>
     <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="13"/>
       <c r="B24" s="2"/>
-      <c r="C24" s="62"/>
-      <c r="D24" s="63"/>
-      <c r="E24" s="60"/>
-      <c r="F24" s="61"/>
+      <c r="C24" s="47"/>
+      <c r="D24" s="48"/>
+      <c r="E24" s="45"/>
+      <c r="F24" s="46"/>
       <c r="G24" s="23"/>
       <c r="H24" s="10"/>
     </row>
     <row r="25" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="13"/>
       <c r="B25" s="2"/>
-      <c r="C25" s="62"/>
-      <c r="D25" s="63"/>
-      <c r="E25" s="60"/>
-      <c r="F25" s="61"/>
+      <c r="C25" s="47"/>
+      <c r="D25" s="48"/>
+      <c r="E25" s="45"/>
+      <c r="F25" s="46"/>
       <c r="G25" s="23"/>
       <c r="H25" s="10"/>
     </row>
     <row r="26" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="13"/>
       <c r="B26" s="2"/>
-      <c r="C26" s="62"/>
-      <c r="D26" s="63"/>
-      <c r="E26" s="60"/>
-      <c r="F26" s="61"/>
+      <c r="C26" s="47"/>
+      <c r="D26" s="48"/>
+      <c r="E26" s="45"/>
+      <c r="F26" s="46"/>
       <c r="G26" s="23"/>
       <c r="H26" s="10"/>
     </row>
     <row r="27" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="13"/>
       <c r="B27" s="2"/>
-      <c r="C27" s="62"/>
-      <c r="D27" s="63"/>
-      <c r="E27" s="60"/>
-      <c r="F27" s="61"/>
+      <c r="C27" s="47"/>
+      <c r="D27" s="48"/>
+      <c r="E27" s="45"/>
+      <c r="F27" s="46"/>
       <c r="G27" s="23"/>
       <c r="H27" s="10"/>
     </row>
     <row r="28" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="13"/>
       <c r="B28" s="2"/>
-      <c r="C28" s="64"/>
-      <c r="D28" s="65"/>
-      <c r="E28" s="60"/>
-      <c r="F28" s="61"/>
+      <c r="C28" s="75"/>
+      <c r="D28" s="76"/>
+      <c r="E28" s="45"/>
+      <c r="F28" s="46"/>
       <c r="G28" s="23"/>
       <c r="H28" s="10"/>
     </row>
     <row r="29" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="13"/>
       <c r="B29" s="2"/>
-      <c r="C29" s="64"/>
-      <c r="D29" s="65"/>
-      <c r="E29" s="60"/>
-      <c r="F29" s="61"/>
+      <c r="C29" s="75"/>
+      <c r="D29" s="76"/>
+      <c r="E29" s="45"/>
+      <c r="F29" s="46"/>
       <c r="G29" s="23"/>
       <c r="H29" s="10"/>
     </row>
     <row r="30" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="13"/>
       <c r="B30" s="2"/>
-      <c r="C30" s="64"/>
-      <c r="D30" s="65"/>
-      <c r="E30" s="60"/>
-      <c r="F30" s="61"/>
+      <c r="C30" s="75"/>
+      <c r="D30" s="76"/>
+      <c r="E30" s="45"/>
+      <c r="F30" s="46"/>
       <c r="G30" s="23"/>
       <c r="H30" s="10"/>
     </row>
     <row r="31" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="13"/>
       <c r="B31" s="2"/>
-      <c r="C31" s="62"/>
-      <c r="D31" s="63"/>
-      <c r="E31" s="60"/>
-      <c r="F31" s="61"/>
+      <c r="C31" s="47"/>
+      <c r="D31" s="48"/>
+      <c r="E31" s="45"/>
+      <c r="F31" s="46"/>
       <c r="G31" s="23"/>
       <c r="H31" s="10"/>
     </row>
     <row r="32" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="13"/>
       <c r="B32" s="2"/>
-      <c r="C32" s="62"/>
-      <c r="D32" s="63"/>
-      <c r="E32" s="60"/>
-      <c r="F32" s="61"/>
+      <c r="C32" s="47"/>
+      <c r="D32" s="48"/>
+      <c r="E32" s="45"/>
+      <c r="F32" s="46"/>
       <c r="G32" s="23"/>
       <c r="H32" s="10"/>
     </row>
     <row r="33" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="13"/>
       <c r="B33" s="2"/>
-      <c r="C33" s="62"/>
-      <c r="D33" s="63"/>
-      <c r="E33" s="60"/>
-      <c r="F33" s="61"/>
+      <c r="C33" s="47"/>
+      <c r="D33" s="48"/>
+      <c r="E33" s="45"/>
+      <c r="F33" s="46"/>
       <c r="G33" s="23"/>
       <c r="H33" s="10"/>
     </row>
     <row r="34" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="13"/>
       <c r="B34" s="2"/>
-      <c r="C34" s="62"/>
-      <c r="D34" s="63"/>
-      <c r="E34" s="60"/>
-      <c r="F34" s="61"/>
+      <c r="C34" s="47"/>
+      <c r="D34" s="48"/>
+      <c r="E34" s="45"/>
+      <c r="F34" s="46"/>
       <c r="G34" s="23"/>
       <c r="H34" s="10"/>
     </row>
     <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="13"/>
       <c r="B35" s="2"/>
-      <c r="C35" s="62"/>
-      <c r="D35" s="63"/>
-      <c r="E35" s="60"/>
-      <c r="F35" s="61"/>
+      <c r="C35" s="47"/>
+      <c r="D35" s="48"/>
+      <c r="E35" s="45"/>
+      <c r="F35" s="46"/>
       <c r="G35" s="23"/>
       <c r="H35" s="10"/>
     </row>
     <row r="36" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="13"/>
       <c r="B36" s="2"/>
-      <c r="C36" s="62"/>
-      <c r="D36" s="63"/>
-      <c r="E36" s="60"/>
-      <c r="F36" s="61"/>
+      <c r="C36" s="47"/>
+      <c r="D36" s="48"/>
+      <c r="E36" s="45"/>
+      <c r="F36" s="46"/>
       <c r="G36" s="23"/>
       <c r="H36" s="10"/>
     </row>
     <row r="37" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="13"/>
       <c r="B37" s="2"/>
-      <c r="C37" s="62"/>
-      <c r="D37" s="63"/>
-      <c r="E37" s="60"/>
-      <c r="F37" s="61"/>
+      <c r="C37" s="47"/>
+      <c r="D37" s="48"/>
+      <c r="E37" s="45"/>
+      <c r="F37" s="46"/>
       <c r="G37" s="23"/>
       <c r="H37" s="10"/>
     </row>
     <row r="38" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="13"/>
       <c r="B38" s="2"/>
-      <c r="C38" s="62"/>
-      <c r="D38" s="63"/>
-      <c r="E38" s="60"/>
-      <c r="F38" s="61"/>
+      <c r="C38" s="47"/>
+      <c r="D38" s="48"/>
+      <c r="E38" s="45"/>
+      <c r="F38" s="46"/>
       <c r="G38" s="23"/>
       <c r="H38" s="10"/>
     </row>
     <row r="39" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="13"/>
       <c r="B39" s="2"/>
-      <c r="C39" s="66"/>
-      <c r="D39" s="67"/>
-      <c r="E39" s="60"/>
-      <c r="F39" s="61"/>
+      <c r="C39" s="49"/>
+      <c r="D39" s="50"/>
+      <c r="E39" s="45"/>
+      <c r="F39" s="46"/>
       <c r="G39" s="23"/>
       <c r="H39" s="10"/>
     </row>
     <row r="40" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="13"/>
       <c r="B40" s="2"/>
-      <c r="C40" s="62"/>
-      <c r="D40" s="63"/>
-      <c r="E40" s="60"/>
-      <c r="F40" s="61"/>
+      <c r="C40" s="47"/>
+      <c r="D40" s="48"/>
+      <c r="E40" s="45"/>
+      <c r="F40" s="46"/>
       <c r="G40" s="23"/>
       <c r="H40" s="10"/>
     </row>
     <row r="41" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="13"/>
       <c r="B41" s="2"/>
-      <c r="C41" s="62"/>
-      <c r="D41" s="63"/>
-      <c r="E41" s="60"/>
-      <c r="F41" s="61"/>
+      <c r="C41" s="47"/>
+      <c r="D41" s="48"/>
+      <c r="E41" s="45"/>
+      <c r="F41" s="46"/>
       <c r="G41" s="23"/>
       <c r="H41" s="10"/>
     </row>
     <row r="42" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="13"/>
       <c r="B42" s="2"/>
-      <c r="C42" s="62"/>
-      <c r="D42" s="63"/>
-      <c r="E42" s="60"/>
-      <c r="F42" s="61"/>
+      <c r="C42" s="47"/>
+      <c r="D42" s="48"/>
+      <c r="E42" s="45"/>
+      <c r="F42" s="46"/>
       <c r="G42" s="23"/>
       <c r="H42" s="10"/>
     </row>
     <row r="43" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="13"/>
       <c r="B43" s="2"/>
-      <c r="C43" s="62"/>
-      <c r="D43" s="63"/>
-      <c r="E43" s="60"/>
-      <c r="F43" s="61"/>
+      <c r="C43" s="47"/>
+      <c r="D43" s="48"/>
+      <c r="E43" s="45"/>
+      <c r="F43" s="46"/>
       <c r="G43" s="23"/>
       <c r="H43" s="10"/>
     </row>
     <row r="44" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="13"/>
       <c r="B44" s="2"/>
-      <c r="C44" s="62"/>
-      <c r="D44" s="63"/>
-      <c r="E44" s="60"/>
-      <c r="F44" s="61"/>
+      <c r="C44" s="47"/>
+      <c r="D44" s="48"/>
+      <c r="E44" s="45"/>
+      <c r="F44" s="46"/>
       <c r="G44" s="23"/>
       <c r="H44" s="10"/>
     </row>
     <row r="45" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="13"/>
       <c r="B45" s="2"/>
-      <c r="C45" s="62"/>
-      <c r="D45" s="63"/>
-      <c r="E45" s="60"/>
-      <c r="F45" s="61"/>
+      <c r="C45" s="47"/>
+      <c r="D45" s="48"/>
+      <c r="E45" s="45"/>
+      <c r="F45" s="46"/>
       <c r="G45" s="23"/>
       <c r="H45" s="10"/>
     </row>
     <row r="46" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="13"/>
       <c r="B46" s="2"/>
-      <c r="C46" s="62"/>
-      <c r="D46" s="63"/>
-      <c r="E46" s="60"/>
-      <c r="F46" s="61"/>
+      <c r="C46" s="47"/>
+      <c r="D46" s="48"/>
+      <c r="E46" s="45"/>
+      <c r="F46" s="46"/>
       <c r="G46" s="23"/>
       <c r="H46" s="10"/>
     </row>
     <row r="47" spans="1:8" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A47" s="13"/>
       <c r="B47" s="2"/>
-      <c r="C47" s="62"/>
-      <c r="D47" s="63"/>
-      <c r="E47" s="60"/>
-      <c r="F47" s="61"/>
+      <c r="C47" s="47"/>
+      <c r="D47" s="48"/>
+      <c r="E47" s="45"/>
+      <c r="F47" s="46"/>
       <c r="G47" s="23"/>
     </row>
     <row r="48" spans="1:8" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="80" t="s">
+      <c r="A48" s="63" t="s">
         <v>14</v>
       </c>
-      <c r="B48" s="81"/>
-      <c r="C48" s="81"/>
-      <c r="D48" s="81"/>
-      <c r="E48" s="82"/>
-      <c r="F48" s="83"/>
-      <c r="G48" s="84"/>
+      <c r="B48" s="64"/>
+      <c r="C48" s="64"/>
+      <c r="D48" s="64"/>
+      <c r="E48" s="65"/>
+      <c r="F48" s="66"/>
+      <c r="G48" s="67"/>
     </row>
     <row r="49" spans="1:7" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="50" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="85" t="s">
+      <c r="A50" s="73" t="s">
         <v>20</v>
       </c>
-      <c r="B50" s="86"/>
-      <c r="C50" s="87" t="s">
+      <c r="B50" s="74"/>
+      <c r="C50" s="70" t="s">
         <v>26</v>
       </c>
-      <c r="D50" s="88"/>
-      <c r="E50" s="88"/>
-      <c r="F50" s="88"/>
-      <c r="G50" s="89"/>
+      <c r="D50" s="71"/>
+      <c r="E50" s="71"/>
+      <c r="F50" s="71"/>
+      <c r="G50" s="72"/>
     </row>
     <row r="51" spans="1:7" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="75" t="s">
+      <c r="A51" s="55" t="s">
         <v>15</v>
       </c>
-      <c r="B51" s="76"/>
-      <c r="C51" s="90"/>
-      <c r="D51" s="91"/>
-      <c r="E51" s="92" t="s">
+      <c r="B51" s="56"/>
+      <c r="C51" s="68"/>
+      <c r="D51" s="69"/>
+      <c r="E51" s="57" t="s">
         <v>5</v>
       </c>
-      <c r="F51" s="93"/>
-      <c r="G51" s="94"/>
+      <c r="F51" s="58"/>
+      <c r="G51" s="59"/>
     </row>
     <row r="52" spans="1:7" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A52" s="75" t="s">
+      <c r="A52" s="55" t="s">
         <v>27</v>
       </c>
-      <c r="B52" s="76"/>
+      <c r="B52" s="56"/>
       <c r="C52" s="32" t="s">
         <v>29</v>
       </c>
       <c r="D52" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="E52" s="68" t="s">
+      <c r="E52" s="60" t="s">
         <v>30</v>
       </c>
-      <c r="F52" s="69"/>
-      <c r="G52" s="70"/>
+      <c r="F52" s="61"/>
+      <c r="G52" s="62"/>
     </row>
     <row r="53" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="71" t="s">
+      <c r="A53" s="51" t="s">
         <v>16</v>
       </c>
-      <c r="B53" s="72"/>
+      <c r="B53" s="52"/>
       <c r="C53" s="33" t="s">
         <v>33</v>
       </c>
       <c r="D53" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="E53" s="73" t="s">
+      <c r="E53" s="53" t="s">
         <v>32</v>
       </c>
-      <c r="F53" s="73"/>
-      <c r="G53" s="74"/>
+      <c r="F53" s="53"/>
+      <c r="G53" s="54"/>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.2">
       <c r="G54" s="3" t="s">
@@ -3043,6 +3061,87 @@
     </row>
   </sheetData>
   <mergeCells count="97">
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="A10:G10"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="E28:F28"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="E30:F30"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="E32:F32"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="E33:F33"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="E34:F34"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="E35:F35"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="E36:F36"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="E37:F37"/>
+    <mergeCell ref="C38:D38"/>
+    <mergeCell ref="E38:F38"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="E39:F39"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="E40:F40"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="E41:F41"/>
+    <mergeCell ref="C47:D47"/>
+    <mergeCell ref="E47:F47"/>
+    <mergeCell ref="C42:D42"/>
+    <mergeCell ref="E42:F42"/>
+    <mergeCell ref="C43:D43"/>
+    <mergeCell ref="E43:F43"/>
+    <mergeCell ref="C44:D44"/>
+    <mergeCell ref="E44:F44"/>
     <mergeCell ref="E52:G52"/>
     <mergeCell ref="A53:B53"/>
     <mergeCell ref="E53:G53"/>
@@ -3059,87 +3158,6 @@
     <mergeCell ref="E45:F45"/>
     <mergeCell ref="C46:D46"/>
     <mergeCell ref="E46:F46"/>
-    <mergeCell ref="C47:D47"/>
-    <mergeCell ref="E47:F47"/>
-    <mergeCell ref="C42:D42"/>
-    <mergeCell ref="E42:F42"/>
-    <mergeCell ref="C43:D43"/>
-    <mergeCell ref="E43:F43"/>
-    <mergeCell ref="C44:D44"/>
-    <mergeCell ref="E44:F44"/>
-    <mergeCell ref="C39:D39"/>
-    <mergeCell ref="E39:F39"/>
-    <mergeCell ref="C40:D40"/>
-    <mergeCell ref="E40:F40"/>
-    <mergeCell ref="C41:D41"/>
-    <mergeCell ref="E41:F41"/>
-    <mergeCell ref="C36:D36"/>
-    <mergeCell ref="E36:F36"/>
-    <mergeCell ref="C37:D37"/>
-    <mergeCell ref="E37:F37"/>
-    <mergeCell ref="C38:D38"/>
-    <mergeCell ref="E38:F38"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="E33:F33"/>
-    <mergeCell ref="C34:D34"/>
-    <mergeCell ref="E34:F34"/>
-    <mergeCell ref="C35:D35"/>
-    <mergeCell ref="E35:F35"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="E30:F30"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="E31:F31"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="E32:F32"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="E27:F27"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="E28:F28"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="E29:F29"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="E25:F25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="E26:F26"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="E21:F21"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="E17:F17"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="E12:F12"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="A10:G10"/>
   </mergeCells>
   <pageMargins left="0.51181102362204722" right="0.19685039370078741" top="0.31496062992125984" bottom="0" header="0.51181102362204722" footer="0.51181102362204722"/>
   <pageSetup paperSize="9" scale="83" fitToHeight="0" orientation="portrait" copies="3" r:id="rId1"/>

</xml_diff>

<commit_message>
login_register page background, icons, mr to property assignment
</commit_message>
<xml_diff>
--- a/procurement_documents/PR Template.xlsx
+++ b/procurement_documents/PR Template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emman\itrac\procurement_documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\I-TRAC\I-TRAC\procurement_documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76FDDAE1-7AA0-4405-B9AA-108DE8B8A00F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FE5E816-BD42-42B1-837C-D4D08562CF1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="739" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="739" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PR" sheetId="59" r:id="rId1"/>
@@ -163,8 +163,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="mm/dd/yy;@"/>
   </numFmts>
   <fonts count="26" x14ac:knownFonts="1">
@@ -836,19 +836,19 @@
   <cellStyleXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="99">
+  <cellXfs count="100">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -873,10 +873,10 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -908,7 +908,7 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="43" fontId="5" fillId="2" borderId="30" xfId="9" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="30" xfId="9" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="32" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -947,11 +947,17 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -959,68 +965,19 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="5" fillId="2" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="36" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="22" fontId="21" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="22" fontId="21" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="5" fillId="2" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1029,14 +986,39 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1046,33 +1028,6 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -1088,37 +1043,85 @@
     <xf numFmtId="39" fontId="25" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="36" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="22" fontId="21" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="22" fontId="21" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="10">
@@ -1769,51 +1772,51 @@
     </row>
     <row r="2" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="14"/>
-      <c r="B2" s="38" t="s">
+      <c r="B2" s="40" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="38"/>
-      <c r="D2" s="39"/>
-      <c r="E2" s="40" t="s">
+      <c r="C2" s="40"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="38"/>
-      <c r="G2" s="39"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="41"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="15"/>
-      <c r="B3" s="41" t="s">
+      <c r="B3" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="41"/>
-      <c r="D3" s="42"/>
-      <c r="E3" s="95" t="s">
+      <c r="C3" s="42"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="37" t="s">
         <v>28</v>
       </c>
-      <c r="F3" s="96"/>
-      <c r="G3" s="97"/>
+      <c r="F3" s="38"/>
+      <c r="G3" s="39"/>
     </row>
     <row r="4" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="14"/>
-      <c r="B4" s="38"/>
-      <c r="C4" s="38"/>
-      <c r="D4" s="39"/>
+      <c r="B4" s="40"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="41"/>
       <c r="E4" s="34"/>
       <c r="F4" s="34"/>
       <c r="G4" s="35"/>
     </row>
     <row r="5" spans="1:14" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="30"/>
-      <c r="B5" s="43" t="s">
+      <c r="B5" s="79" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="43"/>
-      <c r="D5" s="44"/>
-      <c r="E5" s="45" t="s">
+      <c r="C5" s="79"/>
+      <c r="D5" s="80"/>
+      <c r="E5" s="81" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="45"/>
-      <c r="G5" s="46"/>
+      <c r="F5" s="81"/>
+      <c r="G5" s="82"/>
     </row>
     <row r="6" spans="1:14" ht="4.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="16"/>
@@ -1837,37 +1840,37 @@
       <c r="A8" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B8" s="47"/>
-      <c r="C8" s="48"/>
-      <c r="D8" s="49"/>
+      <c r="B8" s="83"/>
+      <c r="C8" s="84"/>
+      <c r="D8" s="85"/>
       <c r="E8" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="F8" s="50"/>
-      <c r="G8" s="51"/>
+      <c r="F8" s="86"/>
+      <c r="G8" s="87"/>
       <c r="H8" s="4"/>
     </row>
     <row r="9" spans="1:14" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="52"/>
-      <c r="C9" s="53"/>
-      <c r="D9" s="54"/>
+      <c r="B9" s="88"/>
+      <c r="C9" s="89"/>
+      <c r="D9" s="90"/>
       <c r="E9" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="55"/>
-      <c r="G9" s="56"/>
+      <c r="F9" s="91"/>
+      <c r="G9" s="92"/>
     </row>
     <row r="10" spans="1:14" ht="5.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="57"/>
-      <c r="B10" s="57"/>
-      <c r="C10" s="57"/>
-      <c r="D10" s="57"/>
-      <c r="E10" s="57"/>
-      <c r="F10" s="57"/>
-      <c r="G10" s="57"/>
+      <c r="A10" s="93"/>
+      <c r="B10" s="93"/>
+      <c r="C10" s="93"/>
+      <c r="D10" s="93"/>
+      <c r="E10" s="93"/>
+      <c r="F10" s="93"/>
+      <c r="G10" s="93"/>
     </row>
     <row r="11" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
@@ -1876,25 +1879,25 @@
       <c r="B11" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="36" t="s">
+      <c r="C11" s="94" t="s">
         <v>7</v>
       </c>
-      <c r="D11" s="37"/>
-      <c r="E11" s="36" t="s">
+      <c r="D11" s="95"/>
+      <c r="E11" s="94" t="s">
         <v>3</v>
       </c>
-      <c r="F11" s="37"/>
+      <c r="F11" s="95"/>
       <c r="G11" s="22" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="12"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="58"/>
-      <c r="D12" s="59"/>
-      <c r="E12" s="60"/>
-      <c r="F12" s="61"/>
+      <c r="B12" s="99"/>
+      <c r="C12" s="77"/>
+      <c r="D12" s="78"/>
+      <c r="E12" s="45"/>
+      <c r="F12" s="46"/>
       <c r="G12" s="23"/>
       <c r="H12" s="11"/>
       <c r="I12" s="5"/>
@@ -1906,11 +1909,11 @@
     </row>
     <row r="13" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="12"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="58"/>
-      <c r="D13" s="59"/>
-      <c r="E13" s="60"/>
-      <c r="F13" s="61"/>
+      <c r="B13" s="99"/>
+      <c r="C13" s="77"/>
+      <c r="D13" s="78"/>
+      <c r="E13" s="45"/>
+      <c r="F13" s="46"/>
       <c r="G13" s="23"/>
       <c r="H13" s="11"/>
       <c r="I13" s="8"/>
@@ -1920,429 +1923,470 @@
     </row>
     <row r="14" spans="1:14" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="13"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="58"/>
-      <c r="D14" s="59"/>
-      <c r="E14" s="60"/>
-      <c r="F14" s="61"/>
+      <c r="B14" s="99"/>
+      <c r="C14" s="77"/>
+      <c r="D14" s="78"/>
+      <c r="E14" s="45"/>
+      <c r="F14" s="46"/>
       <c r="G14" s="23"/>
       <c r="H14" s="11"/>
     </row>
     <row r="15" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="13"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="58"/>
-      <c r="D15" s="59"/>
-      <c r="E15" s="60"/>
-      <c r="F15" s="61"/>
+      <c r="B15" s="99"/>
+      <c r="C15" s="77"/>
+      <c r="D15" s="78"/>
+      <c r="E15" s="45"/>
+      <c r="F15" s="46"/>
       <c r="G15" s="23"/>
       <c r="H15" s="11"/>
     </row>
     <row r="16" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="13"/>
       <c r="B16" s="2"/>
-      <c r="C16" s="58"/>
-      <c r="D16" s="59"/>
-      <c r="E16" s="60"/>
-      <c r="F16" s="61"/>
+      <c r="C16" s="77"/>
+      <c r="D16" s="78"/>
+      <c r="E16" s="45"/>
+      <c r="F16" s="46"/>
       <c r="G16" s="23"/>
       <c r="H16" s="11"/>
     </row>
     <row r="17" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="13"/>
       <c r="B17" s="2"/>
-      <c r="C17" s="58"/>
-      <c r="D17" s="59"/>
-      <c r="E17" s="60"/>
-      <c r="F17" s="61"/>
+      <c r="C17" s="77"/>
+      <c r="D17" s="78"/>
+      <c r="E17" s="45"/>
+      <c r="F17" s="46"/>
       <c r="G17" s="23"/>
       <c r="H17" s="11"/>
     </row>
     <row r="18" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="13"/>
       <c r="B18" s="2"/>
-      <c r="C18" s="62"/>
-      <c r="D18" s="63"/>
-      <c r="E18" s="60"/>
-      <c r="F18" s="61"/>
+      <c r="C18" s="47"/>
+      <c r="D18" s="48"/>
+      <c r="E18" s="45"/>
+      <c r="F18" s="46"/>
       <c r="G18" s="23"/>
       <c r="H18" s="11"/>
     </row>
     <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="13"/>
       <c r="B19" s="2"/>
-      <c r="C19" s="62"/>
-      <c r="D19" s="63"/>
-      <c r="E19" s="60"/>
-      <c r="F19" s="61"/>
+      <c r="C19" s="47"/>
+      <c r="D19" s="48"/>
+      <c r="E19" s="45"/>
+      <c r="F19" s="46"/>
       <c r="G19" s="23"/>
       <c r="H19" s="10"/>
     </row>
     <row r="20" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="13"/>
       <c r="B20" s="2"/>
-      <c r="C20" s="62"/>
-      <c r="D20" s="63"/>
-      <c r="E20" s="60"/>
-      <c r="F20" s="61"/>
+      <c r="C20" s="47"/>
+      <c r="D20" s="48"/>
+      <c r="E20" s="45"/>
+      <c r="F20" s="46"/>
       <c r="G20" s="23"/>
       <c r="H20" s="10"/>
     </row>
     <row r="21" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="13"/>
       <c r="B21" s="2"/>
-      <c r="C21" s="62"/>
-      <c r="D21" s="63"/>
-      <c r="E21" s="60"/>
-      <c r="F21" s="61"/>
+      <c r="C21" s="47"/>
+      <c r="D21" s="48"/>
+      <c r="E21" s="45"/>
+      <c r="F21" s="46"/>
       <c r="G21" s="23"/>
       <c r="H21" s="10"/>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="13"/>
       <c r="B22" s="2"/>
-      <c r="C22" s="62"/>
-      <c r="D22" s="63"/>
-      <c r="E22" s="60"/>
-      <c r="F22" s="61"/>
+      <c r="C22" s="47"/>
+      <c r="D22" s="48"/>
+      <c r="E22" s="45"/>
+      <c r="F22" s="46"/>
       <c r="G22" s="23"/>
       <c r="H22" s="10"/>
     </row>
     <row r="23" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="13"/>
       <c r="B23" s="2"/>
-      <c r="C23" s="62"/>
-      <c r="D23" s="63"/>
-      <c r="E23" s="60"/>
-      <c r="F23" s="61"/>
+      <c r="C23" s="47"/>
+      <c r="D23" s="48"/>
+      <c r="E23" s="45"/>
+      <c r="F23" s="46"/>
       <c r="G23" s="23"/>
       <c r="H23" s="10"/>
     </row>
     <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="13"/>
       <c r="B24" s="2"/>
-      <c r="C24" s="62"/>
-      <c r="D24" s="63"/>
-      <c r="E24" s="60"/>
-      <c r="F24" s="61"/>
+      <c r="C24" s="47"/>
+      <c r="D24" s="48"/>
+      <c r="E24" s="45"/>
+      <c r="F24" s="46"/>
       <c r="G24" s="23"/>
       <c r="H24" s="10"/>
     </row>
     <row r="25" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="13"/>
       <c r="B25" s="2"/>
-      <c r="C25" s="62"/>
-      <c r="D25" s="63"/>
-      <c r="E25" s="60"/>
-      <c r="F25" s="61"/>
+      <c r="C25" s="47"/>
+      <c r="D25" s="48"/>
+      <c r="E25" s="45"/>
+      <c r="F25" s="46"/>
       <c r="G25" s="23"/>
       <c r="H25" s="10"/>
     </row>
     <row r="26" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="13"/>
       <c r="B26" s="2"/>
-      <c r="C26" s="62"/>
-      <c r="D26" s="63"/>
-      <c r="E26" s="60"/>
-      <c r="F26" s="61"/>
+      <c r="C26" s="47"/>
+      <c r="D26" s="48"/>
+      <c r="E26" s="45"/>
+      <c r="F26" s="46"/>
       <c r="G26" s="23"/>
       <c r="H26" s="10"/>
     </row>
     <row r="27" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="13"/>
       <c r="B27" s="2"/>
-      <c r="C27" s="62"/>
-      <c r="D27" s="63"/>
-      <c r="E27" s="60"/>
-      <c r="F27" s="61"/>
+      <c r="C27" s="47"/>
+      <c r="D27" s="48"/>
+      <c r="E27" s="45"/>
+      <c r="F27" s="46"/>
       <c r="G27" s="23"/>
       <c r="H27" s="10"/>
     </row>
     <row r="28" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="13"/>
       <c r="B28" s="2"/>
-      <c r="C28" s="64"/>
-      <c r="D28" s="65"/>
-      <c r="E28" s="60"/>
-      <c r="F28" s="61"/>
+      <c r="C28" s="75"/>
+      <c r="D28" s="76"/>
+      <c r="E28" s="45"/>
+      <c r="F28" s="46"/>
       <c r="G28" s="23"/>
       <c r="H28" s="10"/>
     </row>
     <row r="29" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="13"/>
       <c r="B29" s="2"/>
-      <c r="C29" s="64"/>
-      <c r="D29" s="65"/>
-      <c r="E29" s="60"/>
-      <c r="F29" s="61"/>
+      <c r="C29" s="75"/>
+      <c r="D29" s="76"/>
+      <c r="E29" s="45"/>
+      <c r="F29" s="46"/>
       <c r="G29" s="23"/>
       <c r="H29" s="10"/>
     </row>
     <row r="30" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="13"/>
       <c r="B30" s="2"/>
-      <c r="C30" s="64"/>
-      <c r="D30" s="65"/>
-      <c r="E30" s="60"/>
-      <c r="F30" s="61"/>
+      <c r="C30" s="75"/>
+      <c r="D30" s="76"/>
+      <c r="E30" s="45"/>
+      <c r="F30" s="46"/>
       <c r="G30" s="23"/>
       <c r="H30" s="10"/>
     </row>
     <row r="31" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="13"/>
       <c r="B31" s="2"/>
-      <c r="C31" s="62"/>
-      <c r="D31" s="63"/>
-      <c r="E31" s="60"/>
-      <c r="F31" s="61"/>
+      <c r="C31" s="47"/>
+      <c r="D31" s="48"/>
+      <c r="E31" s="45"/>
+      <c r="F31" s="46"/>
       <c r="G31" s="23"/>
       <c r="H31" s="10"/>
     </row>
     <row r="32" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="13"/>
       <c r="B32" s="2"/>
-      <c r="C32" s="62"/>
-      <c r="D32" s="63"/>
-      <c r="E32" s="60"/>
-      <c r="F32" s="61"/>
+      <c r="C32" s="47"/>
+      <c r="D32" s="48"/>
+      <c r="E32" s="45"/>
+      <c r="F32" s="46"/>
       <c r="G32" s="23"/>
       <c r="H32" s="10"/>
     </row>
     <row r="33" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="13"/>
       <c r="B33" s="2"/>
-      <c r="C33" s="62"/>
-      <c r="D33" s="63"/>
-      <c r="E33" s="60"/>
-      <c r="F33" s="61"/>
+      <c r="C33" s="47"/>
+      <c r="D33" s="48"/>
+      <c r="E33" s="45"/>
+      <c r="F33" s="46"/>
       <c r="G33" s="23"/>
       <c r="H33" s="10"/>
     </row>
     <row r="34" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="13"/>
       <c r="B34" s="2"/>
-      <c r="C34" s="62"/>
-      <c r="D34" s="63"/>
-      <c r="E34" s="60"/>
-      <c r="F34" s="61"/>
+      <c r="C34" s="47"/>
+      <c r="D34" s="48"/>
+      <c r="E34" s="45"/>
+      <c r="F34" s="46"/>
       <c r="G34" s="23"/>
       <c r="H34" s="10"/>
     </row>
     <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="13"/>
       <c r="B35" s="2"/>
-      <c r="C35" s="62"/>
-      <c r="D35" s="63"/>
-      <c r="E35" s="60"/>
-      <c r="F35" s="61"/>
+      <c r="C35" s="47"/>
+      <c r="D35" s="48"/>
+      <c r="E35" s="45"/>
+      <c r="F35" s="46"/>
       <c r="G35" s="23"/>
       <c r="H35" s="10"/>
     </row>
     <row r="36" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="13"/>
       <c r="B36" s="2"/>
-      <c r="C36" s="62"/>
-      <c r="D36" s="63"/>
-      <c r="E36" s="60"/>
-      <c r="F36" s="61"/>
+      <c r="C36" s="47"/>
+      <c r="D36" s="48"/>
+      <c r="E36" s="45"/>
+      <c r="F36" s="46"/>
       <c r="G36" s="23"/>
       <c r="H36" s="10"/>
     </row>
     <row r="37" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="13"/>
       <c r="B37" s="2"/>
-      <c r="C37" s="62"/>
-      <c r="D37" s="63"/>
-      <c r="E37" s="60"/>
-      <c r="F37" s="61"/>
+      <c r="C37" s="47"/>
+      <c r="D37" s="48"/>
+      <c r="E37" s="45"/>
+      <c r="F37" s="46"/>
       <c r="G37" s="23"/>
       <c r="H37" s="10"/>
     </row>
     <row r="38" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="13"/>
       <c r="B38" s="2"/>
-      <c r="C38" s="62"/>
-      <c r="D38" s="63"/>
-      <c r="E38" s="60"/>
-      <c r="F38" s="61"/>
+      <c r="C38" s="47"/>
+      <c r="D38" s="48"/>
+      <c r="E38" s="45"/>
+      <c r="F38" s="46"/>
       <c r="G38" s="23"/>
       <c r="H38" s="10"/>
     </row>
     <row r="39" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="13"/>
       <c r="B39" s="2"/>
-      <c r="C39" s="66"/>
-      <c r="D39" s="67"/>
-      <c r="E39" s="60"/>
-      <c r="F39" s="61"/>
+      <c r="C39" s="49"/>
+      <c r="D39" s="50"/>
+      <c r="E39" s="45"/>
+      <c r="F39" s="46"/>
       <c r="G39" s="23"/>
       <c r="H39" s="10"/>
     </row>
     <row r="40" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="13"/>
       <c r="B40" s="2"/>
-      <c r="C40" s="62"/>
-      <c r="D40" s="63"/>
-      <c r="E40" s="60"/>
-      <c r="F40" s="61"/>
+      <c r="C40" s="47"/>
+      <c r="D40" s="48"/>
+      <c r="E40" s="45"/>
+      <c r="F40" s="46"/>
       <c r="G40" s="23"/>
       <c r="H40" s="10"/>
     </row>
     <row r="41" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="13"/>
       <c r="B41" s="2"/>
-      <c r="C41" s="62"/>
-      <c r="D41" s="63"/>
-      <c r="E41" s="60"/>
-      <c r="F41" s="61"/>
+      <c r="C41" s="47"/>
+      <c r="D41" s="48"/>
+      <c r="E41" s="45"/>
+      <c r="F41" s="46"/>
       <c r="G41" s="23"/>
       <c r="H41" s="10"/>
     </row>
     <row r="42" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="13"/>
       <c r="B42" s="2"/>
-      <c r="C42" s="62"/>
-      <c r="D42" s="63"/>
-      <c r="E42" s="60"/>
-      <c r="F42" s="61"/>
+      <c r="C42" s="47"/>
+      <c r="D42" s="48"/>
+      <c r="E42" s="45"/>
+      <c r="F42" s="46"/>
       <c r="G42" s="23"/>
       <c r="H42" s="10"/>
     </row>
     <row r="43" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="13"/>
       <c r="B43" s="2"/>
-      <c r="C43" s="62"/>
-      <c r="D43" s="63"/>
-      <c r="E43" s="60"/>
-      <c r="F43" s="61"/>
+      <c r="C43" s="47"/>
+      <c r="D43" s="48"/>
+      <c r="E43" s="45"/>
+      <c r="F43" s="46"/>
       <c r="G43" s="23"/>
       <c r="H43" s="10"/>
     </row>
     <row r="44" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="13"/>
       <c r="B44" s="2"/>
-      <c r="C44" s="62"/>
-      <c r="D44" s="63"/>
-      <c r="E44" s="60"/>
-      <c r="F44" s="61"/>
+      <c r="C44" s="47"/>
+      <c r="D44" s="48"/>
+      <c r="E44" s="45"/>
+      <c r="F44" s="46"/>
       <c r="G44" s="23"/>
       <c r="H44" s="10"/>
     </row>
     <row r="45" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="13"/>
       <c r="B45" s="2"/>
-      <c r="C45" s="62"/>
-      <c r="D45" s="63"/>
-      <c r="E45" s="60"/>
-      <c r="F45" s="61"/>
+      <c r="C45" s="47"/>
+      <c r="D45" s="48"/>
+      <c r="E45" s="45"/>
+      <c r="F45" s="46"/>
       <c r="G45" s="23"/>
       <c r="H45" s="10"/>
     </row>
     <row r="46" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="13"/>
       <c r="B46" s="2"/>
-      <c r="C46" s="62"/>
-      <c r="D46" s="63"/>
-      <c r="E46" s="60"/>
-      <c r="F46" s="61"/>
+      <c r="C46" s="47"/>
+      <c r="D46" s="48"/>
+      <c r="E46" s="45"/>
+      <c r="F46" s="46"/>
       <c r="G46" s="23"/>
       <c r="H46" s="10"/>
     </row>
     <row r="47" spans="1:8" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A47" s="13"/>
       <c r="B47" s="2"/>
-      <c r="C47" s="62"/>
-      <c r="D47" s="63"/>
-      <c r="E47" s="60"/>
-      <c r="F47" s="61"/>
+      <c r="C47" s="47"/>
+      <c r="D47" s="48"/>
+      <c r="E47" s="45"/>
+      <c r="F47" s="46"/>
       <c r="G47" s="23"/>
     </row>
     <row r="48" spans="1:8" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="80" t="s">
+      <c r="A48" s="63" t="s">
         <v>14</v>
       </c>
-      <c r="B48" s="81"/>
-      <c r="C48" s="81"/>
-      <c r="D48" s="81"/>
-      <c r="E48" s="82"/>
-      <c r="F48" s="83"/>
-      <c r="G48" s="84"/>
+      <c r="B48" s="64"/>
+      <c r="C48" s="64"/>
+      <c r="D48" s="64"/>
+      <c r="E48" s="65"/>
+      <c r="F48" s="66"/>
+      <c r="G48" s="67"/>
     </row>
     <row r="49" spans="1:7" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="50" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="85" t="s">
+      <c r="A50" s="73" t="s">
         <v>20</v>
       </c>
-      <c r="B50" s="86"/>
-      <c r="C50" s="87"/>
-      <c r="D50" s="88"/>
-      <c r="E50" s="88"/>
-      <c r="F50" s="88"/>
-      <c r="G50" s="89"/>
+      <c r="B50" s="74"/>
+      <c r="C50" s="70"/>
+      <c r="D50" s="71"/>
+      <c r="E50" s="71"/>
+      <c r="F50" s="71"/>
+      <c r="G50" s="72"/>
     </row>
     <row r="51" spans="1:7" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="75" t="s">
+      <c r="A51" s="55" t="s">
         <v>15</v>
       </c>
-      <c r="B51" s="76"/>
-      <c r="C51" s="90"/>
-      <c r="D51" s="91"/>
-      <c r="E51" s="92" t="s">
+      <c r="B51" s="56"/>
+      <c r="C51" s="68"/>
+      <c r="D51" s="69"/>
+      <c r="E51" s="57" t="s">
         <v>5</v>
       </c>
-      <c r="F51" s="93"/>
-      <c r="G51" s="94"/>
+      <c r="F51" s="58"/>
+      <c r="G51" s="59"/>
     </row>
     <row r="52" spans="1:7" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A52" s="75" t="s">
+      <c r="A52" s="55" t="s">
         <v>27</v>
       </c>
-      <c r="B52" s="76"/>
+      <c r="B52" s="56"/>
       <c r="C52" s="32"/>
       <c r="D52" s="31"/>
-      <c r="E52" s="68" t="s">
+      <c r="E52" s="60" t="s">
         <v>18</v>
       </c>
-      <c r="F52" s="69"/>
-      <c r="G52" s="70"/>
+      <c r="F52" s="61"/>
+      <c r="G52" s="62"/>
     </row>
     <row r="53" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="71" t="s">
+      <c r="A53" s="51" t="s">
         <v>16</v>
       </c>
-      <c r="B53" s="72"/>
+      <c r="B53" s="52"/>
       <c r="C53" s="33"/>
       <c r="D53" s="25"/>
-      <c r="E53" s="73" t="s">
+      <c r="E53" s="53" t="s">
         <v>6</v>
       </c>
-      <c r="F53" s="73"/>
-      <c r="G53" s="74"/>
+      <c r="F53" s="53"/>
+      <c r="G53" s="54"/>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="G54" s="98"/>
+      <c r="G54" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="97">
-    <mergeCell ref="E3:G3"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="E36:F36"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="C34:D34"/>
-    <mergeCell ref="C42:D42"/>
-    <mergeCell ref="E42:F42"/>
-    <mergeCell ref="C39:D39"/>
-    <mergeCell ref="E39:F39"/>
-    <mergeCell ref="C40:D40"/>
-    <mergeCell ref="E40:F40"/>
-    <mergeCell ref="C41:D41"/>
-    <mergeCell ref="E41:F41"/>
-    <mergeCell ref="C37:D37"/>
-    <mergeCell ref="E37:F37"/>
+    <mergeCell ref="E43:F43"/>
+    <mergeCell ref="C45:D45"/>
+    <mergeCell ref="E45:F45"/>
+    <mergeCell ref="C46:D46"/>
+    <mergeCell ref="E46:F46"/>
+    <mergeCell ref="C44:D44"/>
+    <mergeCell ref="E44:F44"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="A10:G10"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="E35:F35"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="E32:F32"/>
+    <mergeCell ref="E33:F33"/>
+    <mergeCell ref="E34:F34"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="E28:F28"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="E30:F30"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="C29:D29"/>
     <mergeCell ref="C47:D47"/>
     <mergeCell ref="E47:F47"/>
     <mergeCell ref="C38:D38"/>
@@ -2358,69 +2402,28 @@
     <mergeCell ref="C51:D51"/>
     <mergeCell ref="C50:G50"/>
     <mergeCell ref="A50:B50"/>
+    <mergeCell ref="C43:D43"/>
+    <mergeCell ref="E36:F36"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="C42:D42"/>
+    <mergeCell ref="E42:F42"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="E39:F39"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="E40:F40"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="E41:F41"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="E37:F37"/>
     <mergeCell ref="C35:D35"/>
     <mergeCell ref="C36:D36"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="E27:F27"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="E28:F28"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="E30:F30"/>
-    <mergeCell ref="E29:F29"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="E31:F31"/>
-    <mergeCell ref="E32:F32"/>
-    <mergeCell ref="E33:F33"/>
-    <mergeCell ref="E34:F34"/>
-    <mergeCell ref="E35:F35"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="E25:F25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="E26:F26"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="E21:F21"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="E17:F17"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="E12:F12"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="A10:G10"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="C43:D43"/>
-    <mergeCell ref="E43:F43"/>
-    <mergeCell ref="C45:D45"/>
-    <mergeCell ref="E45:F45"/>
-    <mergeCell ref="C46:D46"/>
-    <mergeCell ref="E46:F46"/>
-    <mergeCell ref="C44:D44"/>
-    <mergeCell ref="E44:F44"/>
+    <mergeCell ref="E3:G3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="B2:D2"/>
   </mergeCells>
   <pageMargins left="0.51181102362204722" right="0.19685039370078741" top="0.31496062992125984" bottom="0" header="0.51181102362204722" footer="0.51181102362204722"/>
   <pageSetup paperSize="9" scale="83" fitToHeight="0" orientation="portrait" copies="3" r:id="rId1"/>
@@ -2460,51 +2463,51 @@
     </row>
     <row r="2" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="14"/>
-      <c r="B2" s="38" t="s">
+      <c r="B2" s="40" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="38"/>
-      <c r="D2" s="39"/>
-      <c r="E2" s="40" t="s">
+      <c r="C2" s="40"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="38"/>
-      <c r="G2" s="39"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="41"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="15"/>
-      <c r="B3" s="41" t="s">
+      <c r="B3" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="41"/>
-      <c r="D3" s="42"/>
-      <c r="E3" s="77" t="s">
+      <c r="C3" s="42"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="96" t="s">
         <v>28</v>
       </c>
-      <c r="F3" s="78"/>
-      <c r="G3" s="79"/>
+      <c r="F3" s="97"/>
+      <c r="G3" s="98"/>
     </row>
     <row r="4" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="14"/>
-      <c r="B4" s="38"/>
-      <c r="C4" s="38"/>
-      <c r="D4" s="39"/>
+      <c r="B4" s="40"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="41"/>
       <c r="E4" s="34"/>
       <c r="F4" s="34"/>
       <c r="G4" s="35"/>
     </row>
     <row r="5" spans="1:14" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="30"/>
-      <c r="B5" s="43" t="s">
+      <c r="B5" s="79" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="43"/>
-      <c r="D5" s="44"/>
-      <c r="E5" s="45" t="s">
+      <c r="C5" s="79"/>
+      <c r="D5" s="80"/>
+      <c r="E5" s="81" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="45"/>
-      <c r="G5" s="46"/>
+      <c r="F5" s="81"/>
+      <c r="G5" s="82"/>
     </row>
     <row r="6" spans="1:14" ht="4.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="16"/>
@@ -2528,45 +2531,45 @@
       <c r="A8" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B8" s="47" t="s">
+      <c r="B8" s="83" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="48"/>
-      <c r="D8" s="49"/>
+      <c r="C8" s="84"/>
+      <c r="D8" s="85"/>
       <c r="E8" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="F8" s="50" t="s">
+      <c r="F8" s="86" t="s">
         <v>24</v>
       </c>
-      <c r="G8" s="51"/>
+      <c r="G8" s="87"/>
       <c r="H8" s="4"/>
     </row>
     <row r="9" spans="1:14" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="52" t="s">
+      <c r="B9" s="88" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="53"/>
-      <c r="D9" s="54"/>
+      <c r="C9" s="89"/>
+      <c r="D9" s="90"/>
       <c r="E9" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="55" t="s">
+      <c r="F9" s="91" t="s">
         <v>25</v>
       </c>
-      <c r="G9" s="56"/>
+      <c r="G9" s="92"/>
     </row>
     <row r="10" spans="1:14" ht="5.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="57"/>
-      <c r="B10" s="57"/>
-      <c r="C10" s="57"/>
-      <c r="D10" s="57"/>
-      <c r="E10" s="57"/>
-      <c r="F10" s="57"/>
-      <c r="G10" s="57"/>
+      <c r="A10" s="93"/>
+      <c r="B10" s="93"/>
+      <c r="C10" s="93"/>
+      <c r="D10" s="93"/>
+      <c r="E10" s="93"/>
+      <c r="F10" s="93"/>
+      <c r="G10" s="93"/>
     </row>
     <row r="11" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
@@ -2575,14 +2578,14 @@
       <c r="B11" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="36" t="s">
+      <c r="C11" s="94" t="s">
         <v>7</v>
       </c>
-      <c r="D11" s="37"/>
-      <c r="E11" s="36" t="s">
+      <c r="D11" s="95"/>
+      <c r="E11" s="94" t="s">
         <v>3</v>
       </c>
-      <c r="F11" s="37"/>
+      <c r="F11" s="95"/>
       <c r="G11" s="22" t="s">
         <v>4</v>
       </c>
@@ -2594,14 +2597,14 @@
       <c r="B12" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C12" s="58" t="s">
+      <c r="C12" s="77" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="59"/>
-      <c r="E12" s="60" t="s">
+      <c r="D12" s="78"/>
+      <c r="E12" s="45" t="s">
         <v>37</v>
       </c>
-      <c r="F12" s="61"/>
+      <c r="F12" s="46"/>
       <c r="G12" s="23"/>
       <c r="H12" s="11"/>
       <c r="I12" s="5"/>
@@ -2614,10 +2617,10 @@
     <row r="13" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="12"/>
       <c r="B13" s="1"/>
-      <c r="C13" s="58"/>
-      <c r="D13" s="59"/>
-      <c r="E13" s="60"/>
-      <c r="F13" s="61"/>
+      <c r="C13" s="77"/>
+      <c r="D13" s="78"/>
+      <c r="E13" s="45"/>
+      <c r="F13" s="46"/>
       <c r="G13" s="23"/>
       <c r="H13" s="11"/>
       <c r="I13" s="8"/>
@@ -2628,413 +2631,413 @@
     <row r="14" spans="1:14" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="13"/>
       <c r="B14" s="1"/>
-      <c r="C14" s="58"/>
-      <c r="D14" s="59"/>
-      <c r="E14" s="60"/>
-      <c r="F14" s="61"/>
+      <c r="C14" s="77"/>
+      <c r="D14" s="78"/>
+      <c r="E14" s="45"/>
+      <c r="F14" s="46"/>
       <c r="G14" s="23"/>
       <c r="H14" s="11"/>
     </row>
     <row r="15" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="13"/>
       <c r="B15" s="1"/>
-      <c r="C15" s="58"/>
-      <c r="D15" s="59"/>
-      <c r="E15" s="60"/>
-      <c r="F15" s="61"/>
+      <c r="C15" s="77"/>
+      <c r="D15" s="78"/>
+      <c r="E15" s="45"/>
+      <c r="F15" s="46"/>
       <c r="G15" s="23"/>
       <c r="H15" s="11"/>
     </row>
     <row r="16" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="13"/>
       <c r="B16" s="2"/>
-      <c r="C16" s="58"/>
-      <c r="D16" s="59"/>
-      <c r="E16" s="60"/>
-      <c r="F16" s="61"/>
+      <c r="C16" s="77"/>
+      <c r="D16" s="78"/>
+      <c r="E16" s="45"/>
+      <c r="F16" s="46"/>
       <c r="G16" s="23"/>
       <c r="H16" s="11"/>
     </row>
     <row r="17" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="13"/>
       <c r="B17" s="2"/>
-      <c r="C17" s="58"/>
-      <c r="D17" s="59"/>
-      <c r="E17" s="60"/>
-      <c r="F17" s="61"/>
+      <c r="C17" s="77"/>
+      <c r="D17" s="78"/>
+      <c r="E17" s="45"/>
+      <c r="F17" s="46"/>
       <c r="G17" s="23"/>
       <c r="H17" s="11"/>
     </row>
     <row r="18" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="13"/>
       <c r="B18" s="2"/>
-      <c r="C18" s="62"/>
-      <c r="D18" s="63"/>
-      <c r="E18" s="60"/>
-      <c r="F18" s="61"/>
+      <c r="C18" s="47"/>
+      <c r="D18" s="48"/>
+      <c r="E18" s="45"/>
+      <c r="F18" s="46"/>
       <c r="G18" s="23"/>
       <c r="H18" s="11"/>
     </row>
     <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="13"/>
       <c r="B19" s="2"/>
-      <c r="C19" s="62"/>
-      <c r="D19" s="63"/>
-      <c r="E19" s="60"/>
-      <c r="F19" s="61"/>
+      <c r="C19" s="47"/>
+      <c r="D19" s="48"/>
+      <c r="E19" s="45"/>
+      <c r="F19" s="46"/>
       <c r="G19" s="23"/>
       <c r="H19" s="10"/>
     </row>
     <row r="20" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="13"/>
       <c r="B20" s="2"/>
-      <c r="C20" s="62"/>
-      <c r="D20" s="63"/>
-      <c r="E20" s="60"/>
-      <c r="F20" s="61"/>
+      <c r="C20" s="47"/>
+      <c r="D20" s="48"/>
+      <c r="E20" s="45"/>
+      <c r="F20" s="46"/>
       <c r="G20" s="23"/>
       <c r="H20" s="10"/>
     </row>
     <row r="21" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="13"/>
       <c r="B21" s="2"/>
-      <c r="C21" s="62"/>
-      <c r="D21" s="63"/>
-      <c r="E21" s="60"/>
-      <c r="F21" s="61"/>
+      <c r="C21" s="47"/>
+      <c r="D21" s="48"/>
+      <c r="E21" s="45"/>
+      <c r="F21" s="46"/>
       <c r="G21" s="23"/>
       <c r="H21" s="10"/>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="13"/>
       <c r="B22" s="2"/>
-      <c r="C22" s="62"/>
-      <c r="D22" s="63"/>
-      <c r="E22" s="60"/>
-      <c r="F22" s="61"/>
+      <c r="C22" s="47"/>
+      <c r="D22" s="48"/>
+      <c r="E22" s="45"/>
+      <c r="F22" s="46"/>
       <c r="G22" s="23"/>
       <c r="H22" s="10"/>
     </row>
     <row r="23" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="13"/>
       <c r="B23" s="2"/>
-      <c r="C23" s="62"/>
-      <c r="D23" s="63"/>
-      <c r="E23" s="60"/>
-      <c r="F23" s="61"/>
+      <c r="C23" s="47"/>
+      <c r="D23" s="48"/>
+      <c r="E23" s="45"/>
+      <c r="F23" s="46"/>
       <c r="G23" s="23"/>
       <c r="H23" s="10"/>
     </row>
     <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="13"/>
       <c r="B24" s="2"/>
-      <c r="C24" s="62"/>
-      <c r="D24" s="63"/>
-      <c r="E24" s="60"/>
-      <c r="F24" s="61"/>
+      <c r="C24" s="47"/>
+      <c r="D24" s="48"/>
+      <c r="E24" s="45"/>
+      <c r="F24" s="46"/>
       <c r="G24" s="23"/>
       <c r="H24" s="10"/>
     </row>
     <row r="25" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="13"/>
       <c r="B25" s="2"/>
-      <c r="C25" s="62"/>
-      <c r="D25" s="63"/>
-      <c r="E25" s="60"/>
-      <c r="F25" s="61"/>
+      <c r="C25" s="47"/>
+      <c r="D25" s="48"/>
+      <c r="E25" s="45"/>
+      <c r="F25" s="46"/>
       <c r="G25" s="23"/>
       <c r="H25" s="10"/>
     </row>
     <row r="26" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="13"/>
       <c r="B26" s="2"/>
-      <c r="C26" s="62"/>
-      <c r="D26" s="63"/>
-      <c r="E26" s="60"/>
-      <c r="F26" s="61"/>
+      <c r="C26" s="47"/>
+      <c r="D26" s="48"/>
+      <c r="E26" s="45"/>
+      <c r="F26" s="46"/>
       <c r="G26" s="23"/>
       <c r="H26" s="10"/>
     </row>
     <row r="27" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="13"/>
       <c r="B27" s="2"/>
-      <c r="C27" s="62"/>
-      <c r="D27" s="63"/>
-      <c r="E27" s="60"/>
-      <c r="F27" s="61"/>
+      <c r="C27" s="47"/>
+      <c r="D27" s="48"/>
+      <c r="E27" s="45"/>
+      <c r="F27" s="46"/>
       <c r="G27" s="23"/>
       <c r="H27" s="10"/>
     </row>
     <row r="28" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="13"/>
       <c r="B28" s="2"/>
-      <c r="C28" s="64"/>
-      <c r="D28" s="65"/>
-      <c r="E28" s="60"/>
-      <c r="F28" s="61"/>
+      <c r="C28" s="75"/>
+      <c r="D28" s="76"/>
+      <c r="E28" s="45"/>
+      <c r="F28" s="46"/>
       <c r="G28" s="23"/>
       <c r="H28" s="10"/>
     </row>
     <row r="29" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="13"/>
       <c r="B29" s="2"/>
-      <c r="C29" s="64"/>
-      <c r="D29" s="65"/>
-      <c r="E29" s="60"/>
-      <c r="F29" s="61"/>
+      <c r="C29" s="75"/>
+      <c r="D29" s="76"/>
+      <c r="E29" s="45"/>
+      <c r="F29" s="46"/>
       <c r="G29" s="23"/>
       <c r="H29" s="10"/>
     </row>
     <row r="30" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="13"/>
       <c r="B30" s="2"/>
-      <c r="C30" s="64"/>
-      <c r="D30" s="65"/>
-      <c r="E30" s="60"/>
-      <c r="F30" s="61"/>
+      <c r="C30" s="75"/>
+      <c r="D30" s="76"/>
+      <c r="E30" s="45"/>
+      <c r="F30" s="46"/>
       <c r="G30" s="23"/>
       <c r="H30" s="10"/>
     </row>
     <row r="31" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="13"/>
       <c r="B31" s="2"/>
-      <c r="C31" s="62"/>
-      <c r="D31" s="63"/>
-      <c r="E31" s="60"/>
-      <c r="F31" s="61"/>
+      <c r="C31" s="47"/>
+      <c r="D31" s="48"/>
+      <c r="E31" s="45"/>
+      <c r="F31" s="46"/>
       <c r="G31" s="23"/>
       <c r="H31" s="10"/>
     </row>
     <row r="32" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="13"/>
       <c r="B32" s="2"/>
-      <c r="C32" s="62"/>
-      <c r="D32" s="63"/>
-      <c r="E32" s="60"/>
-      <c r="F32" s="61"/>
+      <c r="C32" s="47"/>
+      <c r="D32" s="48"/>
+      <c r="E32" s="45"/>
+      <c r="F32" s="46"/>
       <c r="G32" s="23"/>
       <c r="H32" s="10"/>
     </row>
     <row r="33" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="13"/>
       <c r="B33" s="2"/>
-      <c r="C33" s="62"/>
-      <c r="D33" s="63"/>
-      <c r="E33" s="60"/>
-      <c r="F33" s="61"/>
+      <c r="C33" s="47"/>
+      <c r="D33" s="48"/>
+      <c r="E33" s="45"/>
+      <c r="F33" s="46"/>
       <c r="G33" s="23"/>
       <c r="H33" s="10"/>
     </row>
     <row r="34" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="13"/>
       <c r="B34" s="2"/>
-      <c r="C34" s="62"/>
-      <c r="D34" s="63"/>
-      <c r="E34" s="60"/>
-      <c r="F34" s="61"/>
+      <c r="C34" s="47"/>
+      <c r="D34" s="48"/>
+      <c r="E34" s="45"/>
+      <c r="F34" s="46"/>
       <c r="G34" s="23"/>
       <c r="H34" s="10"/>
     </row>
     <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="13"/>
       <c r="B35" s="2"/>
-      <c r="C35" s="62"/>
-      <c r="D35" s="63"/>
-      <c r="E35" s="60"/>
-      <c r="F35" s="61"/>
+      <c r="C35" s="47"/>
+      <c r="D35" s="48"/>
+      <c r="E35" s="45"/>
+      <c r="F35" s="46"/>
       <c r="G35" s="23"/>
       <c r="H35" s="10"/>
     </row>
     <row r="36" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="13"/>
       <c r="B36" s="2"/>
-      <c r="C36" s="62"/>
-      <c r="D36" s="63"/>
-      <c r="E36" s="60"/>
-      <c r="F36" s="61"/>
+      <c r="C36" s="47"/>
+      <c r="D36" s="48"/>
+      <c r="E36" s="45"/>
+      <c r="F36" s="46"/>
       <c r="G36" s="23"/>
       <c r="H36" s="10"/>
     </row>
     <row r="37" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="13"/>
       <c r="B37" s="2"/>
-      <c r="C37" s="62"/>
-      <c r="D37" s="63"/>
-      <c r="E37" s="60"/>
-      <c r="F37" s="61"/>
+      <c r="C37" s="47"/>
+      <c r="D37" s="48"/>
+      <c r="E37" s="45"/>
+      <c r="F37" s="46"/>
       <c r="G37" s="23"/>
       <c r="H37" s="10"/>
     </row>
     <row r="38" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="13"/>
       <c r="B38" s="2"/>
-      <c r="C38" s="62"/>
-      <c r="D38" s="63"/>
-      <c r="E38" s="60"/>
-      <c r="F38" s="61"/>
+      <c r="C38" s="47"/>
+      <c r="D38" s="48"/>
+      <c r="E38" s="45"/>
+      <c r="F38" s="46"/>
       <c r="G38" s="23"/>
       <c r="H38" s="10"/>
     </row>
     <row r="39" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="13"/>
       <c r="B39" s="2"/>
-      <c r="C39" s="66"/>
-      <c r="D39" s="67"/>
-      <c r="E39" s="60"/>
-      <c r="F39" s="61"/>
+      <c r="C39" s="49"/>
+      <c r="D39" s="50"/>
+      <c r="E39" s="45"/>
+      <c r="F39" s="46"/>
       <c r="G39" s="23"/>
       <c r="H39" s="10"/>
     </row>
     <row r="40" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="13"/>
       <c r="B40" s="2"/>
-      <c r="C40" s="62"/>
-      <c r="D40" s="63"/>
-      <c r="E40" s="60"/>
-      <c r="F40" s="61"/>
+      <c r="C40" s="47"/>
+      <c r="D40" s="48"/>
+      <c r="E40" s="45"/>
+      <c r="F40" s="46"/>
       <c r="G40" s="23"/>
       <c r="H40" s="10"/>
     </row>
     <row r="41" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="13"/>
       <c r="B41" s="2"/>
-      <c r="C41" s="62"/>
-      <c r="D41" s="63"/>
-      <c r="E41" s="60"/>
-      <c r="F41" s="61"/>
+      <c r="C41" s="47"/>
+      <c r="D41" s="48"/>
+      <c r="E41" s="45"/>
+      <c r="F41" s="46"/>
       <c r="G41" s="23"/>
       <c r="H41" s="10"/>
     </row>
     <row r="42" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="13"/>
       <c r="B42" s="2"/>
-      <c r="C42" s="62"/>
-      <c r="D42" s="63"/>
-      <c r="E42" s="60"/>
-      <c r="F42" s="61"/>
+      <c r="C42" s="47"/>
+      <c r="D42" s="48"/>
+      <c r="E42" s="45"/>
+      <c r="F42" s="46"/>
       <c r="G42" s="23"/>
       <c r="H42" s="10"/>
     </row>
     <row r="43" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="13"/>
       <c r="B43" s="2"/>
-      <c r="C43" s="62"/>
-      <c r="D43" s="63"/>
-      <c r="E43" s="60"/>
-      <c r="F43" s="61"/>
+      <c r="C43" s="47"/>
+      <c r="D43" s="48"/>
+      <c r="E43" s="45"/>
+      <c r="F43" s="46"/>
       <c r="G43" s="23"/>
       <c r="H43" s="10"/>
     </row>
     <row r="44" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="13"/>
       <c r="B44" s="2"/>
-      <c r="C44" s="62"/>
-      <c r="D44" s="63"/>
-      <c r="E44" s="60"/>
-      <c r="F44" s="61"/>
+      <c r="C44" s="47"/>
+      <c r="D44" s="48"/>
+      <c r="E44" s="45"/>
+      <c r="F44" s="46"/>
       <c r="G44" s="23"/>
       <c r="H44" s="10"/>
     </row>
     <row r="45" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="13"/>
       <c r="B45" s="2"/>
-      <c r="C45" s="62"/>
-      <c r="D45" s="63"/>
-      <c r="E45" s="60"/>
-      <c r="F45" s="61"/>
+      <c r="C45" s="47"/>
+      <c r="D45" s="48"/>
+      <c r="E45" s="45"/>
+      <c r="F45" s="46"/>
       <c r="G45" s="23"/>
       <c r="H45" s="10"/>
     </row>
     <row r="46" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="13"/>
       <c r="B46" s="2"/>
-      <c r="C46" s="62"/>
-      <c r="D46" s="63"/>
-      <c r="E46" s="60"/>
-      <c r="F46" s="61"/>
+      <c r="C46" s="47"/>
+      <c r="D46" s="48"/>
+      <c r="E46" s="45"/>
+      <c r="F46" s="46"/>
       <c r="G46" s="23"/>
       <c r="H46" s="10"/>
     </row>
     <row r="47" spans="1:8" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A47" s="13"/>
       <c r="B47" s="2"/>
-      <c r="C47" s="62"/>
-      <c r="D47" s="63"/>
-      <c r="E47" s="60"/>
-      <c r="F47" s="61"/>
+      <c r="C47" s="47"/>
+      <c r="D47" s="48"/>
+      <c r="E47" s="45"/>
+      <c r="F47" s="46"/>
       <c r="G47" s="23"/>
     </row>
     <row r="48" spans="1:8" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="80" t="s">
+      <c r="A48" s="63" t="s">
         <v>14</v>
       </c>
-      <c r="B48" s="81"/>
-      <c r="C48" s="81"/>
-      <c r="D48" s="81"/>
-      <c r="E48" s="82"/>
-      <c r="F48" s="83"/>
-      <c r="G48" s="84"/>
+      <c r="B48" s="64"/>
+      <c r="C48" s="64"/>
+      <c r="D48" s="64"/>
+      <c r="E48" s="65"/>
+      <c r="F48" s="66"/>
+      <c r="G48" s="67"/>
     </row>
     <row r="49" spans="1:7" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="50" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="85" t="s">
+      <c r="A50" s="73" t="s">
         <v>20</v>
       </c>
-      <c r="B50" s="86"/>
-      <c r="C50" s="87" t="s">
+      <c r="B50" s="74"/>
+      <c r="C50" s="70" t="s">
         <v>26</v>
       </c>
-      <c r="D50" s="88"/>
-      <c r="E50" s="88"/>
-      <c r="F50" s="88"/>
-      <c r="G50" s="89"/>
+      <c r="D50" s="71"/>
+      <c r="E50" s="71"/>
+      <c r="F50" s="71"/>
+      <c r="G50" s="72"/>
     </row>
     <row r="51" spans="1:7" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="75" t="s">
+      <c r="A51" s="55" t="s">
         <v>15</v>
       </c>
-      <c r="B51" s="76"/>
-      <c r="C51" s="90"/>
-      <c r="D51" s="91"/>
-      <c r="E51" s="92" t="s">
+      <c r="B51" s="56"/>
+      <c r="C51" s="68"/>
+      <c r="D51" s="69"/>
+      <c r="E51" s="57" t="s">
         <v>5</v>
       </c>
-      <c r="F51" s="93"/>
-      <c r="G51" s="94"/>
+      <c r="F51" s="58"/>
+      <c r="G51" s="59"/>
     </row>
     <row r="52" spans="1:7" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A52" s="75" t="s">
+      <c r="A52" s="55" t="s">
         <v>27</v>
       </c>
-      <c r="B52" s="76"/>
+      <c r="B52" s="56"/>
       <c r="C52" s="32" t="s">
         <v>29</v>
       </c>
       <c r="D52" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="E52" s="68" t="s">
+      <c r="E52" s="60" t="s">
         <v>30</v>
       </c>
-      <c r="F52" s="69"/>
-      <c r="G52" s="70"/>
+      <c r="F52" s="61"/>
+      <c r="G52" s="62"/>
     </row>
     <row r="53" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="71" t="s">
+      <c r="A53" s="51" t="s">
         <v>16</v>
       </c>
-      <c r="B53" s="72"/>
+      <c r="B53" s="52"/>
       <c r="C53" s="33" t="s">
         <v>33</v>
       </c>
       <c r="D53" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="E53" s="73" t="s">
+      <c r="E53" s="53" t="s">
         <v>32</v>
       </c>
-      <c r="F53" s="73"/>
-      <c r="G53" s="74"/>
+      <c r="F53" s="53"/>
+      <c r="G53" s="54"/>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.2">
       <c r="G54" s="3" t="s">
@@ -3043,6 +3046,87 @@
     </row>
   </sheetData>
   <mergeCells count="97">
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="A10:G10"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="E28:F28"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="E30:F30"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="E32:F32"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="E33:F33"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="E34:F34"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="E35:F35"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="E36:F36"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="E37:F37"/>
+    <mergeCell ref="C38:D38"/>
+    <mergeCell ref="E38:F38"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="E39:F39"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="E40:F40"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="E41:F41"/>
+    <mergeCell ref="C47:D47"/>
+    <mergeCell ref="E47:F47"/>
+    <mergeCell ref="C42:D42"/>
+    <mergeCell ref="E42:F42"/>
+    <mergeCell ref="C43:D43"/>
+    <mergeCell ref="E43:F43"/>
+    <mergeCell ref="C44:D44"/>
+    <mergeCell ref="E44:F44"/>
     <mergeCell ref="E52:G52"/>
     <mergeCell ref="A53:B53"/>
     <mergeCell ref="E53:G53"/>
@@ -3059,87 +3143,6 @@
     <mergeCell ref="E45:F45"/>
     <mergeCell ref="C46:D46"/>
     <mergeCell ref="E46:F46"/>
-    <mergeCell ref="C47:D47"/>
-    <mergeCell ref="E47:F47"/>
-    <mergeCell ref="C42:D42"/>
-    <mergeCell ref="E42:F42"/>
-    <mergeCell ref="C43:D43"/>
-    <mergeCell ref="E43:F43"/>
-    <mergeCell ref="C44:D44"/>
-    <mergeCell ref="E44:F44"/>
-    <mergeCell ref="C39:D39"/>
-    <mergeCell ref="E39:F39"/>
-    <mergeCell ref="C40:D40"/>
-    <mergeCell ref="E40:F40"/>
-    <mergeCell ref="C41:D41"/>
-    <mergeCell ref="E41:F41"/>
-    <mergeCell ref="C36:D36"/>
-    <mergeCell ref="E36:F36"/>
-    <mergeCell ref="C37:D37"/>
-    <mergeCell ref="E37:F37"/>
-    <mergeCell ref="C38:D38"/>
-    <mergeCell ref="E38:F38"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="E33:F33"/>
-    <mergeCell ref="C34:D34"/>
-    <mergeCell ref="E34:F34"/>
-    <mergeCell ref="C35:D35"/>
-    <mergeCell ref="E35:F35"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="E30:F30"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="E31:F31"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="E32:F32"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="E27:F27"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="E28:F28"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="E29:F29"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="E25:F25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="E26:F26"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="E21:F21"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="E17:F17"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="E12:F12"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="A10:G10"/>
   </mergeCells>
   <pageMargins left="0.51181102362204722" right="0.19685039370078741" top="0.31496062992125984" bottom="0" header="0.51181102362204722" footer="0.51181102362204722"/>
   <pageSetup paperSize="9" scale="83" fitToHeight="0" orientation="portrait" copies="3" r:id="rId1"/>

</xml_diff>

<commit_message>
chore: added tup logo in PR PDF
</commit_message>
<xml_diff>
--- a/procurement_documents/PR Template.xlsx
+++ b/procurement_documents/PR Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emman\itrac\procurement_documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C47CE686-06A3-44B9-BE8E-5A3106F2F0D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F9F5D70-2D85-48C1-AD05-C240A549A451}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="739" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -848,7 +848,7 @@
     </xf>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="105">
+  <cellXfs count="115">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -950,12 +950,155 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="36" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="22" fontId="21" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="22" fontId="21" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="39" fontId="25" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="39" fontId="25" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -974,169 +1117,54 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="39" fontId="25" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="39" fontId="25" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="22" fontId="21" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="22" fontId="21" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="36" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="22" fontId="21" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="22" fontId="21" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="22" fontId="21" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="22" fontId="21" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="10">
@@ -1251,7 +1279,7 @@
       <xdr:col>4</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>12</xdr:row>
-      <xdr:rowOff>182705</xdr:rowOff>
+      <xdr:rowOff>182704</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1768,72 +1796,72 @@
     <col min="3" max="3" width="33.85546875" style="3" customWidth="1"/>
     <col min="4" max="4" width="33.7109375" style="3" customWidth="1"/>
     <col min="5" max="5" width="17.28515625" style="3" customWidth="1"/>
-    <col min="6" max="6" width="1.85546875" style="3" customWidth="1"/>
+    <col min="6" max="6" width="7" style="3" customWidth="1"/>
     <col min="7" max="7" width="22.85546875" style="3" customWidth="1"/>
     <col min="8" max="8" width="8.140625" style="3" customWidth="1"/>
     <col min="9" max="16384" width="8.85546875" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="104" t="s">
         <v>8</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="111"/>
       <c r="F1" s="19"/>
       <c r="G1" s="20"/>
     </row>
     <row r="2" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="14"/>
-      <c r="B2" s="40" t="s">
+      <c r="A2" s="105"/>
+      <c r="B2" s="91" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="40"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="44" t="s">
+      <c r="C2" s="91"/>
+      <c r="D2" s="106"/>
+      <c r="E2" s="95" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="40"/>
-      <c r="G2" s="41"/>
+      <c r="F2" s="106"/>
+      <c r="G2" s="92"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="15"/>
-      <c r="B3" s="42" t="s">
+      <c r="A3" s="105"/>
+      <c r="B3" s="93" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="42"/>
-      <c r="D3" s="43"/>
-      <c r="E3" s="37" t="s">
+      <c r="C3" s="93"/>
+      <c r="D3" s="108"/>
+      <c r="E3" s="89" t="s">
         <v>28</v>
       </c>
-      <c r="F3" s="38"/>
-      <c r="G3" s="39"/>
-    </row>
-    <row r="4" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="14"/>
-      <c r="B4" s="40"/>
-      <c r="C4" s="40"/>
-      <c r="D4" s="41"/>
-      <c r="E4" s="34"/>
-      <c r="F4" s="34"/>
-      <c r="G4" s="35"/>
+      <c r="F3" s="107"/>
+      <c r="G3" s="90"/>
+    </row>
+    <row r="4" spans="1:14" ht="10.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="105"/>
+      <c r="B4" s="91" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="91"/>
+      <c r="D4" s="106"/>
+      <c r="E4" s="112" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="110"/>
+      <c r="G4" s="113"/>
     </row>
     <row r="5" spans="1:14" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="30"/>
-      <c r="B5" s="79" t="s">
-        <v>19</v>
-      </c>
-      <c r="C5" s="79"/>
-      <c r="D5" s="80"/>
-      <c r="E5" s="81" t="s">
-        <v>13</v>
-      </c>
-      <c r="F5" s="81"/>
-      <c r="G5" s="82"/>
-    </row>
-    <row r="6" spans="1:14" ht="4.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="109"/>
+      <c r="B5" s="42"/>
+      <c r="C5" s="42"/>
+      <c r="D5" s="42"/>
+      <c r="E5" s="114"/>
+      <c r="F5" s="44"/>
+      <c r="G5" s="45"/>
+    </row>
+    <row r="6" spans="1:14" ht="10.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="16"/>
       <c r="B6" s="17"/>
       <c r="C6" s="17"/>
@@ -1842,7 +1870,7 @@
       <c r="F6" s="17"/>
       <c r="G6" s="17"/>
     </row>
-    <row r="7" spans="1:14" ht="21.75" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="16"/>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
@@ -1855,37 +1883,37 @@
       <c r="A8" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B8" s="83"/>
-      <c r="C8" s="84"/>
-      <c r="D8" s="85"/>
+      <c r="B8" s="48"/>
+      <c r="C8" s="49"/>
+      <c r="D8" s="50"/>
       <c r="E8" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="F8" s="86"/>
-      <c r="G8" s="87"/>
+      <c r="F8" s="51"/>
+      <c r="G8" s="52"/>
       <c r="H8" s="4"/>
     </row>
     <row r="9" spans="1:14" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="88"/>
-      <c r="C9" s="89"/>
-      <c r="D9" s="90"/>
+      <c r="B9" s="53"/>
+      <c r="C9" s="54"/>
+      <c r="D9" s="55"/>
       <c r="E9" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="100"/>
-      <c r="G9" s="101"/>
+      <c r="F9" s="56"/>
+      <c r="G9" s="57"/>
     </row>
     <row r="10" spans="1:14" ht="5.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="93"/>
-      <c r="B10" s="93"/>
-      <c r="C10" s="93"/>
-      <c r="D10" s="93"/>
-      <c r="E10" s="93"/>
-      <c r="F10" s="93"/>
-      <c r="G10" s="93"/>
+      <c r="A10" s="58"/>
+      <c r="B10" s="58"/>
+      <c r="C10" s="58"/>
+      <c r="D10" s="58"/>
+      <c r="E10" s="58"/>
+      <c r="F10" s="58"/>
+      <c r="G10" s="58"/>
     </row>
     <row r="11" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
@@ -1894,14 +1922,14 @@
       <c r="B11" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="94" t="s">
+      <c r="C11" s="59" t="s">
         <v>7</v>
       </c>
-      <c r="D11" s="95"/>
-      <c r="E11" s="94" t="s">
+      <c r="D11" s="60"/>
+      <c r="E11" s="59" t="s">
         <v>3</v>
       </c>
-      <c r="F11" s="95"/>
+      <c r="F11" s="60"/>
       <c r="G11" s="22" t="s">
         <v>4</v>
       </c>
@@ -1909,10 +1937,10 @@
     <row r="12" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="12"/>
       <c r="B12" s="1"/>
-      <c r="C12" s="77"/>
-      <c r="D12" s="78"/>
-      <c r="E12" s="45"/>
-      <c r="F12" s="46"/>
+      <c r="C12" s="46"/>
+      <c r="D12" s="47"/>
+      <c r="E12" s="38"/>
+      <c r="F12" s="39"/>
       <c r="G12" s="23"/>
       <c r="H12" s="11"/>
       <c r="I12" s="5"/>
@@ -1925,10 +1953,10 @@
     <row r="13" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="12"/>
       <c r="B13" s="1"/>
-      <c r="C13" s="77"/>
-      <c r="D13" s="78"/>
-      <c r="E13" s="45"/>
-      <c r="F13" s="46"/>
+      <c r="C13" s="46"/>
+      <c r="D13" s="47"/>
+      <c r="E13" s="38"/>
+      <c r="F13" s="39"/>
       <c r="G13" s="23"/>
       <c r="H13" s="11"/>
       <c r="I13" s="8"/>
@@ -1939,451 +1967,450 @@
     <row r="14" spans="1:14" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="13"/>
       <c r="B14" s="1"/>
-      <c r="C14" s="77"/>
-      <c r="D14" s="78"/>
-      <c r="E14" s="45"/>
-      <c r="F14" s="46"/>
+      <c r="C14" s="46"/>
+      <c r="D14" s="47"/>
+      <c r="E14" s="38"/>
+      <c r="F14" s="39"/>
       <c r="G14" s="23"/>
       <c r="H14" s="11"/>
     </row>
     <row r="15" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="13"/>
       <c r="B15" s="1"/>
-      <c r="C15" s="77"/>
-      <c r="D15" s="78"/>
-      <c r="E15" s="45"/>
-      <c r="F15" s="46"/>
+      <c r="C15" s="46"/>
+      <c r="D15" s="47"/>
+      <c r="E15" s="38"/>
+      <c r="F15" s="39"/>
       <c r="G15" s="23"/>
       <c r="H15" s="11"/>
     </row>
     <row r="16" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="13"/>
-      <c r="B16" s="99"/>
-      <c r="C16" s="77"/>
-      <c r="D16" s="78"/>
-      <c r="E16" s="45"/>
-      <c r="F16" s="46"/>
+      <c r="B16" s="37"/>
+      <c r="C16" s="46"/>
+      <c r="D16" s="47"/>
+      <c r="E16" s="38"/>
+      <c r="F16" s="39"/>
       <c r="G16" s="23"/>
       <c r="H16" s="11"/>
     </row>
     <row r="17" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="13"/>
-      <c r="B17" s="99"/>
-      <c r="C17" s="77"/>
-      <c r="D17" s="78"/>
-      <c r="E17" s="45"/>
-      <c r="F17" s="46"/>
+      <c r="B17" s="37"/>
+      <c r="C17" s="46"/>
+      <c r="D17" s="47"/>
+      <c r="E17" s="38"/>
+      <c r="F17" s="39"/>
       <c r="G17" s="23"/>
       <c r="H17" s="11"/>
     </row>
     <row r="18" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="13"/>
-      <c r="B18" s="99"/>
-      <c r="C18" s="47"/>
-      <c r="D18" s="48"/>
-      <c r="E18" s="45"/>
-      <c r="F18" s="46"/>
+      <c r="B18" s="37"/>
+      <c r="C18" s="40"/>
+      <c r="D18" s="41"/>
+      <c r="E18" s="38"/>
+      <c r="F18" s="39"/>
       <c r="G18" s="23"/>
       <c r="H18" s="11"/>
     </row>
     <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="13"/>
-      <c r="B19" s="99"/>
-      <c r="C19" s="47"/>
-      <c r="D19" s="48"/>
-      <c r="E19" s="45"/>
-      <c r="F19" s="46"/>
+      <c r="B19" s="37"/>
+      <c r="C19" s="40"/>
+      <c r="D19" s="41"/>
+      <c r="E19" s="38"/>
+      <c r="F19" s="39"/>
       <c r="G19" s="23"/>
       <c r="H19" s="10"/>
     </row>
     <row r="20" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="13"/>
-      <c r="B20" s="99"/>
-      <c r="C20" s="47"/>
-      <c r="D20" s="48"/>
-      <c r="E20" s="45"/>
-      <c r="F20" s="46"/>
+      <c r="B20" s="37"/>
+      <c r="C20" s="40"/>
+      <c r="D20" s="41"/>
+      <c r="E20" s="38"/>
+      <c r="F20" s="39"/>
       <c r="G20" s="23"/>
       <c r="H20" s="10"/>
     </row>
     <row r="21" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="13"/>
-      <c r="B21" s="99"/>
-      <c r="C21" s="47"/>
-      <c r="D21" s="48"/>
-      <c r="E21" s="45"/>
-      <c r="F21" s="46"/>
+      <c r="B21" s="37"/>
+      <c r="C21" s="40"/>
+      <c r="D21" s="41"/>
+      <c r="E21" s="38"/>
+      <c r="F21" s="39"/>
       <c r="G21" s="23"/>
       <c r="H21" s="10"/>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="13"/>
-      <c r="B22" s="99"/>
-      <c r="C22" s="47"/>
-      <c r="D22" s="48"/>
-      <c r="E22" s="45"/>
-      <c r="F22" s="46"/>
+      <c r="B22" s="37"/>
+      <c r="C22" s="40"/>
+      <c r="D22" s="41"/>
+      <c r="E22" s="38"/>
+      <c r="F22" s="39"/>
       <c r="G22" s="23"/>
       <c r="H22" s="10"/>
     </row>
     <row r="23" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="13"/>
-      <c r="B23" s="99"/>
-      <c r="C23" s="47"/>
-      <c r="D23" s="48"/>
-      <c r="E23" s="45"/>
-      <c r="F23" s="46"/>
+      <c r="B23" s="37"/>
+      <c r="C23" s="40"/>
+      <c r="D23" s="41"/>
+      <c r="E23" s="38"/>
+      <c r="F23" s="39"/>
       <c r="G23" s="23"/>
       <c r="H23" s="10"/>
     </row>
     <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="13"/>
-      <c r="B24" s="99"/>
-      <c r="C24" s="47"/>
-      <c r="D24" s="48"/>
-      <c r="E24" s="45"/>
-      <c r="F24" s="46"/>
+      <c r="B24" s="37"/>
+      <c r="C24" s="40"/>
+      <c r="D24" s="41"/>
+      <c r="E24" s="38"/>
+      <c r="F24" s="39"/>
       <c r="G24" s="23"/>
       <c r="H24" s="10"/>
     </row>
     <row r="25" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="13"/>
-      <c r="B25" s="99"/>
-      <c r="C25" s="47"/>
-      <c r="D25" s="48"/>
-      <c r="E25" s="45"/>
-      <c r="F25" s="46"/>
+      <c r="B25" s="37"/>
+      <c r="C25" s="40"/>
+      <c r="D25" s="41"/>
+      <c r="E25" s="38"/>
+      <c r="F25" s="39"/>
       <c r="G25" s="23"/>
       <c r="H25" s="10"/>
     </row>
     <row r="26" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="13"/>
-      <c r="B26" s="99"/>
-      <c r="C26" s="47"/>
-      <c r="D26" s="48"/>
-      <c r="E26" s="45"/>
-      <c r="F26" s="46"/>
+      <c r="B26" s="37"/>
+      <c r="C26" s="40"/>
+      <c r="D26" s="41"/>
+      <c r="E26" s="38"/>
+      <c r="F26" s="39"/>
       <c r="G26" s="23"/>
       <c r="H26" s="10"/>
     </row>
     <row r="27" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="13"/>
-      <c r="B27" s="99"/>
-      <c r="C27" s="47"/>
-      <c r="D27" s="48"/>
-      <c r="E27" s="45"/>
-      <c r="F27" s="46"/>
+      <c r="B27" s="37"/>
+      <c r="C27" s="40"/>
+      <c r="D27" s="41"/>
+      <c r="E27" s="38"/>
+      <c r="F27" s="39"/>
       <c r="G27" s="23"/>
       <c r="H27" s="10"/>
     </row>
     <row r="28" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="13"/>
-      <c r="B28" s="99"/>
-      <c r="C28" s="75"/>
-      <c r="D28" s="76"/>
-      <c r="E28" s="45"/>
-      <c r="F28" s="46"/>
+      <c r="B28" s="37"/>
+      <c r="C28" s="61"/>
+      <c r="D28" s="62"/>
+      <c r="E28" s="38"/>
+      <c r="F28" s="39"/>
       <c r="G28" s="23"/>
       <c r="H28" s="10"/>
     </row>
     <row r="29" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="13"/>
-      <c r="B29" s="99"/>
-      <c r="C29" s="75"/>
-      <c r="D29" s="76"/>
-      <c r="E29" s="45"/>
-      <c r="F29" s="46"/>
+      <c r="B29" s="37"/>
+      <c r="C29" s="61"/>
+      <c r="D29" s="62"/>
+      <c r="E29" s="38"/>
+      <c r="F29" s="39"/>
       <c r="G29" s="23"/>
       <c r="H29" s="10"/>
     </row>
     <row r="30" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="13"/>
-      <c r="B30" s="99"/>
-      <c r="C30" s="75"/>
-      <c r="D30" s="76"/>
-      <c r="E30" s="45"/>
-      <c r="F30" s="46"/>
+      <c r="B30" s="37"/>
+      <c r="C30" s="61"/>
+      <c r="D30" s="62"/>
+      <c r="E30" s="38"/>
+      <c r="F30" s="39"/>
       <c r="G30" s="23"/>
       <c r="H30" s="10"/>
     </row>
     <row r="31" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="13"/>
-      <c r="B31" s="99"/>
-      <c r="C31" s="47"/>
-      <c r="D31" s="48"/>
-      <c r="E31" s="45"/>
-      <c r="F31" s="46"/>
+      <c r="B31" s="37"/>
+      <c r="C31" s="40"/>
+      <c r="D31" s="41"/>
+      <c r="E31" s="38"/>
+      <c r="F31" s="39"/>
       <c r="G31" s="23"/>
       <c r="H31" s="10"/>
     </row>
     <row r="32" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="13"/>
-      <c r="B32" s="99"/>
-      <c r="C32" s="47"/>
-      <c r="D32" s="48"/>
-      <c r="E32" s="45"/>
-      <c r="F32" s="46"/>
+      <c r="B32" s="37"/>
+      <c r="C32" s="40"/>
+      <c r="D32" s="41"/>
+      <c r="E32" s="38"/>
+      <c r="F32" s="39"/>
       <c r="G32" s="23"/>
       <c r="H32" s="10"/>
     </row>
     <row r="33" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="13"/>
-      <c r="B33" s="99"/>
-      <c r="C33" s="47"/>
-      <c r="D33" s="48"/>
-      <c r="E33" s="45"/>
-      <c r="F33" s="46"/>
+      <c r="B33" s="37"/>
+      <c r="C33" s="40"/>
+      <c r="D33" s="41"/>
+      <c r="E33" s="38"/>
+      <c r="F33" s="39"/>
       <c r="G33" s="23"/>
       <c r="H33" s="10"/>
     </row>
     <row r="34" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="13"/>
-      <c r="B34" s="99"/>
-      <c r="C34" s="47"/>
-      <c r="D34" s="48"/>
-      <c r="E34" s="45"/>
-      <c r="F34" s="46"/>
+      <c r="B34" s="37"/>
+      <c r="C34" s="40"/>
+      <c r="D34" s="41"/>
+      <c r="E34" s="38"/>
+      <c r="F34" s="39"/>
       <c r="G34" s="23"/>
       <c r="H34" s="10"/>
     </row>
     <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="13"/>
-      <c r="B35" s="99"/>
-      <c r="C35" s="47"/>
-      <c r="D35" s="48"/>
-      <c r="E35" s="45"/>
-      <c r="F35" s="46"/>
+      <c r="B35" s="37"/>
+      <c r="C35" s="40"/>
+      <c r="D35" s="41"/>
+      <c r="E35" s="38"/>
+      <c r="F35" s="39"/>
       <c r="G35" s="23"/>
       <c r="H35" s="10"/>
     </row>
     <row r="36" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="13"/>
-      <c r="B36" s="99"/>
-      <c r="C36" s="47"/>
-      <c r="D36" s="48"/>
-      <c r="E36" s="45"/>
-      <c r="F36" s="46"/>
+      <c r="B36" s="37"/>
+      <c r="C36" s="40"/>
+      <c r="D36" s="41"/>
+      <c r="E36" s="38"/>
+      <c r="F36" s="39"/>
       <c r="G36" s="23"/>
       <c r="H36" s="10"/>
     </row>
     <row r="37" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="13"/>
-      <c r="B37" s="99"/>
-      <c r="C37" s="47"/>
-      <c r="D37" s="48"/>
-      <c r="E37" s="45"/>
-      <c r="F37" s="46"/>
+      <c r="B37" s="37"/>
+      <c r="C37" s="40"/>
+      <c r="D37" s="41"/>
+      <c r="E37" s="38"/>
+      <c r="F37" s="39"/>
       <c r="G37" s="23"/>
       <c r="H37" s="10"/>
     </row>
     <row r="38" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="13"/>
-      <c r="B38" s="99"/>
-      <c r="C38" s="47"/>
-      <c r="D38" s="48"/>
-      <c r="E38" s="45"/>
-      <c r="F38" s="46"/>
+      <c r="B38" s="37"/>
+      <c r="C38" s="40"/>
+      <c r="D38" s="41"/>
+      <c r="E38" s="38"/>
+      <c r="F38" s="39"/>
       <c r="G38" s="23"/>
       <c r="H38" s="10"/>
     </row>
     <row r="39" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="13"/>
-      <c r="B39" s="99"/>
-      <c r="C39" s="49"/>
-      <c r="D39" s="50"/>
-      <c r="E39" s="45"/>
-      <c r="F39" s="46"/>
+      <c r="B39" s="37"/>
+      <c r="C39" s="87"/>
+      <c r="D39" s="88"/>
+      <c r="E39" s="38"/>
+      <c r="F39" s="39"/>
       <c r="G39" s="23"/>
       <c r="H39" s="10"/>
     </row>
     <row r="40" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="13"/>
-      <c r="B40" s="99"/>
-      <c r="C40" s="47"/>
-      <c r="D40" s="48"/>
-      <c r="E40" s="45"/>
-      <c r="F40" s="46"/>
+      <c r="B40" s="37"/>
+      <c r="C40" s="40"/>
+      <c r="D40" s="41"/>
+      <c r="E40" s="38"/>
+      <c r="F40" s="39"/>
       <c r="G40" s="23"/>
       <c r="H40" s="10"/>
     </row>
     <row r="41" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="13"/>
-      <c r="B41" s="99"/>
-      <c r="C41" s="47"/>
-      <c r="D41" s="48"/>
-      <c r="E41" s="45"/>
-      <c r="F41" s="46"/>
+      <c r="B41" s="37"/>
+      <c r="C41" s="40"/>
+      <c r="D41" s="41"/>
+      <c r="E41" s="38"/>
+      <c r="F41" s="39"/>
       <c r="G41" s="23"/>
       <c r="H41" s="10"/>
     </row>
     <row r="42" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="13"/>
-      <c r="B42" s="99"/>
-      <c r="C42" s="47"/>
-      <c r="D42" s="48"/>
-      <c r="E42" s="45"/>
-      <c r="F42" s="46"/>
+      <c r="B42" s="37"/>
+      <c r="C42" s="40"/>
+      <c r="D42" s="41"/>
+      <c r="E42" s="38"/>
+      <c r="F42" s="39"/>
       <c r="G42" s="23"/>
       <c r="H42" s="10"/>
     </row>
     <row r="43" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="13"/>
-      <c r="B43" s="99"/>
-      <c r="C43" s="47"/>
-      <c r="D43" s="48"/>
-      <c r="E43" s="45"/>
-      <c r="F43" s="46"/>
+      <c r="B43" s="37"/>
+      <c r="C43" s="40"/>
+      <c r="D43" s="41"/>
+      <c r="E43" s="38"/>
+      <c r="F43" s="39"/>
       <c r="G43" s="23"/>
       <c r="H43" s="10"/>
     </row>
     <row r="44" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="13"/>
-      <c r="B44" s="99"/>
-      <c r="C44" s="47"/>
-      <c r="D44" s="48"/>
-      <c r="E44" s="45"/>
-      <c r="F44" s="46"/>
+      <c r="B44" s="37"/>
+      <c r="C44" s="40"/>
+      <c r="D44" s="41"/>
+      <c r="E44" s="38"/>
+      <c r="F44" s="39"/>
       <c r="G44" s="23"/>
       <c r="H44" s="10"/>
     </row>
     <row r="45" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="13"/>
-      <c r="B45" s="99"/>
-      <c r="C45" s="47"/>
-      <c r="D45" s="48"/>
-      <c r="E45" s="45"/>
-      <c r="F45" s="46"/>
+      <c r="B45" s="37"/>
+      <c r="C45" s="40"/>
+      <c r="D45" s="41"/>
+      <c r="E45" s="38"/>
+      <c r="F45" s="39"/>
       <c r="G45" s="23"/>
       <c r="H45" s="10"/>
     </row>
     <row r="46" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="13"/>
-      <c r="B46" s="99"/>
-      <c r="C46" s="47"/>
-      <c r="D46" s="48"/>
-      <c r="E46" s="45"/>
-      <c r="F46" s="46"/>
+      <c r="B46" s="37"/>
+      <c r="C46" s="40"/>
+      <c r="D46" s="41"/>
+      <c r="E46" s="38"/>
+      <c r="F46" s="39"/>
       <c r="G46" s="23"/>
       <c r="H46" s="10"/>
     </row>
     <row r="47" spans="1:8" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A47" s="13"/>
-      <c r="B47" s="99"/>
-      <c r="C47" s="47"/>
-      <c r="D47" s="48"/>
-      <c r="E47" s="45"/>
-      <c r="F47" s="46"/>
+      <c r="B47" s="37"/>
+      <c r="C47" s="40"/>
+      <c r="D47" s="41"/>
+      <c r="E47" s="38"/>
+      <c r="F47" s="39"/>
       <c r="G47" s="23"/>
     </row>
     <row r="48" spans="1:8" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="63" t="s">
+      <c r="A48" s="75" t="s">
         <v>14</v>
       </c>
-      <c r="B48" s="64"/>
-      <c r="C48" s="64"/>
-      <c r="D48" s="64"/>
-      <c r="E48" s="65"/>
-      <c r="F48" s="66"/>
-      <c r="G48" s="67"/>
+      <c r="B48" s="76"/>
+      <c r="C48" s="76"/>
+      <c r="D48" s="76"/>
+      <c r="E48" s="77"/>
+      <c r="F48" s="78"/>
+      <c r="G48" s="79"/>
     </row>
     <row r="49" spans="1:7" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="50" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="73" t="s">
+      <c r="A50" s="85" t="s">
         <v>20</v>
       </c>
-      <c r="B50" s="74"/>
-      <c r="C50" s="102"/>
-      <c r="D50" s="103"/>
-      <c r="E50" s="103"/>
-      <c r="F50" s="103"/>
-      <c r="G50" s="104"/>
+      <c r="B50" s="86"/>
+      <c r="C50" s="82"/>
+      <c r="D50" s="83"/>
+      <c r="E50" s="83"/>
+      <c r="F50" s="83"/>
+      <c r="G50" s="84"/>
     </row>
     <row r="51" spans="1:7" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="55" t="s">
+      <c r="A51" s="67" t="s">
         <v>15</v>
       </c>
-      <c r="B51" s="56"/>
-      <c r="C51" s="68"/>
-      <c r="D51" s="69"/>
-      <c r="E51" s="57" t="s">
+      <c r="B51" s="68"/>
+      <c r="C51" s="80"/>
+      <c r="D51" s="81"/>
+      <c r="E51" s="69" t="s">
         <v>5</v>
       </c>
-      <c r="F51" s="58"/>
-      <c r="G51" s="59"/>
+      <c r="F51" s="70"/>
+      <c r="G51" s="71"/>
     </row>
     <row r="52" spans="1:7" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A52" s="55" t="s">
+      <c r="A52" s="67" t="s">
         <v>27</v>
       </c>
-      <c r="B52" s="56"/>
+      <c r="B52" s="68"/>
       <c r="C52" s="32"/>
       <c r="D52" s="31"/>
-      <c r="E52" s="60" t="s">
+      <c r="E52" s="72" t="s">
         <v>18</v>
       </c>
-      <c r="F52" s="61"/>
-      <c r="G52" s="62"/>
+      <c r="F52" s="73"/>
+      <c r="G52" s="74"/>
     </row>
     <row r="53" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="51" t="s">
+      <c r="A53" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="B53" s="52"/>
+      <c r="B53" s="64"/>
       <c r="C53" s="33"/>
       <c r="D53" s="25"/>
-      <c r="E53" s="53" t="s">
+      <c r="E53" s="65" t="s">
         <v>6</v>
       </c>
-      <c r="F53" s="53"/>
-      <c r="G53" s="54"/>
+      <c r="F53" s="65"/>
+      <c r="G53" s="66"/>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.2">
       <c r="G54" s="36"/>
     </row>
   </sheetData>
-  <mergeCells count="97">
-    <mergeCell ref="E43:F43"/>
-    <mergeCell ref="C45:D45"/>
-    <mergeCell ref="E45:F45"/>
-    <mergeCell ref="C46:D46"/>
-    <mergeCell ref="E46:F46"/>
-    <mergeCell ref="C44:D44"/>
-    <mergeCell ref="E44:F44"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="E12:F12"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="A10:G10"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="E17:F17"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="E21:F21"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="E24:F24"/>
+  <mergeCells count="99">
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="A1:A5"/>
+    <mergeCell ref="E4:G4"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="E3:G3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="E40:F40"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="E41:F41"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="E37:F37"/>
+    <mergeCell ref="A48:E48"/>
+    <mergeCell ref="F48:G48"/>
+    <mergeCell ref="C51:D51"/>
+    <mergeCell ref="C50:G50"/>
+    <mergeCell ref="A50:B50"/>
+    <mergeCell ref="A53:B53"/>
+    <mergeCell ref="E53:G53"/>
+    <mergeCell ref="A51:B51"/>
+    <mergeCell ref="E51:G51"/>
+    <mergeCell ref="E52:G52"/>
+    <mergeCell ref="A52:B52"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="C47:D47"/>
+    <mergeCell ref="E47:F47"/>
+    <mergeCell ref="C38:D38"/>
+    <mergeCell ref="E38:F38"/>
+    <mergeCell ref="C43:D43"/>
+    <mergeCell ref="E36:F36"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="C42:D42"/>
+    <mergeCell ref="E42:F42"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="E39:F39"/>
+    <mergeCell ref="C40:D40"/>
     <mergeCell ref="E35:F35"/>
     <mergeCell ref="C25:D25"/>
     <mergeCell ref="E25:F25"/>
@@ -2400,45 +2427,48 @@
     <mergeCell ref="E28:F28"/>
     <mergeCell ref="C30:D30"/>
     <mergeCell ref="E30:F30"/>
-    <mergeCell ref="E29:F29"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="C47:D47"/>
-    <mergeCell ref="E47:F47"/>
-    <mergeCell ref="C38:D38"/>
-    <mergeCell ref="E38:F38"/>
-    <mergeCell ref="A53:B53"/>
-    <mergeCell ref="E53:G53"/>
-    <mergeCell ref="A51:B51"/>
-    <mergeCell ref="E51:G51"/>
-    <mergeCell ref="E52:G52"/>
-    <mergeCell ref="A52:B52"/>
-    <mergeCell ref="A48:E48"/>
-    <mergeCell ref="F48:G48"/>
-    <mergeCell ref="C51:D51"/>
-    <mergeCell ref="C50:G50"/>
-    <mergeCell ref="A50:B50"/>
-    <mergeCell ref="C43:D43"/>
-    <mergeCell ref="E36:F36"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="C34:D34"/>
-    <mergeCell ref="C42:D42"/>
-    <mergeCell ref="E42:F42"/>
-    <mergeCell ref="C39:D39"/>
-    <mergeCell ref="E39:F39"/>
-    <mergeCell ref="C40:D40"/>
-    <mergeCell ref="E40:F40"/>
-    <mergeCell ref="C41:D41"/>
-    <mergeCell ref="E41:F41"/>
-    <mergeCell ref="C37:D37"/>
-    <mergeCell ref="E37:F37"/>
-    <mergeCell ref="C35:D35"/>
-    <mergeCell ref="C36:D36"/>
-    <mergeCell ref="E3:G3"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="A10:G10"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="E43:F43"/>
+    <mergeCell ref="C45:D45"/>
+    <mergeCell ref="E45:F45"/>
+    <mergeCell ref="C46:D46"/>
+    <mergeCell ref="E46:F46"/>
+    <mergeCell ref="C44:D44"/>
+    <mergeCell ref="E44:F44"/>
   </mergeCells>
   <pageMargins left="0.51181102362204722" right="0.19685039370078741" top="0.31496062992125984" bottom="0" header="0.51181102362204722" footer="0.51181102362204722"/>
   <pageSetup paperSize="9" scale="83" fitToHeight="0" orientation="portrait" copies="3" r:id="rId1"/>
@@ -2478,51 +2508,51 @@
     </row>
     <row r="2" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="14"/>
-      <c r="B2" s="40" t="s">
+      <c r="B2" s="91" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="40"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="44" t="s">
+      <c r="C2" s="91"/>
+      <c r="D2" s="92"/>
+      <c r="E2" s="95" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="40"/>
-      <c r="G2" s="41"/>
+      <c r="F2" s="91"/>
+      <c r="G2" s="92"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="15"/>
-      <c r="B3" s="42" t="s">
+      <c r="B3" s="93" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="42"/>
-      <c r="D3" s="43"/>
-      <c r="E3" s="96" t="s">
+      <c r="C3" s="93"/>
+      <c r="D3" s="94"/>
+      <c r="E3" s="98" t="s">
         <v>28</v>
       </c>
-      <c r="F3" s="97"/>
-      <c r="G3" s="98"/>
+      <c r="F3" s="99"/>
+      <c r="G3" s="100"/>
     </row>
     <row r="4" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="14"/>
-      <c r="B4" s="40"/>
-      <c r="C4" s="40"/>
-      <c r="D4" s="41"/>
+      <c r="B4" s="91"/>
+      <c r="C4" s="91"/>
+      <c r="D4" s="92"/>
       <c r="E4" s="34"/>
       <c r="F4" s="34"/>
       <c r="G4" s="35"/>
     </row>
     <row r="5" spans="1:14" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="30"/>
-      <c r="B5" s="79" t="s">
+      <c r="B5" s="42" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="79"/>
-      <c r="D5" s="80"/>
-      <c r="E5" s="81" t="s">
+      <c r="C5" s="42"/>
+      <c r="D5" s="43"/>
+      <c r="E5" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="81"/>
-      <c r="G5" s="82"/>
+      <c r="F5" s="44"/>
+      <c r="G5" s="45"/>
     </row>
     <row r="6" spans="1:14" ht="4.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="16"/>
@@ -2546,45 +2576,45 @@
       <c r="A8" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B8" s="83" t="s">
+      <c r="B8" s="48" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="84"/>
-      <c r="D8" s="85"/>
+      <c r="C8" s="49"/>
+      <c r="D8" s="50"/>
       <c r="E8" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="F8" s="86" t="s">
+      <c r="F8" s="51" t="s">
         <v>24</v>
       </c>
-      <c r="G8" s="87"/>
+      <c r="G8" s="52"/>
       <c r="H8" s="4"/>
     </row>
     <row r="9" spans="1:14" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="88" t="s">
+      <c r="B9" s="53" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="89"/>
-      <c r="D9" s="90"/>
+      <c r="C9" s="54"/>
+      <c r="D9" s="55"/>
       <c r="E9" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="91" t="s">
+      <c r="F9" s="96" t="s">
         <v>25</v>
       </c>
-      <c r="G9" s="92"/>
+      <c r="G9" s="97"/>
     </row>
     <row r="10" spans="1:14" ht="5.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="93"/>
-      <c r="B10" s="93"/>
-      <c r="C10" s="93"/>
-      <c r="D10" s="93"/>
-      <c r="E10" s="93"/>
-      <c r="F10" s="93"/>
-      <c r="G10" s="93"/>
+      <c r="A10" s="58"/>
+      <c r="B10" s="58"/>
+      <c r="C10" s="58"/>
+      <c r="D10" s="58"/>
+      <c r="E10" s="58"/>
+      <c r="F10" s="58"/>
+      <c r="G10" s="58"/>
     </row>
     <row r="11" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
@@ -2593,14 +2623,14 @@
       <c r="B11" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="94" t="s">
+      <c r="C11" s="59" t="s">
         <v>7</v>
       </c>
-      <c r="D11" s="95"/>
-      <c r="E11" s="94" t="s">
+      <c r="D11" s="60"/>
+      <c r="E11" s="59" t="s">
         <v>3</v>
       </c>
-      <c r="F11" s="95"/>
+      <c r="F11" s="60"/>
       <c r="G11" s="22" t="s">
         <v>4</v>
       </c>
@@ -2612,14 +2642,14 @@
       <c r="B12" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C12" s="77" t="s">
+      <c r="C12" s="46" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="78"/>
-      <c r="E12" s="45" t="s">
+      <c r="D12" s="47"/>
+      <c r="E12" s="38" t="s">
         <v>37</v>
       </c>
-      <c r="F12" s="46"/>
+      <c r="F12" s="39"/>
       <c r="G12" s="23"/>
       <c r="H12" s="11"/>
       <c r="I12" s="5"/>
@@ -2632,10 +2662,10 @@
     <row r="13" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="12"/>
       <c r="B13" s="1"/>
-      <c r="C13" s="77"/>
-      <c r="D13" s="78"/>
-      <c r="E13" s="45"/>
-      <c r="F13" s="46"/>
+      <c r="C13" s="46"/>
+      <c r="D13" s="47"/>
+      <c r="E13" s="38"/>
+      <c r="F13" s="39"/>
       <c r="G13" s="23"/>
       <c r="H13" s="11"/>
       <c r="I13" s="8"/>
@@ -2646,413 +2676,413 @@
     <row r="14" spans="1:14" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="13"/>
       <c r="B14" s="1"/>
-      <c r="C14" s="77"/>
-      <c r="D14" s="78"/>
-      <c r="E14" s="45"/>
-      <c r="F14" s="46"/>
+      <c r="C14" s="46"/>
+      <c r="D14" s="47"/>
+      <c r="E14" s="38"/>
+      <c r="F14" s="39"/>
       <c r="G14" s="23"/>
       <c r="H14" s="11"/>
     </row>
     <row r="15" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="13"/>
       <c r="B15" s="1"/>
-      <c r="C15" s="77"/>
-      <c r="D15" s="78"/>
-      <c r="E15" s="45"/>
-      <c r="F15" s="46"/>
+      <c r="C15" s="46"/>
+      <c r="D15" s="47"/>
+      <c r="E15" s="38"/>
+      <c r="F15" s="39"/>
       <c r="G15" s="23"/>
       <c r="H15" s="11"/>
     </row>
     <row r="16" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="13"/>
       <c r="B16" s="2"/>
-      <c r="C16" s="77"/>
-      <c r="D16" s="78"/>
-      <c r="E16" s="45"/>
-      <c r="F16" s="46"/>
+      <c r="C16" s="46"/>
+      <c r="D16" s="47"/>
+      <c r="E16" s="38"/>
+      <c r="F16" s="39"/>
       <c r="G16" s="23"/>
       <c r="H16" s="11"/>
     </row>
     <row r="17" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="13"/>
       <c r="B17" s="2"/>
-      <c r="C17" s="77"/>
-      <c r="D17" s="78"/>
-      <c r="E17" s="45"/>
-      <c r="F17" s="46"/>
+      <c r="C17" s="46"/>
+      <c r="D17" s="47"/>
+      <c r="E17" s="38"/>
+      <c r="F17" s="39"/>
       <c r="G17" s="23"/>
       <c r="H17" s="11"/>
     </row>
     <row r="18" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="13"/>
       <c r="B18" s="2"/>
-      <c r="C18" s="47"/>
-      <c r="D18" s="48"/>
-      <c r="E18" s="45"/>
-      <c r="F18" s="46"/>
+      <c r="C18" s="40"/>
+      <c r="D18" s="41"/>
+      <c r="E18" s="38"/>
+      <c r="F18" s="39"/>
       <c r="G18" s="23"/>
       <c r="H18" s="11"/>
     </row>
     <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="13"/>
       <c r="B19" s="2"/>
-      <c r="C19" s="47"/>
-      <c r="D19" s="48"/>
-      <c r="E19" s="45"/>
-      <c r="F19" s="46"/>
+      <c r="C19" s="40"/>
+      <c r="D19" s="41"/>
+      <c r="E19" s="38"/>
+      <c r="F19" s="39"/>
       <c r="G19" s="23"/>
       <c r="H19" s="10"/>
     </row>
     <row r="20" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="13"/>
       <c r="B20" s="2"/>
-      <c r="C20" s="47"/>
-      <c r="D20" s="48"/>
-      <c r="E20" s="45"/>
-      <c r="F20" s="46"/>
+      <c r="C20" s="40"/>
+      <c r="D20" s="41"/>
+      <c r="E20" s="38"/>
+      <c r="F20" s="39"/>
       <c r="G20" s="23"/>
       <c r="H20" s="10"/>
     </row>
     <row r="21" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="13"/>
       <c r="B21" s="2"/>
-      <c r="C21" s="47"/>
-      <c r="D21" s="48"/>
-      <c r="E21" s="45"/>
-      <c r="F21" s="46"/>
+      <c r="C21" s="40"/>
+      <c r="D21" s="41"/>
+      <c r="E21" s="38"/>
+      <c r="F21" s="39"/>
       <c r="G21" s="23"/>
       <c r="H21" s="10"/>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="13"/>
       <c r="B22" s="2"/>
-      <c r="C22" s="47"/>
-      <c r="D22" s="48"/>
-      <c r="E22" s="45"/>
-      <c r="F22" s="46"/>
+      <c r="C22" s="40"/>
+      <c r="D22" s="41"/>
+      <c r="E22" s="38"/>
+      <c r="F22" s="39"/>
       <c r="G22" s="23"/>
       <c r="H22" s="10"/>
     </row>
     <row r="23" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="13"/>
       <c r="B23" s="2"/>
-      <c r="C23" s="47"/>
-      <c r="D23" s="48"/>
-      <c r="E23" s="45"/>
-      <c r="F23" s="46"/>
+      <c r="C23" s="40"/>
+      <c r="D23" s="41"/>
+      <c r="E23" s="38"/>
+      <c r="F23" s="39"/>
       <c r="G23" s="23"/>
       <c r="H23" s="10"/>
     </row>
     <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="13"/>
       <c r="B24" s="2"/>
-      <c r="C24" s="47"/>
-      <c r="D24" s="48"/>
-      <c r="E24" s="45"/>
-      <c r="F24" s="46"/>
+      <c r="C24" s="40"/>
+      <c r="D24" s="41"/>
+      <c r="E24" s="38"/>
+      <c r="F24" s="39"/>
       <c r="G24" s="23"/>
       <c r="H24" s="10"/>
     </row>
     <row r="25" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="13"/>
       <c r="B25" s="2"/>
-      <c r="C25" s="47"/>
-      <c r="D25" s="48"/>
-      <c r="E25" s="45"/>
-      <c r="F25" s="46"/>
+      <c r="C25" s="40"/>
+      <c r="D25" s="41"/>
+      <c r="E25" s="38"/>
+      <c r="F25" s="39"/>
       <c r="G25" s="23"/>
       <c r="H25" s="10"/>
     </row>
     <row r="26" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="13"/>
       <c r="B26" s="2"/>
-      <c r="C26" s="47"/>
-      <c r="D26" s="48"/>
-      <c r="E26" s="45"/>
-      <c r="F26" s="46"/>
+      <c r="C26" s="40"/>
+      <c r="D26" s="41"/>
+      <c r="E26" s="38"/>
+      <c r="F26" s="39"/>
       <c r="G26" s="23"/>
       <c r="H26" s="10"/>
     </row>
     <row r="27" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="13"/>
       <c r="B27" s="2"/>
-      <c r="C27" s="47"/>
-      <c r="D27" s="48"/>
-      <c r="E27" s="45"/>
-      <c r="F27" s="46"/>
+      <c r="C27" s="40"/>
+      <c r="D27" s="41"/>
+      <c r="E27" s="38"/>
+      <c r="F27" s="39"/>
       <c r="G27" s="23"/>
       <c r="H27" s="10"/>
     </row>
     <row r="28" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="13"/>
       <c r="B28" s="2"/>
-      <c r="C28" s="75"/>
-      <c r="D28" s="76"/>
-      <c r="E28" s="45"/>
-      <c r="F28" s="46"/>
+      <c r="C28" s="61"/>
+      <c r="D28" s="62"/>
+      <c r="E28" s="38"/>
+      <c r="F28" s="39"/>
       <c r="G28" s="23"/>
       <c r="H28" s="10"/>
     </row>
     <row r="29" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="13"/>
       <c r="B29" s="2"/>
-      <c r="C29" s="75"/>
-      <c r="D29" s="76"/>
-      <c r="E29" s="45"/>
-      <c r="F29" s="46"/>
+      <c r="C29" s="61"/>
+      <c r="D29" s="62"/>
+      <c r="E29" s="38"/>
+      <c r="F29" s="39"/>
       <c r="G29" s="23"/>
       <c r="H29" s="10"/>
     </row>
     <row r="30" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="13"/>
       <c r="B30" s="2"/>
-      <c r="C30" s="75"/>
-      <c r="D30" s="76"/>
-      <c r="E30" s="45"/>
-      <c r="F30" s="46"/>
+      <c r="C30" s="61"/>
+      <c r="D30" s="62"/>
+      <c r="E30" s="38"/>
+      <c r="F30" s="39"/>
       <c r="G30" s="23"/>
       <c r="H30" s="10"/>
     </row>
     <row r="31" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="13"/>
       <c r="B31" s="2"/>
-      <c r="C31" s="47"/>
-      <c r="D31" s="48"/>
-      <c r="E31" s="45"/>
-      <c r="F31" s="46"/>
+      <c r="C31" s="40"/>
+      <c r="D31" s="41"/>
+      <c r="E31" s="38"/>
+      <c r="F31" s="39"/>
       <c r="G31" s="23"/>
       <c r="H31" s="10"/>
     </row>
     <row r="32" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="13"/>
       <c r="B32" s="2"/>
-      <c r="C32" s="47"/>
-      <c r="D32" s="48"/>
-      <c r="E32" s="45"/>
-      <c r="F32" s="46"/>
+      <c r="C32" s="40"/>
+      <c r="D32" s="41"/>
+      <c r="E32" s="38"/>
+      <c r="F32" s="39"/>
       <c r="G32" s="23"/>
       <c r="H32" s="10"/>
     </row>
     <row r="33" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="13"/>
       <c r="B33" s="2"/>
-      <c r="C33" s="47"/>
-      <c r="D33" s="48"/>
-      <c r="E33" s="45"/>
-      <c r="F33" s="46"/>
+      <c r="C33" s="40"/>
+      <c r="D33" s="41"/>
+      <c r="E33" s="38"/>
+      <c r="F33" s="39"/>
       <c r="G33" s="23"/>
       <c r="H33" s="10"/>
     </row>
     <row r="34" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="13"/>
       <c r="B34" s="2"/>
-      <c r="C34" s="47"/>
-      <c r="D34" s="48"/>
-      <c r="E34" s="45"/>
-      <c r="F34" s="46"/>
+      <c r="C34" s="40"/>
+      <c r="D34" s="41"/>
+      <c r="E34" s="38"/>
+      <c r="F34" s="39"/>
       <c r="G34" s="23"/>
       <c r="H34" s="10"/>
     </row>
     <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="13"/>
       <c r="B35" s="2"/>
-      <c r="C35" s="47"/>
-      <c r="D35" s="48"/>
-      <c r="E35" s="45"/>
-      <c r="F35" s="46"/>
+      <c r="C35" s="40"/>
+      <c r="D35" s="41"/>
+      <c r="E35" s="38"/>
+      <c r="F35" s="39"/>
       <c r="G35" s="23"/>
       <c r="H35" s="10"/>
     </row>
     <row r="36" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="13"/>
       <c r="B36" s="2"/>
-      <c r="C36" s="47"/>
-      <c r="D36" s="48"/>
-      <c r="E36" s="45"/>
-      <c r="F36" s="46"/>
+      <c r="C36" s="40"/>
+      <c r="D36" s="41"/>
+      <c r="E36" s="38"/>
+      <c r="F36" s="39"/>
       <c r="G36" s="23"/>
       <c r="H36" s="10"/>
     </row>
     <row r="37" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="13"/>
       <c r="B37" s="2"/>
-      <c r="C37" s="47"/>
-      <c r="D37" s="48"/>
-      <c r="E37" s="45"/>
-      <c r="F37" s="46"/>
+      <c r="C37" s="40"/>
+      <c r="D37" s="41"/>
+      <c r="E37" s="38"/>
+      <c r="F37" s="39"/>
       <c r="G37" s="23"/>
       <c r="H37" s="10"/>
     </row>
     <row r="38" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="13"/>
       <c r="B38" s="2"/>
-      <c r="C38" s="47"/>
-      <c r="D38" s="48"/>
-      <c r="E38" s="45"/>
-      <c r="F38" s="46"/>
+      <c r="C38" s="40"/>
+      <c r="D38" s="41"/>
+      <c r="E38" s="38"/>
+      <c r="F38" s="39"/>
       <c r="G38" s="23"/>
       <c r="H38" s="10"/>
     </row>
     <row r="39" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="13"/>
       <c r="B39" s="2"/>
-      <c r="C39" s="49"/>
-      <c r="D39" s="50"/>
-      <c r="E39" s="45"/>
-      <c r="F39" s="46"/>
+      <c r="C39" s="87"/>
+      <c r="D39" s="88"/>
+      <c r="E39" s="38"/>
+      <c r="F39" s="39"/>
       <c r="G39" s="23"/>
       <c r="H39" s="10"/>
     </row>
     <row r="40" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="13"/>
       <c r="B40" s="2"/>
-      <c r="C40" s="47"/>
-      <c r="D40" s="48"/>
-      <c r="E40" s="45"/>
-      <c r="F40" s="46"/>
+      <c r="C40" s="40"/>
+      <c r="D40" s="41"/>
+      <c r="E40" s="38"/>
+      <c r="F40" s="39"/>
       <c r="G40" s="23"/>
       <c r="H40" s="10"/>
     </row>
     <row r="41" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="13"/>
       <c r="B41" s="2"/>
-      <c r="C41" s="47"/>
-      <c r="D41" s="48"/>
-      <c r="E41" s="45"/>
-      <c r="F41" s="46"/>
+      <c r="C41" s="40"/>
+      <c r="D41" s="41"/>
+      <c r="E41" s="38"/>
+      <c r="F41" s="39"/>
       <c r="G41" s="23"/>
       <c r="H41" s="10"/>
     </row>
     <row r="42" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="13"/>
       <c r="B42" s="2"/>
-      <c r="C42" s="47"/>
-      <c r="D42" s="48"/>
-      <c r="E42" s="45"/>
-      <c r="F42" s="46"/>
+      <c r="C42" s="40"/>
+      <c r="D42" s="41"/>
+      <c r="E42" s="38"/>
+      <c r="F42" s="39"/>
       <c r="G42" s="23"/>
       <c r="H42" s="10"/>
     </row>
     <row r="43" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="13"/>
       <c r="B43" s="2"/>
-      <c r="C43" s="47"/>
-      <c r="D43" s="48"/>
-      <c r="E43" s="45"/>
-      <c r="F43" s="46"/>
+      <c r="C43" s="40"/>
+      <c r="D43" s="41"/>
+      <c r="E43" s="38"/>
+      <c r="F43" s="39"/>
       <c r="G43" s="23"/>
       <c r="H43" s="10"/>
     </row>
     <row r="44" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="13"/>
       <c r="B44" s="2"/>
-      <c r="C44" s="47"/>
-      <c r="D44" s="48"/>
-      <c r="E44" s="45"/>
-      <c r="F44" s="46"/>
+      <c r="C44" s="40"/>
+      <c r="D44" s="41"/>
+      <c r="E44" s="38"/>
+      <c r="F44" s="39"/>
       <c r="G44" s="23"/>
       <c r="H44" s="10"/>
     </row>
     <row r="45" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="13"/>
       <c r="B45" s="2"/>
-      <c r="C45" s="47"/>
-      <c r="D45" s="48"/>
-      <c r="E45" s="45"/>
-      <c r="F45" s="46"/>
+      <c r="C45" s="40"/>
+      <c r="D45" s="41"/>
+      <c r="E45" s="38"/>
+      <c r="F45" s="39"/>
       <c r="G45" s="23"/>
       <c r="H45" s="10"/>
     </row>
     <row r="46" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="13"/>
       <c r="B46" s="2"/>
-      <c r="C46" s="47"/>
-      <c r="D46" s="48"/>
-      <c r="E46" s="45"/>
-      <c r="F46" s="46"/>
+      <c r="C46" s="40"/>
+      <c r="D46" s="41"/>
+      <c r="E46" s="38"/>
+      <c r="F46" s="39"/>
       <c r="G46" s="23"/>
       <c r="H46" s="10"/>
     </row>
     <row r="47" spans="1:8" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A47" s="13"/>
       <c r="B47" s="2"/>
-      <c r="C47" s="47"/>
-      <c r="D47" s="48"/>
-      <c r="E47" s="45"/>
-      <c r="F47" s="46"/>
+      <c r="C47" s="40"/>
+      <c r="D47" s="41"/>
+      <c r="E47" s="38"/>
+      <c r="F47" s="39"/>
       <c r="G47" s="23"/>
     </row>
     <row r="48" spans="1:8" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="63" t="s">
+      <c r="A48" s="75" t="s">
         <v>14</v>
       </c>
-      <c r="B48" s="64"/>
-      <c r="C48" s="64"/>
-      <c r="D48" s="64"/>
-      <c r="E48" s="65"/>
-      <c r="F48" s="66"/>
-      <c r="G48" s="67"/>
+      <c r="B48" s="76"/>
+      <c r="C48" s="76"/>
+      <c r="D48" s="76"/>
+      <c r="E48" s="77"/>
+      <c r="F48" s="78"/>
+      <c r="G48" s="79"/>
     </row>
     <row r="49" spans="1:7" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="50" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="73" t="s">
+      <c r="A50" s="85" t="s">
         <v>20</v>
       </c>
-      <c r="B50" s="74"/>
-      <c r="C50" s="70" t="s">
+      <c r="B50" s="86"/>
+      <c r="C50" s="101" t="s">
         <v>26</v>
       </c>
-      <c r="D50" s="71"/>
-      <c r="E50" s="71"/>
-      <c r="F50" s="71"/>
-      <c r="G50" s="72"/>
+      <c r="D50" s="102"/>
+      <c r="E50" s="102"/>
+      <c r="F50" s="102"/>
+      <c r="G50" s="103"/>
     </row>
     <row r="51" spans="1:7" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="55" t="s">
+      <c r="A51" s="67" t="s">
         <v>15</v>
       </c>
-      <c r="B51" s="56"/>
-      <c r="C51" s="68"/>
-      <c r="D51" s="69"/>
-      <c r="E51" s="57" t="s">
+      <c r="B51" s="68"/>
+      <c r="C51" s="80"/>
+      <c r="D51" s="81"/>
+      <c r="E51" s="69" t="s">
         <v>5</v>
       </c>
-      <c r="F51" s="58"/>
-      <c r="G51" s="59"/>
+      <c r="F51" s="70"/>
+      <c r="G51" s="71"/>
     </row>
     <row r="52" spans="1:7" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A52" s="55" t="s">
+      <c r="A52" s="67" t="s">
         <v>27</v>
       </c>
-      <c r="B52" s="56"/>
+      <c r="B52" s="68"/>
       <c r="C52" s="32" t="s">
         <v>29</v>
       </c>
       <c r="D52" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="E52" s="60" t="s">
+      <c r="E52" s="72" t="s">
         <v>30</v>
       </c>
-      <c r="F52" s="61"/>
-      <c r="G52" s="62"/>
+      <c r="F52" s="73"/>
+      <c r="G52" s="74"/>
     </row>
     <row r="53" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="51" t="s">
+      <c r="A53" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="B53" s="52"/>
+      <c r="B53" s="64"/>
       <c r="C53" s="33" t="s">
         <v>33</v>
       </c>
       <c r="D53" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="E53" s="53" t="s">
+      <c r="E53" s="65" t="s">
         <v>32</v>
       </c>
-      <c r="F53" s="53"/>
-      <c r="G53" s="54"/>
+      <c r="F53" s="65"/>
+      <c r="G53" s="66"/>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.2">
       <c r="G54" s="3" t="s">
@@ -3061,87 +3091,6 @@
     </row>
   </sheetData>
   <mergeCells count="97">
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="A10:G10"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="E12:F12"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="E17:F17"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="E21:F21"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="E25:F25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="E26:F26"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="E27:F27"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="E28:F28"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="E29:F29"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="E30:F30"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="E31:F31"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="E32:F32"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="E33:F33"/>
-    <mergeCell ref="C34:D34"/>
-    <mergeCell ref="E34:F34"/>
-    <mergeCell ref="C35:D35"/>
-    <mergeCell ref="E35:F35"/>
-    <mergeCell ref="C36:D36"/>
-    <mergeCell ref="E36:F36"/>
-    <mergeCell ref="C37:D37"/>
-    <mergeCell ref="E37:F37"/>
-    <mergeCell ref="C38:D38"/>
-    <mergeCell ref="E38:F38"/>
-    <mergeCell ref="C39:D39"/>
-    <mergeCell ref="E39:F39"/>
-    <mergeCell ref="C40:D40"/>
-    <mergeCell ref="E40:F40"/>
-    <mergeCell ref="C41:D41"/>
-    <mergeCell ref="E41:F41"/>
-    <mergeCell ref="C47:D47"/>
-    <mergeCell ref="E47:F47"/>
-    <mergeCell ref="C42:D42"/>
-    <mergeCell ref="E42:F42"/>
-    <mergeCell ref="C43:D43"/>
-    <mergeCell ref="E43:F43"/>
-    <mergeCell ref="C44:D44"/>
-    <mergeCell ref="E44:F44"/>
     <mergeCell ref="E52:G52"/>
     <mergeCell ref="A53:B53"/>
     <mergeCell ref="E53:G53"/>
@@ -3158,6 +3107,87 @@
     <mergeCell ref="E45:F45"/>
     <mergeCell ref="C46:D46"/>
     <mergeCell ref="E46:F46"/>
+    <mergeCell ref="C47:D47"/>
+    <mergeCell ref="E47:F47"/>
+    <mergeCell ref="C42:D42"/>
+    <mergeCell ref="E42:F42"/>
+    <mergeCell ref="C43:D43"/>
+    <mergeCell ref="E43:F43"/>
+    <mergeCell ref="C44:D44"/>
+    <mergeCell ref="E44:F44"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="E39:F39"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="E40:F40"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="E41:F41"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="E36:F36"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="E37:F37"/>
+    <mergeCell ref="C38:D38"/>
+    <mergeCell ref="E38:F38"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="E33:F33"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="E34:F34"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="E35:F35"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="E30:F30"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="E32:F32"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="E28:F28"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="A10:G10"/>
   </mergeCells>
   <pageMargins left="0.51181102362204722" right="0.19685039370078741" top="0.31496062992125984" bottom="0" header="0.51181102362204722" footer="0.51181102362204722"/>
   <pageSetup paperSize="9" scale="83" fitToHeight="0" orientation="portrait" copies="3" r:id="rId1"/>

</xml_diff>